<commit_message>
feat: re-import updated EQUIPMENT_Data.xlsx with complete outdoor unit database for 橫綱X series (RXV & RXM models)
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E10BC5-E90E-49FA-A7FC-D232FFD2D56D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF31C842-F600-4979-982D-7C36245E9D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="0" windowWidth="22080" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="6000" yWindow="0" windowWidth="17040" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2782" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2854" uniqueCount="527">
   <si>
     <t>資料型態</t>
   </si>
@@ -1929,6 +1929,58 @@
   <si>
     <t>FTHF71ZVLT</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>橫綱X系列</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM22XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM28XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM36XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM41XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM50XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM60XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM71XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM80XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXM90XVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>550×675×284</t>
+  </si>
+  <si>
+    <t>595×845×300</t>
+  </si>
+  <si>
+    <t>695×930×350</t>
+  </si>
+  <si>
+    <t>990×940×320</t>
   </si>
 </sst>
 </file>
@@ -10009,17 +10061,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14518F8B-544C-42CB-BD27-24B9976359F4}">
-  <dimension ref="A1:FH13"/>
+  <dimension ref="A1:FQ13"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.44140625" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" style="7" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="34.44140625" hidden="1" customWidth="1"/>
-    <col min="5" max="131" width="14.6640625" customWidth="1"/>
+    <col min="5" max="140" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -10033,7 +10085,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:164" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:173" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
@@ -10155,31 +10207,31 @@
         <v>34</v>
       </c>
       <c r="AO2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AP2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AQ2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AR2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AS2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AT2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AU2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AV2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AW2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AX2" s="5" t="s">
         <v>101</v>
@@ -10224,31 +10276,31 @@
         <v>101</v>
       </c>
       <c r="BL2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BM2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BN2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BO2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BP2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BQ2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BR2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BS2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BT2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BU2" s="5" t="s">
         <v>143</v>
@@ -10427,15 +10479,33 @@
       <c r="EA2" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="EB2" s="5"/>
-      <c r="EC2" s="5"/>
-      <c r="ED2" s="5"/>
-      <c r="EE2" s="5"/>
-      <c r="EF2" s="5"/>
-      <c r="EG2" s="5"/>
-      <c r="EH2" s="5"/>
-      <c r="EI2" s="5"/>
-      <c r="EJ2" s="5"/>
+      <c r="EB2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EC2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="ED2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EE2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EF2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EG2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EH2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EI2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EJ2" s="5" t="s">
+        <v>143</v>
+      </c>
       <c r="EK2" s="5"/>
       <c r="EL2" s="5"/>
       <c r="EM2" s="5"/>
@@ -10460,8 +10530,17 @@
       <c r="FF2" s="5"/>
       <c r="FG2" s="5"/>
       <c r="FH2" s="5"/>
+      <c r="FI2" s="5"/>
+      <c r="FJ2" s="5"/>
+      <c r="FK2" s="5"/>
+      <c r="FL2" s="5"/>
+      <c r="FM2" s="5"/>
+      <c r="FN2" s="5"/>
+      <c r="FO2" s="5"/>
+      <c r="FP2" s="5"/>
+      <c r="FQ2" s="5"/>
     </row>
-    <row r="3" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
@@ -10523,91 +10602,91 @@
         <v>75</v>
       </c>
       <c r="U3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="Z3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="AC3" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="AD3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="V3" s="5" t="s">
+      <c r="AE3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="W3" s="5" t="s">
+      <c r="AF3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="X3" s="5" t="s">
+      <c r="AG3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="AH3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="Z3" s="5" t="s">
+      <c r="AI3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="AA3" s="5" t="s">
+      <c r="AJ3" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="AB3" s="5" t="s">
+      <c r="AK3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AC3" s="5" t="s">
+      <c r="AL3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AD3" s="5" t="s">
+      <c r="AM3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AE3" s="5" t="s">
+      <c r="AN3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AF3" s="5" t="s">
+      <c r="AO3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AG3" s="5" t="s">
+      <c r="AP3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AH3" s="5" t="s">
+      <c r="AQ3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AI3" s="5" t="s">
+      <c r="AR3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AJ3" s="5" t="s">
+      <c r="AS3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AK3" s="5" t="s">
+      <c r="AT3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AL3" s="5" t="s">
+      <c r="AU3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AM3" s="5" t="s">
+      <c r="AV3" s="5" t="s">
         <v>488</v>
       </c>
-      <c r="AN3" s="5" t="s">
+      <c r="AW3" s="5" t="s">
         <v>488</v>
-      </c>
-      <c r="AO3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AP3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AQ3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AR3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AS3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AT3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AU3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AV3" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AW3" s="5" t="s">
-        <v>102</v>
       </c>
       <c r="AX3" s="5" t="s">
         <v>102</v>
@@ -10622,103 +10701,103 @@
         <v>102</v>
       </c>
       <c r="BB3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BC3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BD3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BE3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BF3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BG3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BH3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BI3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BJ3" s="5" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="BK3" s="5" t="s">
         <v>111</v>
       </c>
       <c r="BL3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BM3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BN3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BO3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BP3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BQ3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BR3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BS3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BT3" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="BU3" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="BM3" s="5" t="s">
+      <c r="BV3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BN3" s="5" t="s">
+      <c r="BW3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BO3" s="5" t="s">
+      <c r="BX3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BP3" s="5" t="s">
+      <c r="BY3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BQ3" s="5" t="s">
+      <c r="BZ3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BR3" s="5" t="s">
+      <c r="CA3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="BS3" s="5" t="s">
+      <c r="CB3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="BT3" s="5" t="s">
+      <c r="CC3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="BU3" s="5" t="s">
+      <c r="CD3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="BV3" s="5" t="s">
+      <c r="CE3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="BW3" s="5" t="s">
+      <c r="CF3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="BX3" s="5" t="s">
+      <c r="CG3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="BY3" s="5" t="s">
+      <c r="CH3" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="BZ3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CA3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CB3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CC3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CD3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CE3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CF3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CG3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CH3" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="CI3" s="5" t="s">
         <v>201</v>
@@ -10775,31 +10854,31 @@
         <v>201</v>
       </c>
       <c r="DA3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DB3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DC3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DD3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DE3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DF3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DG3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DH3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DI3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DJ3" s="5" t="s">
         <v>42</v>
@@ -10855,15 +10934,33 @@
       <c r="EA3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="EB3" s="5"/>
-      <c r="EC3" s="5"/>
-      <c r="ED3" s="5"/>
-      <c r="EE3" s="5"/>
-      <c r="EF3" s="5"/>
-      <c r="EG3" s="5"/>
-      <c r="EH3" s="5"/>
-      <c r="EI3" s="5"/>
-      <c r="EJ3" s="5"/>
+      <c r="EB3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EC3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="ED3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EE3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EF3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EG3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EH3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EI3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EJ3" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="EK3" s="5"/>
       <c r="EL3" s="5"/>
       <c r="EM3" s="5"/>
@@ -10888,8 +10985,17 @@
       <c r="FF3" s="5"/>
       <c r="FG3" s="5"/>
       <c r="FH3" s="5"/>
+      <c r="FI3" s="5"/>
+      <c r="FJ3" s="5"/>
+      <c r="FK3" s="5"/>
+      <c r="FL3" s="5"/>
+      <c r="FM3" s="5"/>
+      <c r="FN3" s="5"/>
+      <c r="FO3" s="5"/>
+      <c r="FP3" s="5"/>
+      <c r="FQ3" s="5"/>
     </row>
-    <row r="4" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>52</v>
       </c>
@@ -10951,347 +11057,365 @@
         <v>87</v>
       </c>
       <c r="U4" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>515</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>518</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="AB4" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="AC4" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="AD4" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="V4" s="5" t="s">
+      <c r="AE4" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="W4" s="5" t="s">
+      <c r="AF4" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="X4" s="5" t="s">
+      <c r="AG4" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="Y4" s="5" t="s">
+      <c r="AH4" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="Z4" s="5" t="s">
+      <c r="AI4" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AA4" s="5" t="s">
+      <c r="AJ4" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="AB4" s="5" t="s">
+      <c r="AK4" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="AC4" s="5" t="s">
+      <c r="AL4" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AD4" s="5" t="s">
+      <c r="AM4" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AE4" s="5" t="s">
+      <c r="AN4" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="AF4" s="5" t="s">
+      <c r="AO4" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AG4" s="5" t="s">
+      <c r="AP4" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="AH4" s="5" t="s">
+      <c r="AQ4" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="AI4" s="5" t="s">
+      <c r="AR4" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AJ4" s="5" t="s">
+      <c r="AS4" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="AK4" s="5" t="s">
+      <c r="AT4" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AL4" s="5" t="s">
+      <c r="AU4" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="AM4" s="5" t="s">
+      <c r="AV4" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="AN4" s="5" t="s">
+      <c r="AW4" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="AO4" s="5" t="s">
+      <c r="AX4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AP4" s="5" t="s">
+      <c r="AY4" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AQ4" s="5" t="s">
+      <c r="AZ4" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="5" t="s">
+      <c r="BA4" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="AS4" s="5" t="s">
+      <c r="BB4" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="AT4" s="5" t="s">
+      <c r="BC4" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="AU4" s="5" t="s">
+      <c r="BD4" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="AV4" s="5" t="s">
+      <c r="BE4" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="AW4" s="5" t="s">
+      <c r="BF4" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="AX4" s="5" t="s">
+      <c r="BG4" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="AY4" s="5" t="s">
+      <c r="BH4" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="AZ4" s="5" t="s">
+      <c r="BI4" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="BA4" s="5" t="s">
+      <c r="BJ4" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="BB4" s="5" t="s">
+      <c r="BK4" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="BC4" s="5" t="s">
+      <c r="BL4" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="BD4" s="5" t="s">
+      <c r="BM4" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="BE4" s="5" t="s">
+      <c r="BN4" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="BF4" s="5" t="s">
+      <c r="BO4" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="BG4" s="5" t="s">
+      <c r="BP4" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="BH4" s="5" t="s">
+      <c r="BQ4" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="BI4" s="5" t="s">
+      <c r="BR4" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="BJ4" s="5" t="s">
+      <c r="BS4" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="BK4" s="5" t="s">
+      <c r="BT4" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="BL4" s="5" t="s">
+      <c r="BU4" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="BM4" s="5" t="s">
+      <c r="BV4" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="BN4" s="5" t="s">
+      <c r="BW4" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="BO4" s="5" t="s">
+      <c r="BX4" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="BP4" s="5" t="s">
+      <c r="BY4" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="BQ4" s="5" t="s">
+      <c r="BZ4" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="BR4" s="5" t="s">
+      <c r="CA4" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="BS4" s="5" t="s">
+      <c r="CB4" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="BT4" s="5" t="s">
+      <c r="CC4" s="5" t="s">
         <v>505</v>
       </c>
-      <c r="BU4" s="5" t="s">
+      <c r="CD4" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="BV4" s="5" t="s">
+      <c r="CE4" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="BW4" s="5" t="s">
+      <c r="CF4" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="BX4" s="5" t="s">
+      <c r="CG4" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="BY4" s="5" t="s">
+      <c r="CH4" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="BZ4" s="5" t="s">
+      <c r="CI4" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="CA4" s="5" t="s">
+      <c r="CJ4" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="CB4" s="5" t="s">
+      <c r="CK4" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="CC4" s="5" t="s">
+      <c r="CL4" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="CD4" s="5" t="s">
+      <c r="CM4" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="CE4" s="5" t="s">
+      <c r="CN4" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="CF4" s="5" t="s">
+      <c r="CO4" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="CG4" s="5" t="s">
+      <c r="CP4" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="CH4" s="5" t="s">
+      <c r="CQ4" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="CI4" s="5" t="s">
+      <c r="CR4" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="CJ4" s="5" t="s">
+      <c r="CS4" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="CK4" s="5" t="s">
+      <c r="CT4" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="CL4" s="5" t="s">
+      <c r="CU4" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="CM4" s="5" t="s">
+      <c r="CV4" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="CN4" s="5" t="s">
+      <c r="CW4" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="CO4" s="5" t="s">
+      <c r="CX4" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="CP4" s="5" t="s">
+      <c r="CY4" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="CQ4" s="5" t="s">
+      <c r="CZ4" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="CR4" s="5" t="s">
+      <c r="DA4" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="CS4" s="5" t="s">
+      <c r="DB4" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="CT4" s="5" t="s">
+      <c r="DC4" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="CU4" s="5" t="s">
+      <c r="DD4" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="CV4" s="5" t="s">
+      <c r="DE4" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="CW4" s="5" t="s">
+      <c r="DF4" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="CX4" s="5" t="s">
+      <c r="DG4" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="CY4" s="5" t="s">
+      <c r="DH4" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="CZ4" s="5" t="s">
+      <c r="DI4" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="DA4" s="5" t="s">
+      <c r="DJ4" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="DB4" s="5" t="s">
+      <c r="DK4" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="DC4" s="5" t="s">
+      <c r="DL4" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="DD4" s="5" t="s">
+      <c r="DM4" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="DE4" s="5" t="s">
+      <c r="DN4" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="DF4" s="5" t="s">
+      <c r="DO4" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="DG4" s="5" t="s">
+      <c r="DP4" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="DH4" s="5" t="s">
+      <c r="DQ4" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="DI4" s="5" t="s">
+      <c r="DR4" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="DJ4" s="5" t="s">
+      <c r="DS4" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="DK4" s="5" t="s">
+      <c r="DT4" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="DL4" s="5" t="s">
+      <c r="DU4" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="DM4" s="5" t="s">
+      <c r="DV4" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="DN4" s="5" t="s">
+      <c r="DW4" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="DO4" s="5" t="s">
+      <c r="DX4" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="DP4" s="5" t="s">
+      <c r="DY4" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="DQ4" s="5" t="s">
+      <c r="DZ4" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="DR4" s="5" t="s">
+      <c r="EA4" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="DS4" s="5" t="s">
+      <c r="EB4" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="DT4" s="5" t="s">
+      <c r="EC4" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="DU4" s="5" t="s">
+      <c r="ED4" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="DV4" s="5" t="s">
+      <c r="EE4" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="DW4" s="5" t="s">
+      <c r="EF4" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="DX4" s="5" t="s">
+      <c r="EG4" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="DY4" s="5" t="s">
+      <c r="EH4" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="DZ4" s="5" t="s">
+      <c r="EI4" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="EA4" s="5" t="s">
+      <c r="EJ4" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="EB4" s="5"/>
-      <c r="EC4" s="5"/>
-      <c r="ED4" s="5"/>
-      <c r="EE4" s="5"/>
-      <c r="EF4" s="5"/>
-      <c r="EG4" s="5"/>
-      <c r="EH4" s="5"/>
-      <c r="EI4" s="5"/>
-      <c r="EJ4" s="5"/>
       <c r="EK4" s="5"/>
       <c r="EL4" s="5"/>
       <c r="EM4" s="5"/>
@@ -11316,8 +11440,17 @@
       <c r="FF4" s="5"/>
       <c r="FG4" s="5"/>
       <c r="FH4" s="5"/>
+      <c r="FI4" s="5"/>
+      <c r="FJ4" s="5"/>
+      <c r="FK4" s="5"/>
+      <c r="FL4" s="5"/>
+      <c r="FM4" s="5"/>
+      <c r="FN4" s="5"/>
+      <c r="FO4" s="5"/>
+      <c r="FP4" s="5"/>
+      <c r="FQ4" s="5"/>
     </row>
-    <row r="5" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>46</v>
       </c>
@@ -11400,115 +11533,115 @@
         <v>7.2</v>
       </c>
       <c r="AB5" s="5">
+        <v>8</v>
+      </c>
+      <c r="AC5" s="5">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="AD5" s="5">
         <v>2.2000000000000002</v>
       </c>
-      <c r="AC5" s="5">
-        <v>2.5</v>
-      </c>
-      <c r="AD5" s="5">
-        <v>3</v>
-      </c>
       <c r="AE5" s="5">
+        <v>2.8</v>
+      </c>
+      <c r="AF5" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="AG5" s="5">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AF5" s="5">
+      <c r="AH5" s="5">
         <v>5</v>
       </c>
-      <c r="AG5" s="5">
+      <c r="AI5" s="5">
         <v>6</v>
-      </c>
-      <c r="AH5" s="5">
-        <v>7.2</v>
-      </c>
-      <c r="AI5" s="5">
-        <v>5.6</v>
       </c>
       <c r="AJ5" s="5">
         <v>7.2</v>
       </c>
       <c r="AK5" s="5">
-        <v>8.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="AL5" s="5">
-        <v>10.5</v>
+        <v>2.5</v>
       </c>
       <c r="AM5" s="5">
+        <v>3</v>
+      </c>
+      <c r="AN5" s="5">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="AO5" s="5">
         <v>5</v>
       </c>
-      <c r="AN5" s="5">
-        <v>8.5</v>
-      </c>
-      <c r="AO5" s="5">
-        <v>7.2</v>
-      </c>
       <c r="AP5" s="5">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="AQ5" s="5">
         <v>7.2</v>
       </c>
       <c r="AR5" s="5">
+        <v>5.6</v>
+      </c>
+      <c r="AS5" s="5">
         <v>7.2</v>
       </c>
-      <c r="AS5" s="5">
+      <c r="AT5" s="5">
+        <v>8.5</v>
+      </c>
+      <c r="AU5" s="5">
+        <v>10.5</v>
+      </c>
+      <c r="AV5" s="5">
+        <v>5</v>
+      </c>
+      <c r="AW5" s="5">
+        <v>8.5</v>
+      </c>
+      <c r="AX5" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="AY5" s="5">
+        <v>9.5</v>
+      </c>
+      <c r="AZ5" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="BA5" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="BB5" s="5">
         <v>10.1</v>
       </c>
-      <c r="AT5" s="5">
+      <c r="BC5" s="5">
         <v>12.5</v>
       </c>
-      <c r="AU5" s="5">
+      <c r="BD5" s="5">
         <v>14</v>
       </c>
-      <c r="AV5" s="5">
+      <c r="BE5" s="5">
         <v>10.1</v>
       </c>
-      <c r="AW5" s="5">
+      <c r="BF5" s="5">
         <v>12.5</v>
       </c>
-      <c r="AX5" s="5">
+      <c r="BG5" s="5">
         <v>14</v>
       </c>
-      <c r="AY5" s="5">
+      <c r="BH5" s="5">
         <v>10.1</v>
       </c>
-      <c r="AZ5" s="5">
+      <c r="BI5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BA5" s="5">
+      <c r="BJ5" s="5">
         <v>14</v>
       </c>
-      <c r="BB5" s="5">
+      <c r="BK5" s="5">
         <v>7.2</v>
       </c>
-      <c r="BC5" s="5">
+      <c r="BL5" s="5">
         <v>10.4</v>
-      </c>
-      <c r="BD5" s="5">
-        <v>12.5</v>
-      </c>
-      <c r="BE5" s="5">
-        <v>14</v>
-      </c>
-      <c r="BF5" s="5">
-        <v>10.4</v>
-      </c>
-      <c r="BG5" s="5">
-        <v>12.5</v>
-      </c>
-      <c r="BH5" s="5">
-        <v>14</v>
-      </c>
-      <c r="BI5" s="5">
-        <v>10.4</v>
-      </c>
-      <c r="BJ5" s="5">
-        <v>12.5</v>
-      </c>
-      <c r="BK5" s="5">
-        <v>14</v>
-      </c>
-      <c r="BL5" s="5">
-        <v>11.2</v>
       </c>
       <c r="BM5" s="5">
         <v>12.5</v>
@@ -11517,209 +11650,227 @@
         <v>14</v>
       </c>
       <c r="BO5" s="5">
+        <v>10.4</v>
+      </c>
+      <c r="BP5" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="BQ5" s="5">
+        <v>14</v>
+      </c>
+      <c r="BR5" s="5">
+        <v>10.4</v>
+      </c>
+      <c r="BS5" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="BT5" s="5">
+        <v>14</v>
+      </c>
+      <c r="BU5" s="5">
+        <v>11.2</v>
+      </c>
+      <c r="BV5" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="BW5" s="5">
+        <v>14</v>
+      </c>
+      <c r="BX5" s="5">
         <v>16</v>
       </c>
-      <c r="BP5" s="5">
+      <c r="BY5" s="5">
         <v>28</v>
       </c>
-      <c r="BQ5" s="5">
+      <c r="BZ5" s="5">
         <v>33.5</v>
       </c>
-      <c r="BR5" s="5">
+      <c r="CA5" s="5">
         <v>22.4</v>
       </c>
-      <c r="BS5" s="5">
+      <c r="CB5" s="5">
         <v>25</v>
       </c>
-      <c r="BT5" s="5">
+      <c r="CC5" s="5">
         <v>15.5</v>
       </c>
-      <c r="BU5" s="5">
+      <c r="CD5" s="5">
         <v>20</v>
       </c>
-      <c r="BV5" s="5">
+      <c r="CE5" s="5">
         <v>24</v>
       </c>
-      <c r="BW5" s="5">
+      <c r="CF5" s="5">
         <v>11.2</v>
       </c>
-      <c r="BX5" s="5">
+      <c r="CG5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BY5" s="5">
+      <c r="CH5" s="5">
         <v>14</v>
       </c>
-      <c r="BZ5" s="5">
+      <c r="CI5" s="5">
         <v>22.4</v>
       </c>
-      <c r="CA5" s="5">
+      <c r="CJ5" s="5">
         <v>28</v>
       </c>
-      <c r="CB5" s="5">
+      <c r="CK5" s="5">
         <v>33.5</v>
       </c>
-      <c r="CC5" s="5">
+      <c r="CL5" s="5">
         <v>40</v>
       </c>
-      <c r="CD5" s="5">
+      <c r="CM5" s="5">
         <v>45</v>
       </c>
-      <c r="CE5" s="5">
+      <c r="CN5" s="5">
         <v>50</v>
       </c>
-      <c r="CF5" s="5">
+      <c r="CO5" s="5">
         <v>54</v>
       </c>
-      <c r="CG5" s="5">
+      <c r="CP5" s="5">
         <v>61.5</v>
       </c>
-      <c r="CH5" s="5">
+      <c r="CQ5" s="5">
         <v>67</v>
       </c>
-      <c r="CI5" s="5">
+      <c r="CR5" s="5">
         <v>73.5</v>
       </c>
-      <c r="CJ5" s="5">
+      <c r="CS5" s="5">
         <v>78.5</v>
       </c>
-      <c r="CK5" s="5">
+      <c r="CT5" s="5">
         <v>85</v>
       </c>
-      <c r="CL5" s="5">
+      <c r="CU5" s="5">
         <v>90</v>
       </c>
-      <c r="CM5" s="5">
+      <c r="CV5" s="5">
         <v>95</v>
       </c>
-      <c r="CN5" s="5">
+      <c r="CW5" s="5">
         <v>100</v>
       </c>
-      <c r="CO5" s="5">
+      <c r="CX5" s="5">
         <v>104</v>
       </c>
-      <c r="CP5" s="5">
+      <c r="CY5" s="5">
         <v>108</v>
       </c>
-      <c r="CQ5" s="5">
+      <c r="CZ5" s="5">
         <v>117</v>
       </c>
-      <c r="CR5" s="5">
+      <c r="DA5" s="5">
         <v>121</v>
       </c>
-      <c r="CS5" s="5">
+      <c r="DB5" s="5">
         <v>130</v>
       </c>
-      <c r="CT5" s="5">
+      <c r="DC5" s="5">
         <v>135</v>
       </c>
-      <c r="CU5" s="5">
+      <c r="DD5" s="5">
         <v>140</v>
       </c>
-      <c r="CV5" s="5">
+      <c r="DE5" s="5">
         <v>145</v>
       </c>
-      <c r="CW5" s="5">
+      <c r="DF5" s="5">
         <v>150</v>
       </c>
-      <c r="CX5" s="5">
+      <c r="DG5" s="5">
         <v>154</v>
       </c>
-      <c r="CY5" s="5">
+      <c r="DH5" s="5">
         <v>158</v>
       </c>
-      <c r="CZ5" s="5">
+      <c r="DI5" s="5">
         <v>162</v>
       </c>
-      <c r="DA5" s="5">
+      <c r="DJ5" s="5">
         <v>22.4</v>
       </c>
-      <c r="DB5" s="5">
+      <c r="DK5" s="5">
         <v>28</v>
       </c>
-      <c r="DC5" s="5">
+      <c r="DL5" s="5">
         <v>33.5</v>
       </c>
-      <c r="DD5" s="5">
+      <c r="DM5" s="5">
         <v>40</v>
       </c>
-      <c r="DE5" s="5">
+      <c r="DN5" s="5">
         <v>45</v>
       </c>
-      <c r="DF5" s="5">
+      <c r="DO5" s="5">
         <v>50</v>
       </c>
-      <c r="DG5" s="5">
+      <c r="DP5" s="5">
         <v>54</v>
       </c>
-      <c r="DH5" s="5">
+      <c r="DQ5" s="5">
         <v>61.5</v>
       </c>
-      <c r="DI5" s="5">
+      <c r="DR5" s="5">
         <v>67</v>
       </c>
-      <c r="DJ5" s="5">
+      <c r="DS5" s="5">
         <v>73.5</v>
       </c>
-      <c r="DK5" s="5">
+      <c r="DT5" s="5">
         <v>78.5</v>
       </c>
-      <c r="DL5" s="5">
+      <c r="DU5" s="5">
         <v>85</v>
       </c>
-      <c r="DM5" s="5">
+      <c r="DV5" s="5">
         <v>90</v>
       </c>
-      <c r="DN5" s="5">
+      <c r="DW5" s="5">
         <v>95</v>
       </c>
-      <c r="DO5" s="5">
+      <c r="DX5" s="5">
         <v>100</v>
       </c>
-      <c r="DP5" s="5">
+      <c r="DY5" s="5">
         <v>104</v>
       </c>
-      <c r="DQ5" s="5">
+      <c r="DZ5" s="5">
         <v>108</v>
       </c>
-      <c r="DR5" s="5">
+      <c r="EA5" s="5">
         <v>117</v>
       </c>
-      <c r="DS5" s="5">
+      <c r="EB5" s="5">
         <v>121</v>
       </c>
-      <c r="DT5" s="5">
+      <c r="EC5" s="5">
         <v>130</v>
       </c>
-      <c r="DU5" s="5">
+      <c r="ED5" s="5">
         <v>135</v>
       </c>
-      <c r="DV5" s="5">
+      <c r="EE5" s="5">
         <v>140</v>
       </c>
-      <c r="DW5" s="5">
+      <c r="EF5" s="5">
         <v>145</v>
       </c>
-      <c r="DX5" s="5">
+      <c r="EG5" s="5">
         <v>150</v>
       </c>
-      <c r="DY5" s="5">
+      <c r="EH5" s="5">
         <v>154</v>
       </c>
-      <c r="DZ5" s="5">
+      <c r="EI5" s="5">
         <v>158</v>
       </c>
-      <c r="EA5" s="5">
+      <c r="EJ5" s="5">
         <v>162</v>
       </c>
-      <c r="EB5" s="5"/>
-      <c r="EC5" s="5"/>
-      <c r="ED5" s="5"/>
-      <c r="EE5" s="5"/>
-      <c r="EF5" s="5"/>
-      <c r="EG5" s="5"/>
-      <c r="EH5" s="5"/>
-      <c r="EI5" s="5"/>
-      <c r="EJ5" s="5"/>
       <c r="EK5" s="5"/>
       <c r="EL5" s="5"/>
       <c r="EM5" s="5"/>
@@ -11744,8 +11895,17 @@
       <c r="FF5" s="5"/>
       <c r="FG5" s="5"/>
       <c r="FH5" s="5"/>
+      <c r="FI5" s="5"/>
+      <c r="FJ5" s="5"/>
+      <c r="FK5" s="5"/>
+      <c r="FL5" s="5"/>
+      <c r="FM5" s="5"/>
+      <c r="FN5" s="5"/>
+      <c r="FO5" s="5"/>
+      <c r="FP5" s="5"/>
+      <c r="FQ5" s="5"/>
     </row>
-    <row r="6" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
@@ -11935,219 +12095,237 @@
       <c r="BK6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="BL6" s="5">
+      <c r="BL6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BM6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BN6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BO6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BP6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BQ6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BR6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BS6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BT6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BU6" s="5">
         <v>100</v>
       </c>
-      <c r="BM6" s="5">
+      <c r="BV6" s="5">
         <v>112.5</v>
       </c>
-      <c r="BN6" s="5">
+      <c r="BW6" s="5">
         <v>125</v>
       </c>
-      <c r="BO6" s="5">
+      <c r="BX6" s="5">
         <v>150</v>
       </c>
-      <c r="BP6" s="5">
+      <c r="BY6" s="5">
         <v>250</v>
       </c>
-      <c r="BQ6" s="5">
+      <c r="BZ6" s="5">
         <v>300</v>
       </c>
-      <c r="BR6" s="5">
+      <c r="CA6" s="5">
         <v>200</v>
       </c>
-      <c r="BS6" s="5">
+      <c r="CB6" s="5">
         <v>223</v>
       </c>
-      <c r="BT6" s="5">
+      <c r="CC6" s="5">
         <v>140</v>
       </c>
-      <c r="BU6" s="5">
+      <c r="CD6" s="5">
         <v>180</v>
       </c>
-      <c r="BV6" s="5">
+      <c r="CE6" s="5">
         <v>215</v>
       </c>
-      <c r="BW6" s="5">
+      <c r="CF6" s="5">
         <v>100</v>
       </c>
-      <c r="BX6" s="5">
+      <c r="CG6" s="5">
         <v>112.5</v>
       </c>
-      <c r="BY6" s="5">
+      <c r="CH6" s="5">
         <v>125</v>
       </c>
-      <c r="BZ6" s="5">
+      <c r="CI6" s="5">
         <v>200</v>
       </c>
-      <c r="CA6" s="5">
+      <c r="CJ6" s="5">
         <v>250</v>
       </c>
-      <c r="CB6" s="5">
+      <c r="CK6" s="5">
         <v>300</v>
       </c>
-      <c r="CC6" s="5">
+      <c r="CL6" s="5">
         <v>350</v>
       </c>
-      <c r="CD6" s="5">
+      <c r="CM6" s="5">
         <v>400</v>
       </c>
-      <c r="CE6" s="5">
+      <c r="CN6" s="5">
         <v>450</v>
       </c>
-      <c r="CF6" s="5">
+      <c r="CO6" s="5">
         <v>500</v>
       </c>
-      <c r="CG6" s="5">
+      <c r="CP6" s="5">
         <v>550</v>
       </c>
-      <c r="CH6" s="5">
+      <c r="CQ6" s="5">
         <v>600</v>
       </c>
-      <c r="CI6" s="5">
+      <c r="CR6" s="5">
         <v>650</v>
       </c>
-      <c r="CJ6" s="5">
+      <c r="CS6" s="5">
         <v>700</v>
       </c>
-      <c r="CK6" s="5">
+      <c r="CT6" s="5">
         <v>750</v>
       </c>
-      <c r="CL6" s="5">
+      <c r="CU6" s="5">
         <v>800</v>
       </c>
-      <c r="CM6" s="5">
+      <c r="CV6" s="5">
         <v>850</v>
       </c>
-      <c r="CN6" s="5">
+      <c r="CW6" s="5">
         <v>900</v>
       </c>
-      <c r="CO6" s="5">
+      <c r="CX6" s="5">
         <v>950</v>
       </c>
-      <c r="CP6" s="5">
+      <c r="CY6" s="5">
         <v>1000</v>
       </c>
-      <c r="CQ6" s="5">
+      <c r="CZ6" s="5">
         <v>1050</v>
       </c>
-      <c r="CR6" s="5">
+      <c r="DA6" s="5">
         <v>1100</v>
       </c>
-      <c r="CS6" s="5">
+      <c r="DB6" s="5">
         <v>1150</v>
       </c>
-      <c r="CT6" s="5">
+      <c r="DC6" s="5">
         <v>1200</v>
       </c>
-      <c r="CU6" s="5">
+      <c r="DD6" s="5">
         <v>1250</v>
       </c>
-      <c r="CV6" s="5">
+      <c r="DE6" s="5">
         <v>1300</v>
       </c>
-      <c r="CW6" s="5">
+      <c r="DF6" s="5">
         <v>1350</v>
       </c>
-      <c r="CX6" s="5">
+      <c r="DG6" s="5">
         <v>1400</v>
       </c>
-      <c r="CY6" s="5">
+      <c r="DH6" s="5">
         <v>1450</v>
       </c>
-      <c r="CZ6" s="5">
+      <c r="DI6" s="5">
         <v>1500</v>
       </c>
-      <c r="DA6" s="5">
+      <c r="DJ6" s="5">
         <v>200</v>
       </c>
-      <c r="DB6" s="5">
+      <c r="DK6" s="5">
         <v>250</v>
       </c>
-      <c r="DC6" s="5">
+      <c r="DL6" s="5">
         <v>300</v>
       </c>
-      <c r="DD6" s="5">
+      <c r="DM6" s="5">
         <v>350</v>
       </c>
-      <c r="DE6" s="5">
+      <c r="DN6" s="5">
         <v>400</v>
       </c>
-      <c r="DF6" s="5">
+      <c r="DO6" s="5">
         <v>450</v>
       </c>
-      <c r="DG6" s="5">
+      <c r="DP6" s="5">
         <v>500</v>
       </c>
-      <c r="DH6" s="5">
+      <c r="DQ6" s="5">
         <v>550</v>
       </c>
-      <c r="DI6" s="5">
+      <c r="DR6" s="5">
         <v>600</v>
       </c>
-      <c r="DJ6" s="5">
+      <c r="DS6" s="5">
         <v>650</v>
       </c>
-      <c r="DK6" s="5">
+      <c r="DT6" s="5">
         <v>700</v>
       </c>
-      <c r="DL6" s="5">
+      <c r="DU6" s="5">
         <v>750</v>
       </c>
-      <c r="DM6" s="5">
+      <c r="DV6" s="5">
         <v>800</v>
       </c>
-      <c r="DN6" s="5">
+      <c r="DW6" s="5">
         <v>850</v>
       </c>
-      <c r="DO6" s="5">
+      <c r="DX6" s="5">
         <v>900</v>
       </c>
-      <c r="DP6" s="5">
+      <c r="DY6" s="5">
         <v>950</v>
       </c>
-      <c r="DQ6" s="5">
+      <c r="DZ6" s="5">
         <v>1000</v>
       </c>
-      <c r="DR6" s="5">
+      <c r="EA6" s="5">
         <v>1050</v>
       </c>
-      <c r="DS6" s="5">
+      <c r="EB6" s="5">
         <v>1100</v>
       </c>
-      <c r="DT6" s="5">
+      <c r="EC6" s="5">
         <v>1150</v>
       </c>
-      <c r="DU6" s="5">
+      <c r="ED6" s="5">
         <v>1200</v>
       </c>
-      <c r="DV6" s="5">
+      <c r="EE6" s="5">
         <v>1250</v>
       </c>
-      <c r="DW6" s="5">
+      <c r="EF6" s="5">
         <v>1300</v>
       </c>
-      <c r="DX6" s="5">
+      <c r="EG6" s="5">
         <v>1350</v>
       </c>
-      <c r="DY6" s="5">
+      <c r="EH6" s="5">
         <v>1400</v>
       </c>
-      <c r="DZ6" s="5">
+      <c r="EI6" s="5">
         <v>1450</v>
       </c>
-      <c r="EA6" s="5">
+      <c r="EJ6" s="5">
         <v>1500</v>
       </c>
-      <c r="EB6" s="5"/>
-      <c r="EC6" s="5"/>
-      <c r="ED6" s="5"/>
-      <c r="EE6" s="5"/>
-      <c r="EF6" s="5"/>
-      <c r="EG6" s="5"/>
-      <c r="EH6" s="5"/>
-      <c r="EI6" s="5"/>
-      <c r="EJ6" s="5"/>
       <c r="EK6" s="5"/>
       <c r="EL6" s="5"/>
       <c r="EM6" s="5"/>
@@ -12172,8 +12350,17 @@
       <c r="FF6" s="5"/>
       <c r="FG6" s="5"/>
       <c r="FH6" s="5"/>
+      <c r="FI6" s="5"/>
+      <c r="FJ6" s="5"/>
+      <c r="FK6" s="5"/>
+      <c r="FL6" s="5"/>
+      <c r="FM6" s="5"/>
+      <c r="FN6" s="5"/>
+      <c r="FO6" s="5"/>
+      <c r="FP6" s="5"/>
+      <c r="FQ6" s="5"/>
     </row>
-    <row r="7" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>48</v>
       </c>
@@ -12316,34 +12503,34 @@
         <v>9</v>
       </c>
       <c r="AV7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AW7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AX7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AY7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="AZ7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BA7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BB7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BC7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BD7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BE7" s="5" t="s">
         <v>507</v>
-      </c>
-      <c r="AW7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="AX7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="AY7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="AZ7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="BA7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="BB7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="BC7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="BD7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="BE7" s="5" t="s">
-        <v>137</v>
       </c>
       <c r="BF7" s="5" t="s">
         <v>507</v>
@@ -12352,7 +12539,7 @@
         <v>507</v>
       </c>
       <c r="BH7" s="5" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="BI7" s="5" t="s">
         <v>506</v>
@@ -12361,7 +12548,7 @@
         <v>506</v>
       </c>
       <c r="BK7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="BL7" s="5" t="s">
         <v>137</v>
@@ -12373,28 +12560,28 @@
         <v>137</v>
       </c>
       <c r="BO7" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="BP7" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="BQ7" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="BR7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="BS7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="BT7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="BU7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BP7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="BQ7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="BR7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="BS7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="BT7" s="5" t="s">
+      <c r="BV7" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="BU7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="BV7" s="5" t="s">
-        <v>506</v>
       </c>
       <c r="BW7" s="5" t="s">
         <v>137</v>
@@ -12403,19 +12590,19 @@
         <v>137</v>
       </c>
       <c r="BY7" s="5" t="s">
-        <v>137</v>
+        <v>506</v>
       </c>
       <c r="BZ7" s="5" t="s">
         <v>506</v>
       </c>
       <c r="CA7" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="CB7" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="CC7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CD7" s="5" t="s">
         <v>506</v>
@@ -12424,13 +12611,13 @@
         <v>506</v>
       </c>
       <c r="CF7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CG7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CH7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CI7" s="5" t="s">
         <v>506</v>
@@ -12567,15 +12754,33 @@
       <c r="EA7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="EB7" s="5"/>
-      <c r="EC7" s="5"/>
-      <c r="ED7" s="5"/>
-      <c r="EE7" s="5"/>
-      <c r="EF7" s="5"/>
-      <c r="EG7" s="5"/>
-      <c r="EH7" s="5"/>
-      <c r="EI7" s="5"/>
-      <c r="EJ7" s="5"/>
+      <c r="EB7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EC7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="ED7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EE7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EF7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EG7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EH7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EI7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EJ7" s="5" t="s">
+        <v>506</v>
+      </c>
       <c r="EK7" s="5"/>
       <c r="EL7" s="5"/>
       <c r="EM7" s="5"/>
@@ -12600,8 +12805,17 @@
       <c r="FF7" s="5"/>
       <c r="FG7" s="5"/>
       <c r="FH7" s="5"/>
+      <c r="FI7" s="5"/>
+      <c r="FJ7" s="5"/>
+      <c r="FK7" s="5"/>
+      <c r="FL7" s="5"/>
+      <c r="FM7" s="5"/>
+      <c r="FN7" s="5"/>
+      <c r="FO7" s="5"/>
+      <c r="FP7" s="5"/>
+      <c r="FQ7" s="5"/>
     </row>
-    <row r="8" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>47</v>
       </c>
@@ -12663,347 +12877,365 @@
         <v>1.89</v>
       </c>
       <c r="U8" s="5">
-        <v>0.45800000000000002</v>
+        <v>0.44</v>
       </c>
       <c r="V8" s="5">
-        <v>0.67</v>
+        <v>0.6</v>
       </c>
       <c r="W8" s="5">
         <v>0.78</v>
       </c>
       <c r="X8" s="5">
+        <v>0.995</v>
+      </c>
+      <c r="Y8" s="5">
+        <v>1.37</v>
+      </c>
+      <c r="Z8" s="5">
+        <v>1.58</v>
+      </c>
+      <c r="AA8" s="5">
+        <v>2.09</v>
+      </c>
+      <c r="AB8" s="5">
+        <v>2.12</v>
+      </c>
+      <c r="AC8" s="5">
+        <v>2.4</v>
+      </c>
+      <c r="AD8" s="5">
+        <v>0.45800000000000002</v>
+      </c>
+      <c r="AE8" s="5">
+        <v>0.67</v>
+      </c>
+      <c r="AF8" s="5">
+        <v>0.78</v>
+      </c>
+      <c r="AG8" s="5">
         <v>0.98</v>
       </c>
-      <c r="Y8" s="5">
+      <c r="AH8" s="5">
         <v>1.29</v>
       </c>
-      <c r="Z8" s="5">
+      <c r="AI8" s="5">
         <v>1.72</v>
       </c>
-      <c r="AA8" s="5">
+      <c r="AJ8" s="5">
         <v>2.15</v>
       </c>
-      <c r="AB8" s="5">
+      <c r="AK8" s="5">
         <v>0.46500000000000002</v>
       </c>
-      <c r="AC8" s="5">
+      <c r="AL8" s="5">
         <v>0.55000000000000004</v>
       </c>
-      <c r="AD8" s="5">
+      <c r="AM8" s="5">
         <v>0.68400000000000005</v>
       </c>
-      <c r="AE8" s="5">
+      <c r="AN8" s="5">
         <v>1</v>
       </c>
-      <c r="AF8" s="5">
+      <c r="AO8" s="5">
         <v>1.3149999999999999</v>
       </c>
-      <c r="AG8" s="5">
+      <c r="AP8" s="5">
         <v>1.72</v>
       </c>
-      <c r="AH8" s="5">
+      <c r="AQ8" s="5">
         <v>2.15</v>
       </c>
-      <c r="AI8" s="5">
+      <c r="AR8" s="5">
         <v>1.375</v>
       </c>
-      <c r="AJ8" s="5">
+      <c r="AS8" s="5">
         <v>1.82</v>
       </c>
-      <c r="AK8" s="5">
+      <c r="AT8" s="5">
         <v>2.27</v>
       </c>
-      <c r="AL8" s="5">
+      <c r="AU8" s="5">
         <v>2.71</v>
       </c>
-      <c r="AM8" s="5">
+      <c r="AV8" s="5">
         <v>1.52</v>
       </c>
-      <c r="AN8" s="5">
+      <c r="AW8" s="5">
         <v>2.67</v>
       </c>
-      <c r="AO8" s="5">
+      <c r="AX8" s="5">
         <v>2.23</v>
       </c>
-      <c r="AP8" s="5">
+      <c r="AY8" s="5">
         <v>2.8</v>
       </c>
-      <c r="AQ8" s="5">
+      <c r="AZ8" s="5">
         <v>1.9</v>
       </c>
-      <c r="AR8" s="5">
+      <c r="BA8" s="5">
         <v>1.9</v>
       </c>
-      <c r="AS8" s="5">
+      <c r="BB8" s="5">
         <v>2.88</v>
       </c>
-      <c r="AT8" s="5">
+      <c r="BC8" s="5">
         <v>4</v>
       </c>
-      <c r="AU8" s="5">
+      <c r="BD8" s="5">
         <v>4.8</v>
       </c>
-      <c r="AV8" s="5">
+      <c r="BE8" s="5">
         <v>2.86</v>
       </c>
-      <c r="AW8" s="5">
+      <c r="BF8" s="5">
         <v>4</v>
       </c>
-      <c r="AX8" s="5">
+      <c r="BG8" s="5">
         <v>4.8</v>
       </c>
-      <c r="AY8" s="5">
+      <c r="BH8" s="5">
         <v>2.88</v>
       </c>
-      <c r="AZ8" s="5">
+      <c r="BI8" s="5">
         <v>4</v>
       </c>
-      <c r="BA8" s="5">
+      <c r="BJ8" s="5">
         <v>4.8</v>
       </c>
-      <c r="BB8" s="5">
+      <c r="BK8" s="5">
         <v>1.88</v>
       </c>
-      <c r="BC8" s="5">
+      <c r="BL8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BD8" s="5">
+      <c r="BM8" s="5">
         <v>3.75</v>
       </c>
-      <c r="BE8" s="5">
+      <c r="BN8" s="5">
         <v>4.7</v>
       </c>
-      <c r="BF8" s="5">
+      <c r="BO8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BG8" s="5">
+      <c r="BP8" s="5">
         <v>3.75</v>
       </c>
-      <c r="BH8" s="5">
+      <c r="BQ8" s="5">
         <v>4.7</v>
       </c>
-      <c r="BI8" s="5">
+      <c r="BR8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BJ8" s="5">
+      <c r="BS8" s="5">
         <v>3.75</v>
       </c>
-      <c r="BK8" s="5">
+      <c r="BT8" s="5">
         <v>4.7</v>
       </c>
-      <c r="BL8" s="5">
+      <c r="BU8" s="5">
         <v>2.25</v>
       </c>
-      <c r="BM8" s="5">
+      <c r="BV8" s="5">
         <v>2.66</v>
       </c>
-      <c r="BN8" s="5">
+      <c r="BW8" s="5">
         <v>3.08</v>
       </c>
-      <c r="BO8" s="5">
+      <c r="BX8" s="5">
         <v>3.97</v>
       </c>
-      <c r="BP8" s="5">
+      <c r="BY8" s="5">
         <v>6.72</v>
       </c>
-      <c r="BQ8" s="5">
+      <c r="BZ8" s="5">
         <v>8.93</v>
       </c>
-      <c r="BR8" s="5">
+      <c r="CA8" s="5">
         <v>6.3</v>
       </c>
-      <c r="BS8" s="5">
+      <c r="CB8" s="5">
         <v>7.8</v>
       </c>
-      <c r="BT8" s="5">
+      <c r="CC8" s="5">
         <v>4.3899999999999997</v>
       </c>
-      <c r="BU8" s="5">
+      <c r="CD8" s="5">
         <v>5.91</v>
       </c>
-      <c r="BV8" s="5">
+      <c r="CE8" s="5">
         <v>7.51</v>
       </c>
-      <c r="BW8" s="5">
+      <c r="CF8" s="5">
         <v>2.81</v>
       </c>
-      <c r="BX8" s="5">
+      <c r="CG8" s="5">
         <v>3.28</v>
       </c>
-      <c r="BY8" s="5">
+      <c r="CH8" s="5">
         <v>4.01</v>
       </c>
-      <c r="BZ8" s="5">
+      <c r="CI8" s="5">
         <v>5.32</v>
       </c>
-      <c r="CA8" s="5">
+      <c r="CJ8" s="5">
         <v>7.26</v>
       </c>
-      <c r="CB8" s="5">
+      <c r="CK8" s="5">
         <v>9.26</v>
       </c>
-      <c r="CC8" s="5">
+      <c r="CL8" s="5">
         <v>11.35</v>
       </c>
-      <c r="CD8" s="5">
+      <c r="CM8" s="5">
         <v>12.15</v>
       </c>
-      <c r="CE8" s="5">
+      <c r="CN8" s="5">
         <v>14.82</v>
       </c>
-      <c r="CF8" s="5">
+      <c r="CO8" s="5">
         <v>16.239999999999998</v>
       </c>
-      <c r="CG8" s="5">
+      <c r="CP8" s="5">
         <v>16.52</v>
       </c>
-      <c r="CH8" s="5">
+      <c r="CQ8" s="5">
         <v>18.52</v>
       </c>
-      <c r="CI8" s="5">
+      <c r="CR8" s="5">
         <v>20.61</v>
       </c>
-      <c r="CJ8" s="5">
+      <c r="CS8" s="5">
         <v>21.41</v>
       </c>
-      <c r="CK8" s="5">
+      <c r="CT8" s="5">
         <v>23.5</v>
       </c>
-      <c r="CL8" s="5">
+      <c r="CU8" s="5">
         <v>26.17</v>
       </c>
-      <c r="CM8" s="5">
+      <c r="CV8" s="5">
         <v>26.97</v>
       </c>
-      <c r="CN8" s="5">
+      <c r="CW8" s="5">
         <v>29.64</v>
       </c>
-      <c r="CO8" s="5">
+      <c r="CX8" s="5">
         <v>31.06</v>
       </c>
-      <c r="CP8" s="5">
+      <c r="CY8" s="5">
         <v>32.479999999999997</v>
       </c>
-      <c r="CQ8" s="5">
+      <c r="CZ8" s="5">
         <v>33.340000000000003</v>
       </c>
-      <c r="CR8" s="5">
+      <c r="DA8" s="5">
         <v>34.76</v>
       </c>
-      <c r="CS8" s="5">
+      <c r="DB8" s="5">
         <v>37.520000000000003</v>
       </c>
-      <c r="CT8" s="5">
+      <c r="DC8" s="5">
         <v>38.32</v>
       </c>
-      <c r="CU8" s="5">
+      <c r="DD8" s="5">
         <v>40.99</v>
       </c>
-      <c r="CV8" s="5">
+      <c r="DE8" s="5">
         <v>41.79</v>
       </c>
-      <c r="CW8" s="5">
+      <c r="DF8" s="5">
         <v>44.46</v>
       </c>
-      <c r="CX8" s="5">
+      <c r="DG8" s="5">
         <v>45.88</v>
       </c>
-      <c r="CY8" s="5">
+      <c r="DH8" s="5">
         <v>47.3</v>
       </c>
-      <c r="CZ8" s="5">
+      <c r="DI8" s="5">
         <v>48.72</v>
       </c>
-      <c r="DA8" s="5">
+      <c r="DJ8" s="5">
         <v>5.65</v>
       </c>
-      <c r="DB8" s="5">
+      <c r="DK8" s="5">
         <v>7.09</v>
       </c>
-      <c r="DC8" s="5">
+      <c r="DL8" s="5">
         <v>9.9700000000000006</v>
       </c>
-      <c r="DD8" s="5">
+      <c r="DM8" s="5">
         <v>12.08</v>
       </c>
-      <c r="DE8" s="5">
+      <c r="DN8" s="5">
         <v>13.92</v>
       </c>
-      <c r="DF8" s="5">
+      <c r="DO8" s="5">
         <v>15.07</v>
       </c>
-      <c r="DG8" s="5">
+      <c r="DP8" s="5">
         <v>16.5</v>
       </c>
-      <c r="DH8" s="5">
+      <c r="DQ8" s="5">
         <v>17.059999999999999</v>
       </c>
-      <c r="DI8" s="5">
+      <c r="DR8" s="5">
         <v>19.940000000000001</v>
       </c>
-      <c r="DJ8" s="5">
+      <c r="DS8" s="5">
         <v>22.05</v>
       </c>
-      <c r="DK8" s="5">
+      <c r="DT8" s="5">
         <v>23.89</v>
       </c>
-      <c r="DL8" s="5">
+      <c r="DU8" s="5">
         <v>26</v>
       </c>
-      <c r="DM8" s="5">
+      <c r="DV8" s="5">
         <v>27.15</v>
       </c>
-      <c r="DN8" s="5">
+      <c r="DW8" s="5">
         <v>28.99</v>
       </c>
-      <c r="DO8" s="5">
+      <c r="DX8" s="5">
         <v>30.14</v>
       </c>
-      <c r="DP8" s="5">
+      <c r="DY8" s="5">
         <v>31.57</v>
       </c>
-      <c r="DQ8" s="5">
+      <c r="DZ8" s="5">
         <v>33</v>
       </c>
-      <c r="DR8" s="5">
+      <c r="EA8" s="5">
         <v>35.01</v>
       </c>
-      <c r="DS8" s="5">
+      <c r="EB8" s="5">
         <v>36.44</v>
       </c>
-      <c r="DT8" s="5">
+      <c r="EC8" s="5">
         <v>39.229999999999997</v>
       </c>
-      <c r="DU8" s="5">
+      <c r="ED8" s="5">
         <v>41.07</v>
       </c>
-      <c r="DV8" s="5">
+      <c r="EE8" s="5">
         <v>42.22</v>
       </c>
-      <c r="DW8" s="5">
+      <c r="EF8" s="5">
         <v>44.06</v>
       </c>
-      <c r="DX8" s="5">
+      <c r="EG8" s="5">
         <v>45.21</v>
       </c>
-      <c r="DY8" s="5">
+      <c r="EH8" s="5">
         <v>46.64</v>
       </c>
-      <c r="DZ8" s="5">
+      <c r="EI8" s="5">
         <v>48.07</v>
       </c>
-      <c r="EA8" s="5">
+      <c r="EJ8" s="5">
         <v>49.5</v>
       </c>
-      <c r="EB8" s="5"/>
-      <c r="EC8" s="5"/>
-      <c r="ED8" s="5"/>
-      <c r="EE8" s="5"/>
-      <c r="EF8" s="5"/>
-      <c r="EG8" s="5"/>
-      <c r="EH8" s="5"/>
-      <c r="EI8" s="5"/>
-      <c r="EJ8" s="5"/>
       <c r="EK8" s="5"/>
       <c r="EL8" s="5"/>
       <c r="EM8" s="5"/>
@@ -13028,8 +13260,17 @@
       <c r="FF8" s="5"/>
       <c r="FG8" s="5"/>
       <c r="FH8" s="5"/>
+      <c r="FI8" s="5"/>
+      <c r="FJ8" s="5"/>
+      <c r="FK8" s="5"/>
+      <c r="FL8" s="5"/>
+      <c r="FM8" s="5"/>
+      <c r="FN8" s="5"/>
+      <c r="FO8" s="5"/>
+      <c r="FP8" s="5"/>
+      <c r="FQ8" s="5"/>
     </row>
-    <row r="9" spans="1:164" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>50</v>
       </c>
@@ -13090,348 +13331,366 @@
       <c r="T9" s="5">
         <v>17.5</v>
       </c>
-      <c r="U9" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="V9" s="5" t="s">
-        <v>76</v>
+      <c r="U9" s="5">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="V9" s="5">
+        <v>2.9</v>
       </c>
       <c r="W9" s="5">
-        <v>8.8000000000000007</v>
+        <v>3.8</v>
       </c>
       <c r="X9" s="5">
+        <v>4.7</v>
+      </c>
+      <c r="Y9" s="5">
+        <v>6.3</v>
+      </c>
+      <c r="Z9" s="5">
+        <v>7.5</v>
+      </c>
+      <c r="AA9" s="5">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="AB9" s="5">
         <v>10</v>
       </c>
-      <c r="Y9" s="5">
-        <v>10</v>
-      </c>
-      <c r="Z9" s="5">
-        <v>10</v>
-      </c>
-      <c r="AA9" s="5">
-        <v>11</v>
-      </c>
-      <c r="AB9" s="5">
-        <v>7.3</v>
-      </c>
-      <c r="AC9" s="5" t="s">
-        <v>76</v>
+      <c r="AC9" s="5">
+        <v>11.3</v>
       </c>
       <c r="AD9" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="AE9" s="5">
-        <v>10</v>
+      <c r="AE9" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="AF9" s="5">
-        <v>10</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="AG9" s="5">
         <v>10</v>
       </c>
       <c r="AH9" s="5">
+        <v>10</v>
+      </c>
+      <c r="AI9" s="5">
+        <v>10</v>
+      </c>
+      <c r="AJ9" s="5">
         <v>11</v>
       </c>
-      <c r="AI9" s="5">
+      <c r="AK9" s="5">
+        <v>7.3</v>
+      </c>
+      <c r="AL9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AM9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="AN9" s="5">
+        <v>10</v>
+      </c>
+      <c r="AO9" s="5">
+        <v>10</v>
+      </c>
+      <c r="AP9" s="5">
+        <v>10</v>
+      </c>
+      <c r="AQ9" s="5">
+        <v>11</v>
+      </c>
+      <c r="AR9" s="5">
         <v>16</v>
       </c>
-      <c r="AJ9" s="5">
+      <c r="AS9" s="5">
         <v>16</v>
       </c>
-      <c r="AK9" s="5">
+      <c r="AT9" s="5">
         <v>16</v>
       </c>
-      <c r="AL9" s="5">
+      <c r="AU9" s="5">
         <v>23</v>
       </c>
-      <c r="AM9" s="5">
+      <c r="AV9" s="5">
         <v>9.6999999999999993</v>
       </c>
-      <c r="AN9" s="5">
+      <c r="AW9" s="5">
         <v>16</v>
       </c>
-      <c r="AO9" s="5">
+      <c r="AX9" s="5">
         <v>11</v>
       </c>
-      <c r="AP9" s="5">
+      <c r="AY9" s="5">
         <v>15</v>
       </c>
-      <c r="AQ9" s="5">
+      <c r="AZ9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="AR9" s="5">
+      <c r="BA9" s="5">
         <v>15.3</v>
       </c>
-      <c r="AS9" s="5">
+      <c r="BB9" s="5">
         <v>30.3</v>
       </c>
-      <c r="AT9" s="5">
+      <c r="BC9" s="5">
         <v>30.3</v>
       </c>
-      <c r="AU9" s="5">
+      <c r="BD9" s="5">
         <v>30.3</v>
       </c>
-      <c r="AV9" s="5">
+      <c r="BE9" s="5">
         <v>26.4</v>
       </c>
-      <c r="AW9" s="5">
+      <c r="BF9" s="5">
         <v>26.4</v>
       </c>
-      <c r="AX9" s="5">
+      <c r="BG9" s="5">
         <v>26.4</v>
       </c>
-      <c r="AY9" s="5">
+      <c r="BH9" s="5">
         <v>16.899999999999999</v>
       </c>
-      <c r="AZ9" s="5">
+      <c r="BI9" s="5">
         <v>16.899999999999999</v>
       </c>
-      <c r="BA9" s="5">
+      <c r="BJ9" s="5">
         <v>16.899999999999999</v>
       </c>
-      <c r="BB9" s="5">
+      <c r="BK9" s="5">
         <v>18.8</v>
       </c>
-      <c r="BC9" s="5">
+      <c r="BL9" s="5">
         <v>24.1</v>
       </c>
-      <c r="BD9" s="5">
+      <c r="BM9" s="5">
         <v>29.6</v>
       </c>
-      <c r="BE9" s="5">
+      <c r="BN9" s="5">
         <v>29.6</v>
       </c>
-      <c r="BF9" s="5">
+      <c r="BO9" s="5">
         <v>26.3</v>
       </c>
-      <c r="BG9" s="5">
+      <c r="BP9" s="5">
         <v>26.3</v>
       </c>
-      <c r="BH9" s="5">
+      <c r="BQ9" s="5">
         <v>26.3</v>
       </c>
-      <c r="BI9" s="5">
+      <c r="BR9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BJ9" s="5">
+      <c r="BS9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BK9" s="5">
+      <c r="BT9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BL9" s="5">
+      <c r="BU9" s="5">
         <v>20</v>
       </c>
-      <c r="BM9" s="5">
+      <c r="BV9" s="5">
         <v>27</v>
       </c>
-      <c r="BN9" s="5">
+      <c r="BW9" s="5">
         <v>27</v>
-      </c>
-      <c r="BO9" s="5">
-        <v>27</v>
-      </c>
-      <c r="BP9" s="5">
-        <v>22</v>
-      </c>
-      <c r="BQ9" s="5">
-        <v>24</v>
-      </c>
-      <c r="BR9" s="5">
-        <v>26.5</v>
-      </c>
-      <c r="BS9" s="5">
-        <v>26.5</v>
-      </c>
-      <c r="BT9" s="5">
-        <v>21.1</v>
-      </c>
-      <c r="BU9" s="5">
-        <v>18.5</v>
-      </c>
-      <c r="BV9" s="5">
-        <v>18.5</v>
-      </c>
-      <c r="BW9" s="5">
-        <v>17.5</v>
       </c>
       <c r="BX9" s="5">
         <v>27</v>
       </c>
       <c r="BY9" s="5">
+        <v>22</v>
+      </c>
+      <c r="BZ9" s="5">
+        <v>24</v>
+      </c>
+      <c r="CA9" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="CB9" s="5">
+        <v>26.5</v>
+      </c>
+      <c r="CC9" s="5">
+        <v>21.1</v>
+      </c>
+      <c r="CD9" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="CE9" s="5">
+        <v>18.5</v>
+      </c>
+      <c r="CF9" s="5">
+        <v>17.5</v>
+      </c>
+      <c r="CG9" s="5">
         <v>27</v>
       </c>
-      <c r="BZ9" s="5">
+      <c r="CH9" s="5">
+        <v>27</v>
+      </c>
+      <c r="CI9" s="5">
         <v>16.100000000000001</v>
       </c>
-      <c r="CA9" s="5">
+      <c r="CJ9" s="5">
         <v>21.2</v>
       </c>
-      <c r="CB9" s="5">
+      <c r="CK9" s="5">
         <v>22.5</v>
       </c>
-      <c r="CC9" s="5">
+      <c r="CL9" s="5">
         <v>30.2</v>
       </c>
-      <c r="CD9" s="5">
+      <c r="CM9" s="5">
         <v>33.700000000000003</v>
       </c>
-      <c r="CE9" s="5">
+      <c r="CN9" s="5">
         <v>34.5</v>
       </c>
-      <c r="CF9" s="5">
+      <c r="CO9" s="5">
         <v>38.5</v>
       </c>
-      <c r="CG9" s="5">
+      <c r="CP9" s="5">
         <v>43.7</v>
       </c>
-      <c r="CH9" s="5">
+      <c r="CQ9" s="5">
         <v>45</v>
       </c>
-      <c r="CI9" s="5">
+      <c r="CR9" s="5">
         <v>52.7</v>
       </c>
-      <c r="CJ9" s="5">
+      <c r="CS9" s="5">
         <v>56.2</v>
       </c>
-      <c r="CK9" s="5">
+      <c r="CT9" s="5">
         <v>63.9</v>
       </c>
-      <c r="CL9" s="5">
+      <c r="CU9" s="5">
         <v>64.7</v>
       </c>
-      <c r="CM9" s="5">
+      <c r="CV9" s="5">
         <v>68.2</v>
       </c>
-      <c r="CN9" s="5">
+      <c r="CW9" s="5">
         <v>69</v>
       </c>
-      <c r="CO9" s="5">
+      <c r="CX9" s="5">
         <v>73</v>
       </c>
-      <c r="CP9" s="5">
+      <c r="CY9" s="5">
         <v>77</v>
       </c>
-      <c r="CQ9" s="5">
+      <c r="CZ9" s="5">
         <v>79.5</v>
       </c>
-      <c r="CR9" s="5">
+      <c r="DA9" s="5">
         <v>83.5</v>
       </c>
-      <c r="CS9" s="5">
+      <c r="DB9" s="5">
         <v>94.9</v>
       </c>
-      <c r="CT9" s="5">
+      <c r="DC9" s="5">
         <v>98.4</v>
       </c>
-      <c r="CU9" s="5">
+      <c r="DD9" s="5">
         <v>99.2</v>
       </c>
-      <c r="CV9" s="5">
+      <c r="DE9" s="5">
         <v>102.7</v>
       </c>
-      <c r="CW9" s="5">
+      <c r="DF9" s="5">
         <v>103.5</v>
       </c>
-      <c r="CX9" s="5">
+      <c r="DG9" s="5">
         <v>107.5</v>
       </c>
-      <c r="CY9" s="5">
+      <c r="DH9" s="5">
         <v>111.5</v>
       </c>
-      <c r="CZ9" s="5">
+      <c r="DI9" s="5">
         <v>115.5</v>
       </c>
-      <c r="DA9" s="5">
+      <c r="DJ9" s="5">
         <v>16.100000000000001</v>
       </c>
-      <c r="DB9" s="5">
+      <c r="DK9" s="5">
         <v>21.5</v>
       </c>
-      <c r="DC9" s="5">
+      <c r="DL9" s="5">
         <v>22.9</v>
       </c>
-      <c r="DD9" s="5">
+      <c r="DM9" s="5">
         <v>30.2</v>
       </c>
-      <c r="DE9" s="5">
+      <c r="DN9" s="5">
         <v>34</v>
       </c>
-      <c r="DF9" s="5">
+      <c r="DO9" s="5">
         <v>34.700000000000003</v>
       </c>
-      <c r="DG9" s="5">
+      <c r="DP9" s="5">
         <v>39.700000000000003</v>
       </c>
-      <c r="DH9" s="5">
+      <c r="DQ9" s="5">
         <v>44.4</v>
       </c>
-      <c r="DI9" s="5">
+      <c r="DR9" s="5">
         <v>45.8</v>
       </c>
-      <c r="DJ9" s="5">
+      <c r="DS9" s="5">
         <v>53.1</v>
       </c>
-      <c r="DK9" s="5">
+      <c r="DT9" s="5">
         <v>56.9</v>
       </c>
-      <c r="DL9" s="5">
+      <c r="DU9" s="5">
         <v>64.2</v>
       </c>
-      <c r="DM9" s="5">
+      <c r="DV9" s="5">
         <v>64.900000000000006</v>
       </c>
-      <c r="DN9" s="5">
+      <c r="DW9" s="5">
         <v>68.7</v>
       </c>
-      <c r="DO9" s="5">
+      <c r="DX9" s="5">
         <v>69.400000000000006</v>
       </c>
-      <c r="DP9" s="5">
+      <c r="DY9" s="5">
         <v>74.400000000000006</v>
       </c>
-      <c r="DQ9" s="5">
+      <c r="DZ9" s="5">
         <v>79.400000000000006</v>
       </c>
-      <c r="DR9" s="5">
+      <c r="EA9" s="5">
         <v>80.5</v>
       </c>
-      <c r="DS9" s="5">
+      <c r="EB9" s="5">
         <v>85.5</v>
       </c>
-      <c r="DT9" s="5">
+      <c r="EC9" s="5">
         <v>95.1</v>
       </c>
-      <c r="DU9" s="5">
+      <c r="ED9" s="5">
         <v>98.9</v>
       </c>
-      <c r="DV9" s="5">
+      <c r="EE9" s="5">
         <v>99.6</v>
       </c>
-      <c r="DW9" s="5">
+      <c r="EF9" s="5">
         <v>103.4</v>
       </c>
-      <c r="DX9" s="5">
+      <c r="EG9" s="5">
         <v>104.1</v>
       </c>
-      <c r="DY9" s="5">
+      <c r="EH9" s="5">
         <v>109.1</v>
       </c>
-      <c r="DZ9" s="5">
+      <c r="EI9" s="5">
         <v>114.1</v>
       </c>
-      <c r="EA9" s="5">
+      <c r="EJ9" s="5">
         <v>119.1</v>
       </c>
-      <c r="EB9" s="5"/>
-      <c r="EC9" s="5"/>
-      <c r="ED9" s="5"/>
-      <c r="EE9" s="5"/>
-      <c r="EF9" s="5"/>
-      <c r="EG9" s="5"/>
-      <c r="EH9" s="5"/>
-      <c r="EI9" s="5"/>
-      <c r="EJ9" s="5"/>
       <c r="EK9" s="5"/>
       <c r="EL9" s="5"/>
       <c r="EM9" s="5"/>
@@ -13456,8 +13715,17 @@
       <c r="FF9" s="5"/>
       <c r="FG9" s="5"/>
       <c r="FH9" s="5"/>
+      <c r="FI9" s="5"/>
+      <c r="FJ9" s="5"/>
+      <c r="FK9" s="5"/>
+      <c r="FL9" s="5"/>
+      <c r="FM9" s="5"/>
+      <c r="FN9" s="5"/>
+      <c r="FO9" s="5"/>
+      <c r="FP9" s="5"/>
+      <c r="FQ9" s="5"/>
     </row>
-    <row r="10" spans="1:164" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:173" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>49</v>
       </c>
@@ -13514,32 +13782,32 @@
       <c r="T10" s="5">
         <v>20</v>
       </c>
-      <c r="U10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="V10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="W10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="X10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AB10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AC10" s="5" t="s">
-        <v>63</v>
+      <c r="U10" s="5">
+        <v>10</v>
+      </c>
+      <c r="V10" s="5">
+        <v>10</v>
+      </c>
+      <c r="W10" s="5">
+        <v>10</v>
+      </c>
+      <c r="X10" s="5">
+        <v>15</v>
+      </c>
+      <c r="Y10" s="5">
+        <v>15</v>
+      </c>
+      <c r="Z10" s="5">
+        <v>15</v>
+      </c>
+      <c r="AA10" s="5">
+        <v>15</v>
+      </c>
+      <c r="AB10" s="5">
+        <v>20</v>
+      </c>
+      <c r="AC10" s="5">
+        <v>20</v>
       </c>
       <c r="AD10" s="5" t="s">
         <v>63</v>
@@ -13556,53 +13824,53 @@
       <c r="AH10" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AI10" s="5">
+      <c r="AI10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AK10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AM10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AN10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AO10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AP10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AQ10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AR10" s="5">
         <v>20</v>
       </c>
-      <c r="AJ10" s="5">
+      <c r="AS10" s="5">
         <v>20</v>
       </c>
-      <c r="AK10" s="5">
+      <c r="AT10" s="5">
         <v>20</v>
       </c>
-      <c r="AL10" s="5">
+      <c r="AU10" s="5">
         <v>30</v>
       </c>
-      <c r="AM10" s="5">
+      <c r="AV10" s="5">
         <v>10</v>
       </c>
-      <c r="AN10" s="5">
+      <c r="AW10" s="5">
         <v>20</v>
       </c>
-      <c r="AO10" s="5">
+      <c r="AX10" s="5">
         <v>19.600000000000001</v>
-      </c>
-      <c r="AP10" s="5">
-        <v>20</v>
-      </c>
-      <c r="AQ10" s="5">
-        <v>20</v>
-      </c>
-      <c r="AR10" s="5">
-        <v>16</v>
-      </c>
-      <c r="AS10" s="5">
-        <v>32</v>
-      </c>
-      <c r="AT10" s="5">
-        <v>32</v>
-      </c>
-      <c r="AU10" s="5">
-        <v>32</v>
-      </c>
-      <c r="AV10" s="5">
-        <v>32</v>
-      </c>
-      <c r="AW10" s="5">
-        <v>32</v>
-      </c>
-      <c r="AX10" s="5">
-        <v>32</v>
       </c>
       <c r="AY10" s="5">
         <v>20</v>
@@ -13611,13 +13879,13 @@
         <v>20</v>
       </c>
       <c r="BA10" s="5">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="BB10" s="5">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="BC10" s="5">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="BD10" s="5">
         <v>32</v>
@@ -13632,7 +13900,7 @@
         <v>32</v>
       </c>
       <c r="BH10" s="5">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="BI10" s="5">
         <v>20</v>
@@ -13647,215 +13915,233 @@
         <v>25</v>
       </c>
       <c r="BM10" s="5">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="BN10" s="5">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="BO10" s="5">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="BP10" s="5">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="BQ10" s="5">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="BR10" s="5">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="BS10" s="5">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="BT10" s="5">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="BU10" s="5">
         <v>25</v>
       </c>
       <c r="BV10" s="5">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="BW10" s="5">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="BX10" s="5">
         <v>30</v>
       </c>
       <c r="BY10" s="5">
+        <v>25</v>
+      </c>
+      <c r="BZ10" s="5">
         <v>30</v>
       </c>
-      <c r="BZ10" s="5">
+      <c r="CA10" s="5">
+        <v>30</v>
+      </c>
+      <c r="CB10" s="5">
+        <v>30</v>
+      </c>
+      <c r="CC10" s="5">
+        <v>30</v>
+      </c>
+      <c r="CD10" s="5">
+        <v>25</v>
+      </c>
+      <c r="CE10" s="5">
+        <v>25</v>
+      </c>
+      <c r="CF10" s="5">
+        <v>25</v>
+      </c>
+      <c r="CG10" s="5">
+        <v>30</v>
+      </c>
+      <c r="CH10" s="5">
+        <v>30</v>
+      </c>
+      <c r="CI10" s="5">
         <v>20</v>
       </c>
-      <c r="CA10" s="5">
+      <c r="CJ10" s="5">
         <v>25</v>
       </c>
-      <c r="CB10" s="5">
+      <c r="CK10" s="5">
         <v>25</v>
       </c>
-      <c r="CC10" s="5">
+      <c r="CL10" s="5">
         <v>35</v>
       </c>
-      <c r="CD10" s="5">
+      <c r="CM10" s="5">
         <v>40</v>
       </c>
-      <c r="CE10" s="5">
+      <c r="CN10" s="5">
         <v>40</v>
       </c>
-      <c r="CF10" s="5">
+      <c r="CO10" s="5">
         <v>45</v>
       </c>
-      <c r="CG10" s="5">
+      <c r="CP10" s="5">
         <v>50</v>
       </c>
-      <c r="CH10" s="5">
+      <c r="CQ10" s="5">
         <v>50</v>
       </c>
-      <c r="CI10" s="5">
+      <c r="CR10" s="5">
         <v>60</v>
       </c>
-      <c r="CJ10" s="5">
+      <c r="CS10" s="5">
         <v>70</v>
       </c>
-      <c r="CK10" s="5">
+      <c r="CT10" s="5">
         <v>80</v>
       </c>
-      <c r="CL10" s="5">
+      <c r="CU10" s="5">
         <v>80</v>
       </c>
-      <c r="CM10" s="5">
+      <c r="CV10" s="5">
         <v>80</v>
       </c>
-      <c r="CN10" s="5">
+      <c r="CW10" s="5">
         <v>80</v>
       </c>
-      <c r="CO10" s="5">
+      <c r="CX10" s="5">
         <v>90</v>
       </c>
-      <c r="CP10" s="5">
+      <c r="CY10" s="5">
         <v>90</v>
       </c>
-      <c r="CQ10" s="5">
+      <c r="CZ10" s="5">
         <v>90</v>
       </c>
-      <c r="CR10" s="5">
+      <c r="DA10" s="5">
         <v>100</v>
       </c>
-      <c r="CS10" s="5">
+      <c r="DB10" s="5">
         <v>110</v>
       </c>
-      <c r="CT10" s="5">
+      <c r="DC10" s="5">
         <v>110</v>
       </c>
-      <c r="CU10" s="5">
+      <c r="DD10" s="5">
         <v>110</v>
       </c>
-      <c r="CV10" s="5">
+      <c r="DE10" s="5">
         <v>125</v>
       </c>
-      <c r="CW10" s="5">
+      <c r="DF10" s="5">
         <v>125</v>
       </c>
-      <c r="CX10" s="5">
+      <c r="DG10" s="5">
         <v>125</v>
       </c>
-      <c r="CY10" s="5">
+      <c r="DH10" s="5">
         <v>125</v>
       </c>
-      <c r="CZ10" s="5">
+      <c r="DI10" s="5">
         <v>150</v>
       </c>
-      <c r="DA10" s="5">
+      <c r="DJ10" s="5">
         <v>20</v>
       </c>
-      <c r="DB10" s="5">
+      <c r="DK10" s="5">
         <v>25</v>
       </c>
-      <c r="DC10" s="5">
+      <c r="DL10" s="5">
         <v>30</v>
       </c>
-      <c r="DD10" s="5">
+      <c r="DM10" s="5">
         <v>35</v>
       </c>
-      <c r="DE10" s="5">
+      <c r="DN10" s="5">
         <v>40</v>
       </c>
-      <c r="DF10" s="5">
+      <c r="DO10" s="5">
         <v>40</v>
       </c>
-      <c r="DG10" s="5">
+      <c r="DP10" s="5">
         <v>45</v>
       </c>
-      <c r="DH10" s="5">
+      <c r="DQ10" s="5">
         <v>50</v>
       </c>
-      <c r="DI10" s="5">
+      <c r="DR10" s="5">
         <v>60</v>
       </c>
-      <c r="DJ10" s="5">
+      <c r="DS10" s="5">
         <v>60</v>
       </c>
-      <c r="DK10" s="5">
+      <c r="DT10" s="5">
         <v>70</v>
       </c>
-      <c r="DL10" s="5">
+      <c r="DU10" s="5">
         <v>80</v>
       </c>
-      <c r="DM10" s="5">
+      <c r="DV10" s="5">
         <v>80</v>
       </c>
-      <c r="DN10" s="5">
+      <c r="DW10" s="5">
         <v>80</v>
       </c>
-      <c r="DO10" s="5">
+      <c r="DX10" s="5">
         <v>80</v>
       </c>
-      <c r="DP10" s="5">
+      <c r="DY10" s="5">
         <v>90</v>
       </c>
-      <c r="DQ10" s="5">
+      <c r="DZ10" s="5">
         <v>90</v>
       </c>
-      <c r="DR10" s="5">
+      <c r="EA10" s="5">
         <v>90</v>
       </c>
-      <c r="DS10" s="5">
+      <c r="EB10" s="5">
         <v>100</v>
       </c>
-      <c r="DT10" s="5">
+      <c r="EC10" s="5">
         <v>110</v>
       </c>
-      <c r="DU10" s="5">
+      <c r="ED10" s="5">
         <v>110</v>
       </c>
-      <c r="DV10" s="5">
+      <c r="EE10" s="5">
         <v>110</v>
       </c>
-      <c r="DW10" s="5">
+      <c r="EF10" s="5">
         <v>125</v>
       </c>
-      <c r="DX10" s="5">
+      <c r="EG10" s="5">
         <v>125</v>
       </c>
-      <c r="DY10" s="5">
+      <c r="EH10" s="5">
         <v>125</v>
       </c>
-      <c r="DZ10" s="5">
+      <c r="EI10" s="5">
         <v>150</v>
       </c>
-      <c r="EA10" s="5">
+      <c r="EJ10" s="5">
         <v>150</v>
       </c>
-      <c r="EB10" s="5"/>
-      <c r="EC10" s="5"/>
-      <c r="ED10" s="5"/>
-      <c r="EE10" s="5"/>
-      <c r="EF10" s="5"/>
-      <c r="EG10" s="5"/>
-      <c r="EH10" s="5"/>
-      <c r="EI10" s="5"/>
-      <c r="EJ10" s="5"/>
       <c r="EK10" s="5"/>
       <c r="EL10" s="5"/>
       <c r="EM10" s="5"/>
@@ -13880,8 +14166,17 @@
       <c r="FF10" s="5"/>
       <c r="FG10" s="5"/>
       <c r="FH10" s="5"/>
+      <c r="FI10" s="5"/>
+      <c r="FJ10" s="5"/>
+      <c r="FK10" s="5"/>
+      <c r="FL10" s="5"/>
+      <c r="FM10" s="5"/>
+      <c r="FN10" s="5"/>
+      <c r="FO10" s="5"/>
+      <c r="FP10" s="5"/>
+      <c r="FQ10" s="5"/>
     </row>
-    <row r="11" spans="1:164" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:173" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>58</v>
       </c>
@@ -14069,17 +14364,17 @@
       <c r="BK11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="BL11" s="15">
-        <v>40</v>
-      </c>
-      <c r="BM11" s="15">
-        <v>40</v>
-      </c>
-      <c r="BN11" s="15">
-        <v>40</v>
-      </c>
-      <c r="BO11" s="15">
-        <v>40</v>
+      <c r="BL11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BM11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BN11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BO11" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="BP11" s="15" t="s">
         <v>37</v>
@@ -14096,47 +14391,47 @@
       <c r="BT11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="BU11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="BV11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="BW11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="BX11" s="15" t="s">
-        <v>37</v>
+      <c r="BU11" s="15">
+        <v>40</v>
+      </c>
+      <c r="BV11" s="15">
+        <v>40</v>
+      </c>
+      <c r="BW11" s="15">
+        <v>40</v>
+      </c>
+      <c r="BX11" s="15">
+        <v>40</v>
       </c>
       <c r="BY11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="BZ11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CA11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CB11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CC11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CD11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CE11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CF11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CG11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CH11" s="15">
-        <v>78.400000000000006</v>
+      <c r="BZ11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CA11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CB11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CC11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CD11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CE11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CF11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CG11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CH11" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="CI11" s="15">
         <v>78.400000000000006</v>
@@ -14273,15 +14568,33 @@
       <c r="EA11" s="15">
         <v>78.400000000000006</v>
       </c>
-      <c r="EB11" s="15"/>
-      <c r="EC11" s="15"/>
-      <c r="ED11" s="15"/>
-      <c r="EE11" s="15"/>
-      <c r="EF11" s="15"/>
-      <c r="EG11" s="15"/>
-      <c r="EH11" s="15"/>
-      <c r="EI11" s="15"/>
-      <c r="EJ11" s="15"/>
+      <c r="EB11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EC11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="ED11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EE11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EF11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EG11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EH11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EI11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EJ11" s="15">
+        <v>78.400000000000006</v>
+      </c>
       <c r="EK11" s="15"/>
       <c r="EL11" s="15"/>
       <c r="EM11" s="15"/>
@@ -14306,8 +14619,17 @@
       <c r="FF11" s="15"/>
       <c r="FG11" s="15"/>
       <c r="FH11" s="15"/>
+      <c r="FI11" s="15"/>
+      <c r="FJ11" s="15"/>
+      <c r="FK11" s="15"/>
+      <c r="FL11" s="15"/>
+      <c r="FM11" s="15"/>
+      <c r="FN11" s="15"/>
+      <c r="FO11" s="15"/>
+      <c r="FP11" s="15"/>
+      <c r="FQ11" s="15"/>
     </row>
-    <row r="12" spans="1:164" ht="60" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:173" ht="60" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>51</v>
       </c>
@@ -14369,37 +14691,37 @@
         <v>72</v>
       </c>
       <c r="U12" s="15" t="s">
-        <v>40</v>
+        <v>523</v>
       </c>
       <c r="V12" s="15" t="s">
-        <v>40</v>
+        <v>523</v>
       </c>
       <c r="W12" s="15" t="s">
-        <v>71</v>
+        <v>524</v>
       </c>
       <c r="X12" s="15" t="s">
-        <v>71</v>
+        <v>524</v>
       </c>
       <c r="Y12" s="15" t="s">
-        <v>71</v>
+        <v>524</v>
       </c>
       <c r="Z12" s="15" t="s">
-        <v>71</v>
+        <v>525</v>
       </c>
       <c r="AA12" s="15" t="s">
-        <v>71</v>
+        <v>525</v>
       </c>
       <c r="AB12" s="15" t="s">
-        <v>40</v>
+        <v>526</v>
       </c>
       <c r="AC12" s="15" t="s">
-        <v>40</v>
+        <v>526</v>
       </c>
       <c r="AD12" s="15" t="s">
         <v>40</v>
       </c>
       <c r="AE12" s="15" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="AF12" s="15" t="s">
         <v>71</v>
@@ -14411,64 +14733,64 @@
         <v>71</v>
       </c>
       <c r="AI12" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AJ12" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AK12" s="15" t="s">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="AL12" s="15" t="s">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="AM12" s="15" t="s">
         <v>40</v>
       </c>
       <c r="AN12" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AO12" s="15" t="s">
         <v>71</v>
       </c>
       <c r="AP12" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AQ12" s="15" t="s">
         <v>71</v>
       </c>
       <c r="AR12" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AS12" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="AT12" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="AU12" s="15" t="s">
         <v>74</v>
       </c>
       <c r="AV12" s="15" t="s">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="AW12" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="AX12" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AY12" s="15" t="s">
         <v>74</v>
       </c>
       <c r="AZ12" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="BA12" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="BB12" s="15" t="s">
         <v>74</v>
-      </c>
-      <c r="BA12" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="BB12" s="15" t="s">
-        <v>128</v>
       </c>
       <c r="BC12" s="15" t="s">
         <v>74</v>
@@ -14486,7 +14808,7 @@
         <v>74</v>
       </c>
       <c r="BH12" s="15" t="s">
-        <v>133</v>
+        <v>74</v>
       </c>
       <c r="BI12" s="15" t="s">
         <v>74</v>
@@ -14495,221 +14817,239 @@
         <v>74</v>
       </c>
       <c r="BK12" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL12" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="BL12" s="15" t="s">
+      <c r="BM12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BN12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BO12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BP12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BQ12" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="BR12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BS12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BT12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="BU12" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="BM12" s="15" t="s">
+      <c r="BV12" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="BN12" s="15" t="s">
+      <c r="BW12" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="BO12" s="15" t="s">
+      <c r="BX12" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="BP12" s="15" t="s">
+      <c r="BY12" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="BQ12" s="15" t="s">
+      <c r="BZ12" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="BR12" s="15" t="s">
+      <c r="CA12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="BS12" s="15" t="s">
+      <c r="CB12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="BT12" s="15" t="s">
+      <c r="CC12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="BU12" s="15" t="s">
+      <c r="CD12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="BV12" s="15" t="s">
+      <c r="CE12" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="BW12" s="15" t="s">
+      <c r="CF12" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="BX12" s="15" t="s">
+      <c r="CG12" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="BY12" s="15" t="s">
+      <c r="CH12" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="BZ12" s="15" t="s">
+      <c r="CI12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CA12" s="15" t="s">
+      <c r="CJ12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CB12" s="15" t="s">
+      <c r="CK12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CC12" s="15" t="s">
+      <c r="CL12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CD12" s="15" t="s">
+      <c r="CM12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CE12" s="15" t="s">
+      <c r="CN12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CF12" s="15" t="s">
+      <c r="CO12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CG12" s="15" t="s">
+      <c r="CP12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="CH12" s="15" t="s">
+      <c r="CQ12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="CI12" s="15" t="s">
+      <c r="CR12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="CJ12" s="15" t="s">
+      <c r="CS12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="CK12" s="15" t="s">
+      <c r="CT12" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="CL12" s="15" t="s">
+      <c r="CU12" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="CM12" s="15" t="s">
+      <c r="CV12" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="CN12" s="15" t="s">
+      <c r="CW12" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="CO12" s="15" t="s">
+      <c r="CX12" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="CP12" s="15" t="s">
+      <c r="CY12" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="CQ12" s="15" t="s">
+      <c r="CZ12" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="CR12" s="15" t="s">
+      <c r="DA12" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="CS12" s="15" t="s">
+      <c r="DB12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CT12" s="15" t="s">
+      <c r="DC12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CU12" s="15" t="s">
+      <c r="DD12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CV12" s="15" t="s">
+      <c r="DE12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CW12" s="15" t="s">
+      <c r="DF12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CX12" s="15" t="s">
+      <c r="DG12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CY12" s="15" t="s">
+      <c r="DH12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="CZ12" s="15" t="s">
+      <c r="DI12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DA12" s="15" t="s">
+      <c r="DJ12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DB12" s="15" t="s">
+      <c r="DK12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DC12" s="15" t="s">
+      <c r="DL12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DD12" s="15" t="s">
+      <c r="DM12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DE12" s="15" t="s">
+      <c r="DN12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DF12" s="15" t="s">
+      <c r="DO12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DG12" s="15" t="s">
+      <c r="DP12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DH12" s="15" t="s">
+      <c r="DQ12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="DI12" s="15" t="s">
+      <c r="DR12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="DJ12" s="15" t="s">
+      <c r="DS12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="DK12" s="15" t="s">
+      <c r="DT12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="DL12" s="15" t="s">
+      <c r="DU12" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="DM12" s="15" t="s">
+      <c r="DV12" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="DN12" s="15" t="s">
+      <c r="DW12" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="DO12" s="15" t="s">
+      <c r="DX12" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="DP12" s="15" t="s">
+      <c r="DY12" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="DQ12" s="15" t="s">
+      <c r="DZ12" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="DR12" s="15" t="s">
+      <c r="EA12" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="DS12" s="15" t="s">
+      <c r="EB12" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="DT12" s="15" t="s">
+      <c r="EC12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DU12" s="15" t="s">
+      <c r="ED12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DV12" s="15" t="s">
+      <c r="EE12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DW12" s="15" t="s">
+      <c r="EF12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DX12" s="15" t="s">
+      <c r="EG12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DY12" s="15" t="s">
+      <c r="EH12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DZ12" s="15" t="s">
+      <c r="EI12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EA12" s="15" t="s">
+      <c r="EJ12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EB12" s="15"/>
-      <c r="EC12" s="15"/>
-      <c r="ED12" s="15"/>
-      <c r="EE12" s="15"/>
-      <c r="EF12" s="15"/>
-      <c r="EG12" s="15"/>
-      <c r="EH12" s="15"/>
-      <c r="EI12" s="15"/>
-      <c r="EJ12" s="15"/>
       <c r="EK12" s="15"/>
       <c r="EL12" s="15"/>
       <c r="EM12" s="15"/>
@@ -14732,8 +15072,17 @@
       <c r="FD12" s="15"/>
       <c r="FE12" s="15"/>
       <c r="FF12" s="15"/>
+      <c r="FG12" s="15"/>
+      <c r="FH12" s="15"/>
+      <c r="FI12" s="15"/>
+      <c r="FJ12" s="15"/>
+      <c r="FK12" s="15"/>
+      <c r="FL12" s="15"/>
+      <c r="FM12" s="15"/>
+      <c r="FN12" s="15"/>
+      <c r="FO12" s="15"/>
     </row>
-    <row r="13" spans="1:164" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:173" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
         <v>54</v>
       </c>
@@ -14934,25 +15283,25 @@
         <v>56</v>
       </c>
       <c r="BP13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BQ13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BR13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BS13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BT13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BU13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BV13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BW13" s="12" t="s">
         <v>56</v>
@@ -14961,34 +15310,34 @@
         <v>56</v>
       </c>
       <c r="BY13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="BZ13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="CA13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="CB13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="CC13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="CD13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="CE13" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="CF13" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="BZ13" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="CA13" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="CB13" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="CC13" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="CD13" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="CE13" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="CF13" s="12" t="s">
-        <v>200</v>
-      </c>
       <c r="CG13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CH13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CI13" s="12" t="s">
         <v>200</v>
@@ -15125,15 +15474,33 @@
       <c r="EA13" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="EB13" s="12"/>
-      <c r="EC13" s="12"/>
-      <c r="ED13" s="12"/>
-      <c r="EE13" s="12"/>
-      <c r="EF13" s="12"/>
-      <c r="EG13" s="12"/>
-      <c r="EH13" s="12"/>
-      <c r="EI13" s="12"/>
-      <c r="EJ13" s="12"/>
+      <c r="EB13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EC13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="ED13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EE13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EF13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EG13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EH13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EI13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EJ13" s="12" t="s">
+        <v>200</v>
+      </c>
       <c r="EK13" s="12"/>
       <c r="EL13" s="12"/>
       <c r="EM13" s="12"/>
@@ -15158,6 +15525,15 @@
       <c r="FF13" s="12"/>
       <c r="FG13" s="12"/>
       <c r="FH13" s="12"/>
+      <c r="FI13" s="12"/>
+      <c r="FJ13" s="12"/>
+      <c r="FK13" s="12"/>
+      <c r="FL13" s="12"/>
+      <c r="FM13" s="12"/>
+      <c r="FN13" s="12"/>
+      <c r="FO13" s="12"/>
+      <c r="FP13" s="12"/>
+      <c r="FQ13" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
feat: re-import updated outdoor units for 大關U系列 and 經典V / 經典VA系列 from EQUIPMENT_Data.xlsx
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF31C842-F600-4979-982D-7C36245E9D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{030EB678-98A4-45CC-901F-1D6F245ED83C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6000" yWindow="0" windowWidth="17040" windowHeight="12240" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2854" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2980" uniqueCount="544">
   <si>
     <t>資料型態</t>
   </si>
@@ -1981,6 +1981,66 @@
   </si>
   <si>
     <t>990×940×320</t>
+  </si>
+  <si>
+    <t>大關U系列</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV22UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV28UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV36UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV41UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV50UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV60UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RXV71UVLT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>550×845×300</t>
+  </si>
+  <si>
+    <t>RHF20VAVLT</t>
+  </si>
+  <si>
+    <t>RHF25VAVLT</t>
+  </si>
+  <si>
+    <t>RHF30VAVLT</t>
+  </si>
+  <si>
+    <t>RHF40VVLT</t>
+  </si>
+  <si>
+    <t>RHF50VVLT</t>
+  </si>
+  <si>
+    <t>RHF60VVLT</t>
+  </si>
+  <si>
+    <t>RHF71VVLT</t>
+  </si>
+  <si>
+    <t>經典V系列</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -10061,17 +10121,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14518F8B-544C-42CB-BD27-24B9976359F4}">
-  <dimension ref="A1:FQ13"/>
+  <dimension ref="A1:GE13"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.44140625" customWidth="1"/>
     <col min="3" max="3" width="16.44140625" style="7" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="34.44140625" hidden="1" customWidth="1"/>
-    <col min="5" max="140" width="14.6640625" customWidth="1"/>
+    <col min="5" max="154" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -10085,7 +10145,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:173" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:187" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>41</v>
       </c>
@@ -10234,46 +10294,46 @@
         <v>34</v>
       </c>
       <c r="AX2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AY2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="AZ2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BA2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BB2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BC2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BD2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BE2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BF2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BG2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BH2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BI2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BJ2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BK2" s="5" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="BL2" s="5" t="s">
         <v>101</v>
@@ -10303,46 +10363,46 @@
         <v>101</v>
       </c>
       <c r="BU2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BV2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BW2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BX2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BY2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="BZ2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CA2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CB2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CC2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CD2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CE2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CF2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CG2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CH2" s="5" t="s">
-        <v>143</v>
+        <v>101</v>
       </c>
       <c r="CI2" s="5" t="s">
         <v>143</v>
@@ -10506,20 +10566,48 @@
       <c r="EJ2" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="EK2" s="5"/>
-      <c r="EL2" s="5"/>
-      <c r="EM2" s="5"/>
-      <c r="EN2" s="5"/>
-      <c r="EO2" s="5"/>
-      <c r="EP2" s="5"/>
-      <c r="EQ2" s="5"/>
-      <c r="ER2" s="5"/>
-      <c r="ES2" s="5"/>
-      <c r="ET2" s="5"/>
-      <c r="EU2" s="5"/>
-      <c r="EV2" s="5"/>
-      <c r="EW2" s="5"/>
-      <c r="EX2" s="5"/>
+      <c r="EK2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EL2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EM2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EN2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EO2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EP2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EQ2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="ER2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="ES2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="ET2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EU2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EV2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EW2" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="EX2" s="5" t="s">
+        <v>143</v>
+      </c>
       <c r="EY2" s="5"/>
       <c r="EZ2" s="5"/>
       <c r="FA2" s="5"/>
@@ -10539,8 +10627,22 @@
       <c r="FO2" s="5"/>
       <c r="FP2" s="5"/>
       <c r="FQ2" s="5"/>
+      <c r="FR2" s="5"/>
+      <c r="FS2" s="5"/>
+      <c r="FT2" s="5"/>
+      <c r="FU2" s="5"/>
+      <c r="FV2" s="5"/>
+      <c r="FW2" s="5"/>
+      <c r="FX2" s="5"/>
+      <c r="FY2" s="5"/>
+      <c r="FZ2" s="5"/>
+      <c r="GA2" s="5"/>
+      <c r="GB2" s="5"/>
+      <c r="GC2" s="5"/>
+      <c r="GD2" s="5"/>
+      <c r="GE2" s="5"/>
     </row>
-    <row r="3" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>44</v>
       </c>
@@ -10650,196 +10752,196 @@
         <v>77</v>
       </c>
       <c r="AK3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AL3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AM3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AN3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AO3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AP3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AQ3" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="AR3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AL3" s="5" t="s">
+      <c r="AS3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AM3" s="5" t="s">
+      <c r="AT3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AN3" s="5" t="s">
+      <c r="AU3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AO3" s="5" t="s">
+      <c r="AV3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AP3" s="5" t="s">
+      <c r="AW3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AQ3" s="5" t="s">
+      <c r="AX3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AR3" s="5" t="s">
+      <c r="AY3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="AZ3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="BA3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="BB3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="BC3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="BD3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="BE3" s="5" t="s">
+        <v>543</v>
+      </c>
+      <c r="BF3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AS3" s="5" t="s">
+      <c r="BG3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AT3" s="5" t="s">
+      <c r="BH3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AU3" s="5" t="s">
+      <c r="BI3" s="5" t="s">
         <v>489</v>
       </c>
-      <c r="AV3" s="5" t="s">
+      <c r="BJ3" s="5" t="s">
         <v>488</v>
       </c>
-      <c r="AW3" s="5" t="s">
+      <c r="BK3" s="5" t="s">
         <v>488</v>
       </c>
-      <c r="AX3" s="5" t="s">
+      <c r="BL3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="AY3" s="5" t="s">
+      <c r="BM3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="AZ3" s="5" t="s">
+      <c r="BN3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BA3" s="5" t="s">
+      <c r="BO3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BB3" s="5" t="s">
+      <c r="BP3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BC3" s="5" t="s">
+      <c r="BQ3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BD3" s="5" t="s">
+      <c r="BR3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BE3" s="5" t="s">
+      <c r="BS3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BF3" s="5" t="s">
+      <c r="BT3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BG3" s="5" t="s">
+      <c r="BU3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BH3" s="5" t="s">
+      <c r="BV3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BI3" s="5" t="s">
+      <c r="BW3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BJ3" s="5" t="s">
+      <c r="BX3" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="BK3" s="5" t="s">
+      <c r="BY3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BL3" s="5" t="s">
+      <c r="BZ3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BM3" s="5" t="s">
+      <c r="CA3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BN3" s="5" t="s">
+      <c r="CB3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BO3" s="5" t="s">
+      <c r="CC3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BP3" s="5" t="s">
+      <c r="CD3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BQ3" s="5" t="s">
+      <c r="CE3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BR3" s="5" t="s">
+      <c r="CF3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BS3" s="5" t="s">
+      <c r="CG3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BT3" s="5" t="s">
+      <c r="CH3" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="BU3" s="5" t="s">
+      <c r="CI3" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="BV3" s="5" t="s">
+      <c r="CJ3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BW3" s="5" t="s">
+      <c r="CK3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BX3" s="5" t="s">
+      <c r="CL3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BY3" s="5" t="s">
+      <c r="CM3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="BZ3" s="5" t="s">
+      <c r="CN3" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="CA3" s="5" t="s">
+      <c r="CO3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="CB3" s="5" t="s">
+      <c r="CP3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="CC3" s="5" t="s">
+      <c r="CQ3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="CD3" s="5" t="s">
+      <c r="CR3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="CE3" s="5" t="s">
+      <c r="CS3" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="CF3" s="5" t="s">
+      <c r="CT3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="CG3" s="5" t="s">
+      <c r="CU3" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="CH3" s="5" t="s">
+      <c r="CV3" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="CI3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CJ3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CK3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CL3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CM3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CN3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CO3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CP3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CQ3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CR3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CS3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CT3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CU3" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="CV3" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="CW3" s="5" t="s">
         <v>201</v>
@@ -10881,46 +10983,46 @@
         <v>201</v>
       </c>
       <c r="DJ3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DK3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DL3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DM3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DN3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DO3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DP3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DQ3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DR3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DS3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DT3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DU3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DV3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DW3" s="5" t="s">
-        <v>42</v>
+        <v>201</v>
       </c>
       <c r="DX3" s="5" t="s">
         <v>42</v>
@@ -10961,20 +11063,48 @@
       <c r="EJ3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="EK3" s="5"/>
-      <c r="EL3" s="5"/>
-      <c r="EM3" s="5"/>
-      <c r="EN3" s="5"/>
-      <c r="EO3" s="5"/>
-      <c r="EP3" s="5"/>
-      <c r="EQ3" s="5"/>
-      <c r="ER3" s="5"/>
-      <c r="ES3" s="5"/>
-      <c r="ET3" s="5"/>
-      <c r="EU3" s="5"/>
-      <c r="EV3" s="5"/>
-      <c r="EW3" s="5"/>
-      <c r="EX3" s="5"/>
+      <c r="EK3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EL3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EM3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EN3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EO3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EP3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EQ3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="ER3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="ES3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="ET3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EU3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EV3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EW3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="EX3" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="EY3" s="5"/>
       <c r="EZ3" s="5"/>
       <c r="FA3" s="5"/>
@@ -10994,8 +11124,22 @@
       <c r="FO3" s="5"/>
       <c r="FP3" s="5"/>
       <c r="FQ3" s="5"/>
+      <c r="FR3" s="5"/>
+      <c r="FS3" s="5"/>
+      <c r="FT3" s="5"/>
+      <c r="FU3" s="5"/>
+      <c r="FV3" s="5"/>
+      <c r="FW3" s="5"/>
+      <c r="FX3" s="5"/>
+      <c r="FY3" s="5"/>
+      <c r="FZ3" s="5"/>
+      <c r="GA3" s="5"/>
+      <c r="GB3" s="5"/>
+      <c r="GC3" s="5"/>
+      <c r="GD3" s="5"/>
+      <c r="GE3" s="5"/>
     </row>
-    <row r="4" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>52</v>
       </c>
@@ -11105,331 +11249,359 @@
         <v>94</v>
       </c>
       <c r="AK4" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="AL4" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="AM4" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="AN4" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="AO4" s="5" t="s">
+        <v>532</v>
+      </c>
+      <c r="AP4" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="AQ4" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="AR4" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="AL4" s="5" t="s">
+      <c r="AS4" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AM4" s="5" t="s">
+      <c r="AT4" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AN4" s="5" t="s">
+      <c r="AU4" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="AO4" s="5" t="s">
+      <c r="AV4" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AP4" s="5" t="s">
+      <c r="AW4" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="AQ4" s="5" t="s">
+      <c r="AX4" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="AR4" s="5" t="s">
+      <c r="AY4" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="AZ4" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="BA4" s="5" t="s">
+        <v>538</v>
+      </c>
+      <c r="BB4" s="5" t="s">
+        <v>539</v>
+      </c>
+      <c r="BC4" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="BD4" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="BE4" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="BF4" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AS4" s="5" t="s">
+      <c r="BG4" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="AT4" s="5" t="s">
+      <c r="BH4" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AU4" s="5" t="s">
+      <c r="BI4" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="AV4" s="5" t="s">
+      <c r="BJ4" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="AW4" s="5" t="s">
+      <c r="BK4" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="AX4" s="5" t="s">
+      <c r="BL4" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AY4" s="5" t="s">
+      <c r="BM4" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AZ4" s="5" t="s">
+      <c r="BN4" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="BA4" s="5" t="s">
+      <c r="BO4" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="BB4" s="5" t="s">
+      <c r="BP4" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="BC4" s="5" t="s">
+      <c r="BQ4" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="BD4" s="5" t="s">
+      <c r="BR4" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="BE4" s="5" t="s">
+      <c r="BS4" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="BF4" s="5" t="s">
+      <c r="BT4" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="BG4" s="5" t="s">
+      <c r="BU4" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="BH4" s="5" t="s">
+      <c r="BV4" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="BI4" s="5" t="s">
+      <c r="BW4" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="BJ4" s="5" t="s">
+      <c r="BX4" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="BK4" s="5" t="s">
+      <c r="BY4" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="BL4" s="5" t="s">
+      <c r="BZ4" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="BM4" s="5" t="s">
+      <c r="CA4" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="BN4" s="5" t="s">
+      <c r="CB4" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="BO4" s="5" t="s">
+      <c r="CC4" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="BP4" s="5" t="s">
+      <c r="CD4" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="BQ4" s="5" t="s">
+      <c r="CE4" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="BR4" s="5" t="s">
+      <c r="CF4" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="BS4" s="5" t="s">
+      <c r="CG4" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="BT4" s="5" t="s">
+      <c r="CH4" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="BU4" s="5" t="s">
+      <c r="CI4" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="BV4" s="5" t="s">
+      <c r="CJ4" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="BW4" s="5" t="s">
+      <c r="CK4" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="BX4" s="5" t="s">
+      <c r="CL4" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="BY4" s="5" t="s">
+      <c r="CM4" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="BZ4" s="5" t="s">
+      <c r="CN4" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="CA4" s="5" t="s">
+      <c r="CO4" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="CB4" s="5" t="s">
+      <c r="CP4" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="CC4" s="5" t="s">
+      <c r="CQ4" s="5" t="s">
         <v>505</v>
       </c>
-      <c r="CD4" s="5" t="s">
+      <c r="CR4" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="CE4" s="5" t="s">
+      <c r="CS4" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="CF4" s="5" t="s">
+      <c r="CT4" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="CG4" s="5" t="s">
+      <c r="CU4" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="CH4" s="5" t="s">
+      <c r="CV4" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="CI4" s="5" t="s">
+      <c r="CW4" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="CJ4" s="5" t="s">
+      <c r="CX4" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="CK4" s="5" t="s">
+      <c r="CY4" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="CL4" s="5" t="s">
+      <c r="CZ4" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="CM4" s="5" t="s">
+      <c r="DA4" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="CN4" s="5" t="s">
+      <c r="DB4" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="CO4" s="5" t="s">
+      <c r="DC4" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="CP4" s="5" t="s">
+      <c r="DD4" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="CQ4" s="5" t="s">
+      <c r="DE4" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="CR4" s="5" t="s">
+      <c r="DF4" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="CS4" s="5" t="s">
+      <c r="DG4" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="CT4" s="5" t="s">
+      <c r="DH4" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="CU4" s="5" t="s">
+      <c r="DI4" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="CV4" s="5" t="s">
+      <c r="DJ4" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="CW4" s="5" t="s">
+      <c r="DK4" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="CX4" s="5" t="s">
+      <c r="DL4" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="CY4" s="5" t="s">
+      <c r="DM4" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="CZ4" s="5" t="s">
+      <c r="DN4" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="DA4" s="5" t="s">
+      <c r="DO4" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="DB4" s="5" t="s">
+      <c r="DP4" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="DC4" s="5" t="s">
+      <c r="DQ4" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="DD4" s="5" t="s">
+      <c r="DR4" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="DE4" s="5" t="s">
+      <c r="DS4" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="DF4" s="5" t="s">
+      <c r="DT4" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="DG4" s="5" t="s">
+      <c r="DU4" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="DH4" s="5" t="s">
+      <c r="DV4" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="DI4" s="5" t="s">
+      <c r="DW4" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="DJ4" s="5" t="s">
+      <c r="DX4" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="DK4" s="5" t="s">
+      <c r="DY4" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="DL4" s="5" t="s">
+      <c r="DZ4" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="DM4" s="5" t="s">
+      <c r="EA4" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="DN4" s="5" t="s">
+      <c r="EB4" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="DO4" s="5" t="s">
+      <c r="EC4" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="DP4" s="5" t="s">
+      <c r="ED4" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="DQ4" s="5" t="s">
+      <c r="EE4" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="DR4" s="5" t="s">
+      <c r="EF4" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="DS4" s="5" t="s">
+      <c r="EG4" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="DT4" s="5" t="s">
+      <c r="EH4" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="DU4" s="5" t="s">
+      <c r="EI4" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="DV4" s="5" t="s">
+      <c r="EJ4" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="DW4" s="5" t="s">
+      <c r="EK4" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="DX4" s="5" t="s">
+      <c r="EL4" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="DY4" s="5" t="s">
+      <c r="EM4" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="DZ4" s="5" t="s">
+      <c r="EN4" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="EA4" s="5" t="s">
+      <c r="EO4" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="EB4" s="5" t="s">
+      <c r="EP4" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="EC4" s="5" t="s">
+      <c r="EQ4" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="ED4" s="5" t="s">
+      <c r="ER4" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="EE4" s="5" t="s">
+      <c r="ES4" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="EF4" s="5" t="s">
+      <c r="ET4" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="EG4" s="5" t="s">
+      <c r="EU4" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="EH4" s="5" t="s">
+      <c r="EV4" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="EI4" s="5" t="s">
+      <c r="EW4" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="EJ4" s="5" t="s">
+      <c r="EX4" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="EK4" s="5"/>
-      <c r="EL4" s="5"/>
-      <c r="EM4" s="5"/>
-      <c r="EN4" s="5"/>
-      <c r="EO4" s="5"/>
-      <c r="EP4" s="5"/>
-      <c r="EQ4" s="5"/>
-      <c r="ER4" s="5"/>
-      <c r="ES4" s="5"/>
-      <c r="ET4" s="5"/>
-      <c r="EU4" s="5"/>
-      <c r="EV4" s="5"/>
-      <c r="EW4" s="5"/>
-      <c r="EX4" s="5"/>
       <c r="EY4" s="5"/>
       <c r="EZ4" s="5"/>
       <c r="FA4" s="5"/>
@@ -11449,8 +11621,22 @@
       <c r="FO4" s="5"/>
       <c r="FP4" s="5"/>
       <c r="FQ4" s="5"/>
+      <c r="FR4" s="5"/>
+      <c r="FS4" s="5"/>
+      <c r="FT4" s="5"/>
+      <c r="FU4" s="5"/>
+      <c r="FV4" s="5"/>
+      <c r="FW4" s="5"/>
+      <c r="FX4" s="5"/>
+      <c r="FY4" s="5"/>
+      <c r="FZ4" s="5"/>
+      <c r="GA4" s="5"/>
+      <c r="GB4" s="5"/>
+      <c r="GC4" s="5"/>
+      <c r="GD4" s="5"/>
+      <c r="GE4" s="5"/>
     </row>
-    <row r="5" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>46</v>
       </c>
@@ -11563,10 +11749,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="AL5" s="5">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="AM5" s="5">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="AN5" s="5">
         <v>4.0999999999999996</v>
@@ -11581,127 +11767,127 @@
         <v>7.2</v>
       </c>
       <c r="AR5" s="5">
-        <v>5.6</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="AS5" s="5">
-        <v>7.2</v>
+        <v>2.5</v>
       </c>
       <c r="AT5" s="5">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="AU5" s="5">
-        <v>10.5</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="AV5" s="5">
         <v>5</v>
       </c>
       <c r="AW5" s="5">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="AX5" s="5">
         <v>7.2</v>
       </c>
       <c r="AY5" s="5">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AZ5" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="BA5" s="5">
+        <v>3</v>
+      </c>
+      <c r="BB5" s="5">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="BC5" s="5">
+        <v>5</v>
+      </c>
+      <c r="BD5" s="5">
+        <v>6</v>
+      </c>
+      <c r="BE5" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="BF5" s="5">
+        <v>5.6</v>
+      </c>
+      <c r="BG5" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="BH5" s="5">
+        <v>8.5</v>
+      </c>
+      <c r="BI5" s="5">
+        <v>10.5</v>
+      </c>
+      <c r="BJ5" s="5">
+        <v>5</v>
+      </c>
+      <c r="BK5" s="5">
+        <v>8.5</v>
+      </c>
+      <c r="BL5" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="BM5" s="5">
         <v>9.5</v>
       </c>
-      <c r="AZ5" s="5">
+      <c r="BN5" s="5">
         <v>7.2</v>
       </c>
-      <c r="BA5" s="5">
+      <c r="BO5" s="5">
         <v>7.2</v>
       </c>
-      <c r="BB5" s="5">
+      <c r="BP5" s="5">
         <v>10.1</v>
       </c>
-      <c r="BC5" s="5">
+      <c r="BQ5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BD5" s="5">
+      <c r="BR5" s="5">
         <v>14</v>
       </c>
-      <c r="BE5" s="5">
+      <c r="BS5" s="5">
         <v>10.1</v>
       </c>
-      <c r="BF5" s="5">
+      <c r="BT5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BG5" s="5">
+      <c r="BU5" s="5">
         <v>14</v>
       </c>
-      <c r="BH5" s="5">
+      <c r="BV5" s="5">
         <v>10.1</v>
       </c>
-      <c r="BI5" s="5">
+      <c r="BW5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BJ5" s="5">
+      <c r="BX5" s="5">
         <v>14</v>
       </c>
-      <c r="BK5" s="5">
+      <c r="BY5" s="5">
         <v>7.2</v>
       </c>
-      <c r="BL5" s="5">
+      <c r="BZ5" s="5">
         <v>10.4</v>
       </c>
-      <c r="BM5" s="5">
+      <c r="CA5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BN5" s="5">
+      <c r="CB5" s="5">
         <v>14</v>
       </c>
-      <c r="BO5" s="5">
+      <c r="CC5" s="5">
         <v>10.4</v>
       </c>
-      <c r="BP5" s="5">
+      <c r="CD5" s="5">
         <v>12.5</v>
       </c>
-      <c r="BQ5" s="5">
+      <c r="CE5" s="5">
         <v>14</v>
       </c>
-      <c r="BR5" s="5">
+      <c r="CF5" s="5">
         <v>10.4</v>
-      </c>
-      <c r="BS5" s="5">
-        <v>12.5</v>
-      </c>
-      <c r="BT5" s="5">
-        <v>14</v>
-      </c>
-      <c r="BU5" s="5">
-        <v>11.2</v>
-      </c>
-      <c r="BV5" s="5">
-        <v>12.5</v>
-      </c>
-      <c r="BW5" s="5">
-        <v>14</v>
-      </c>
-      <c r="BX5" s="5">
-        <v>16</v>
-      </c>
-      <c r="BY5" s="5">
-        <v>28</v>
-      </c>
-      <c r="BZ5" s="5">
-        <v>33.5</v>
-      </c>
-      <c r="CA5" s="5">
-        <v>22.4</v>
-      </c>
-      <c r="CB5" s="5">
-        <v>25</v>
-      </c>
-      <c r="CC5" s="5">
-        <v>15.5</v>
-      </c>
-      <c r="CD5" s="5">
-        <v>20</v>
-      </c>
-      <c r="CE5" s="5">
-        <v>24</v>
-      </c>
-      <c r="CF5" s="5">
-        <v>11.2</v>
       </c>
       <c r="CG5" s="5">
         <v>12.5</v>
@@ -11710,181 +11896,209 @@
         <v>14</v>
       </c>
       <c r="CI5" s="5">
+        <v>11.2</v>
+      </c>
+      <c r="CJ5" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="CK5" s="5">
+        <v>14</v>
+      </c>
+      <c r="CL5" s="5">
+        <v>16</v>
+      </c>
+      <c r="CM5" s="5">
+        <v>28</v>
+      </c>
+      <c r="CN5" s="5">
+        <v>33.5</v>
+      </c>
+      <c r="CO5" s="5">
         <v>22.4</v>
       </c>
-      <c r="CJ5" s="5">
+      <c r="CP5" s="5">
+        <v>25</v>
+      </c>
+      <c r="CQ5" s="5">
+        <v>15.5</v>
+      </c>
+      <c r="CR5" s="5">
+        <v>20</v>
+      </c>
+      <c r="CS5" s="5">
+        <v>24</v>
+      </c>
+      <c r="CT5" s="5">
+        <v>11.2</v>
+      </c>
+      <c r="CU5" s="5">
+        <v>12.5</v>
+      </c>
+      <c r="CV5" s="5">
+        <v>14</v>
+      </c>
+      <c r="CW5" s="5">
+        <v>22.4</v>
+      </c>
+      <c r="CX5" s="5">
         <v>28</v>
       </c>
-      <c r="CK5" s="5">
+      <c r="CY5" s="5">
         <v>33.5</v>
       </c>
-      <c r="CL5" s="5">
+      <c r="CZ5" s="5">
         <v>40</v>
       </c>
-      <c r="CM5" s="5">
+      <c r="DA5" s="5">
         <v>45</v>
       </c>
-      <c r="CN5" s="5">
+      <c r="DB5" s="5">
         <v>50</v>
       </c>
-      <c r="CO5" s="5">
+      <c r="DC5" s="5">
         <v>54</v>
       </c>
-      <c r="CP5" s="5">
+      <c r="DD5" s="5">
         <v>61.5</v>
       </c>
-      <c r="CQ5" s="5">
+      <c r="DE5" s="5">
         <v>67</v>
       </c>
-      <c r="CR5" s="5">
+      <c r="DF5" s="5">
         <v>73.5</v>
       </c>
-      <c r="CS5" s="5">
+      <c r="DG5" s="5">
         <v>78.5</v>
       </c>
-      <c r="CT5" s="5">
+      <c r="DH5" s="5">
         <v>85</v>
       </c>
-      <c r="CU5" s="5">
+      <c r="DI5" s="5">
         <v>90</v>
       </c>
-      <c r="CV5" s="5">
+      <c r="DJ5" s="5">
         <v>95</v>
       </c>
-      <c r="CW5" s="5">
+      <c r="DK5" s="5">
         <v>100</v>
       </c>
-      <c r="CX5" s="5">
+      <c r="DL5" s="5">
         <v>104</v>
       </c>
-      <c r="CY5" s="5">
+      <c r="DM5" s="5">
         <v>108</v>
       </c>
-      <c r="CZ5" s="5">
+      <c r="DN5" s="5">
         <v>117</v>
       </c>
-      <c r="DA5" s="5">
+      <c r="DO5" s="5">
         <v>121</v>
       </c>
-      <c r="DB5" s="5">
+      <c r="DP5" s="5">
         <v>130</v>
       </c>
-      <c r="DC5" s="5">
+      <c r="DQ5" s="5">
         <v>135</v>
       </c>
-      <c r="DD5" s="5">
+      <c r="DR5" s="5">
         <v>140</v>
       </c>
-      <c r="DE5" s="5">
+      <c r="DS5" s="5">
         <v>145</v>
       </c>
-      <c r="DF5" s="5">
+      <c r="DT5" s="5">
         <v>150</v>
       </c>
-      <c r="DG5" s="5">
+      <c r="DU5" s="5">
         <v>154</v>
       </c>
-      <c r="DH5" s="5">
+      <c r="DV5" s="5">
         <v>158</v>
       </c>
-      <c r="DI5" s="5">
+      <c r="DW5" s="5">
         <v>162</v>
       </c>
-      <c r="DJ5" s="5">
+      <c r="DX5" s="5">
         <v>22.4</v>
       </c>
-      <c r="DK5" s="5">
+      <c r="DY5" s="5">
         <v>28</v>
       </c>
-      <c r="DL5" s="5">
+      <c r="DZ5" s="5">
         <v>33.5</v>
       </c>
-      <c r="DM5" s="5">
+      <c r="EA5" s="5">
         <v>40</v>
       </c>
-      <c r="DN5" s="5">
+      <c r="EB5" s="5">
         <v>45</v>
       </c>
-      <c r="DO5" s="5">
+      <c r="EC5" s="5">
         <v>50</v>
       </c>
-      <c r="DP5" s="5">
+      <c r="ED5" s="5">
         <v>54</v>
       </c>
-      <c r="DQ5" s="5">
+      <c r="EE5" s="5">
         <v>61.5</v>
       </c>
-      <c r="DR5" s="5">
+      <c r="EF5" s="5">
         <v>67</v>
       </c>
-      <c r="DS5" s="5">
+      <c r="EG5" s="5">
         <v>73.5</v>
       </c>
-      <c r="DT5" s="5">
+      <c r="EH5" s="5">
         <v>78.5</v>
       </c>
-      <c r="DU5" s="5">
+      <c r="EI5" s="5">
         <v>85</v>
       </c>
-      <c r="DV5" s="5">
+      <c r="EJ5" s="5">
         <v>90</v>
       </c>
-      <c r="DW5" s="5">
+      <c r="EK5" s="5">
         <v>95</v>
       </c>
-      <c r="DX5" s="5">
+      <c r="EL5" s="5">
         <v>100</v>
       </c>
-      <c r="DY5" s="5">
+      <c r="EM5" s="5">
         <v>104</v>
       </c>
-      <c r="DZ5" s="5">
+      <c r="EN5" s="5">
         <v>108</v>
       </c>
-      <c r="EA5" s="5">
+      <c r="EO5" s="5">
         <v>117</v>
       </c>
-      <c r="EB5" s="5">
+      <c r="EP5" s="5">
         <v>121</v>
       </c>
-      <c r="EC5" s="5">
+      <c r="EQ5" s="5">
         <v>130</v>
       </c>
-      <c r="ED5" s="5">
+      <c r="ER5" s="5">
         <v>135</v>
       </c>
-      <c r="EE5" s="5">
+      <c r="ES5" s="5">
         <v>140</v>
       </c>
-      <c r="EF5" s="5">
+      <c r="ET5" s="5">
         <v>145</v>
       </c>
-      <c r="EG5" s="5">
+      <c r="EU5" s="5">
         <v>150</v>
       </c>
-      <c r="EH5" s="5">
+      <c r="EV5" s="5">
         <v>154</v>
       </c>
-      <c r="EI5" s="5">
+      <c r="EW5" s="5">
         <v>158</v>
       </c>
-      <c r="EJ5" s="5">
+      <c r="EX5" s="5">
         <v>162</v>
       </c>
-      <c r="EK5" s="5"/>
-      <c r="EL5" s="5"/>
-      <c r="EM5" s="5"/>
-      <c r="EN5" s="5"/>
-      <c r="EO5" s="5"/>
-      <c r="EP5" s="5"/>
-      <c r="EQ5" s="5"/>
-      <c r="ER5" s="5"/>
-      <c r="ES5" s="5"/>
-      <c r="ET5" s="5"/>
-      <c r="EU5" s="5"/>
-      <c r="EV5" s="5"/>
-      <c r="EW5" s="5"/>
-      <c r="EX5" s="5"/>
       <c r="EY5" s="5"/>
       <c r="EZ5" s="5"/>
       <c r="FA5" s="5"/>
@@ -11904,8 +12118,22 @@
       <c r="FO5" s="5"/>
       <c r="FP5" s="5"/>
       <c r="FQ5" s="5"/>
+      <c r="FR5" s="5"/>
+      <c r="FS5" s="5"/>
+      <c r="FT5" s="5"/>
+      <c r="FU5" s="5"/>
+      <c r="FV5" s="5"/>
+      <c r="FW5" s="5"/>
+      <c r="FX5" s="5"/>
+      <c r="FY5" s="5"/>
+      <c r="FZ5" s="5"/>
+      <c r="GA5" s="5"/>
+      <c r="GB5" s="5"/>
+      <c r="GC5" s="5"/>
+      <c r="GD5" s="5"/>
+      <c r="GE5" s="5"/>
     </row>
-    <row r="6" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>45</v>
       </c>
@@ -12122,224 +12350,252 @@
       <c r="BT6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="BU6" s="5">
+      <c r="BU6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BV6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BW6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BX6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BY6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="BZ6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CA6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CB6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CC6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CD6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CE6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CF6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CG6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CH6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="CI6" s="5">
         <v>100</v>
       </c>
-      <c r="BV6" s="5">
+      <c r="CJ6" s="5">
         <v>112.5</v>
       </c>
-      <c r="BW6" s="5">
+      <c r="CK6" s="5">
         <v>125</v>
       </c>
-      <c r="BX6" s="5">
+      <c r="CL6" s="5">
         <v>150</v>
       </c>
-      <c r="BY6" s="5">
+      <c r="CM6" s="5">
         <v>250</v>
       </c>
-      <c r="BZ6" s="5">
+      <c r="CN6" s="5">
         <v>300</v>
       </c>
-      <c r="CA6" s="5">
+      <c r="CO6" s="5">
         <v>200</v>
       </c>
-      <c r="CB6" s="5">
+      <c r="CP6" s="5">
         <v>223</v>
       </c>
-      <c r="CC6" s="5">
+      <c r="CQ6" s="5">
         <v>140</v>
       </c>
-      <c r="CD6" s="5">
+      <c r="CR6" s="5">
         <v>180</v>
       </c>
-      <c r="CE6" s="5">
+      <c r="CS6" s="5">
         <v>215</v>
       </c>
-      <c r="CF6" s="5">
+      <c r="CT6" s="5">
         <v>100</v>
       </c>
-      <c r="CG6" s="5">
+      <c r="CU6" s="5">
         <v>112.5</v>
       </c>
-      <c r="CH6" s="5">
+      <c r="CV6" s="5">
         <v>125</v>
       </c>
-      <c r="CI6" s="5">
+      <c r="CW6" s="5">
         <v>200</v>
       </c>
-      <c r="CJ6" s="5">
+      <c r="CX6" s="5">
         <v>250</v>
       </c>
-      <c r="CK6" s="5">
+      <c r="CY6" s="5">
         <v>300</v>
       </c>
-      <c r="CL6" s="5">
+      <c r="CZ6" s="5">
         <v>350</v>
       </c>
-      <c r="CM6" s="5">
+      <c r="DA6" s="5">
         <v>400</v>
       </c>
-      <c r="CN6" s="5">
+      <c r="DB6" s="5">
         <v>450</v>
       </c>
-      <c r="CO6" s="5">
+      <c r="DC6" s="5">
         <v>500</v>
       </c>
-      <c r="CP6" s="5">
+      <c r="DD6" s="5">
         <v>550</v>
       </c>
-      <c r="CQ6" s="5">
+      <c r="DE6" s="5">
         <v>600</v>
       </c>
-      <c r="CR6" s="5">
+      <c r="DF6" s="5">
         <v>650</v>
       </c>
-      <c r="CS6" s="5">
+      <c r="DG6" s="5">
         <v>700</v>
       </c>
-      <c r="CT6" s="5">
+      <c r="DH6" s="5">
         <v>750</v>
       </c>
-      <c r="CU6" s="5">
+      <c r="DI6" s="5">
         <v>800</v>
       </c>
-      <c r="CV6" s="5">
+      <c r="DJ6" s="5">
         <v>850</v>
       </c>
-      <c r="CW6" s="5">
+      <c r="DK6" s="5">
         <v>900</v>
       </c>
-      <c r="CX6" s="5">
+      <c r="DL6" s="5">
         <v>950</v>
       </c>
-      <c r="CY6" s="5">
+      <c r="DM6" s="5">
         <v>1000</v>
       </c>
-      <c r="CZ6" s="5">
+      <c r="DN6" s="5">
         <v>1050</v>
       </c>
-      <c r="DA6" s="5">
+      <c r="DO6" s="5">
         <v>1100</v>
       </c>
-      <c r="DB6" s="5">
+      <c r="DP6" s="5">
         <v>1150</v>
       </c>
-      <c r="DC6" s="5">
+      <c r="DQ6" s="5">
         <v>1200</v>
       </c>
-      <c r="DD6" s="5">
+      <c r="DR6" s="5">
         <v>1250</v>
       </c>
-      <c r="DE6" s="5">
+      <c r="DS6" s="5">
         <v>1300</v>
       </c>
-      <c r="DF6" s="5">
+      <c r="DT6" s="5">
         <v>1350</v>
       </c>
-      <c r="DG6" s="5">
+      <c r="DU6" s="5">
         <v>1400</v>
       </c>
-      <c r="DH6" s="5">
+      <c r="DV6" s="5">
         <v>1450</v>
       </c>
-      <c r="DI6" s="5">
+      <c r="DW6" s="5">
         <v>1500</v>
       </c>
-      <c r="DJ6" s="5">
+      <c r="DX6" s="5">
         <v>200</v>
       </c>
-      <c r="DK6" s="5">
+      <c r="DY6" s="5">
         <v>250</v>
       </c>
-      <c r="DL6" s="5">
+      <c r="DZ6" s="5">
         <v>300</v>
       </c>
-      <c r="DM6" s="5">
+      <c r="EA6" s="5">
         <v>350</v>
       </c>
-      <c r="DN6" s="5">
+      <c r="EB6" s="5">
         <v>400</v>
       </c>
-      <c r="DO6" s="5">
+      <c r="EC6" s="5">
         <v>450</v>
       </c>
-      <c r="DP6" s="5">
+      <c r="ED6" s="5">
         <v>500</v>
       </c>
-      <c r="DQ6" s="5">
+      <c r="EE6" s="5">
         <v>550</v>
       </c>
-      <c r="DR6" s="5">
+      <c r="EF6" s="5">
         <v>600</v>
       </c>
-      <c r="DS6" s="5">
+      <c r="EG6" s="5">
         <v>650</v>
       </c>
-      <c r="DT6" s="5">
+      <c r="EH6" s="5">
         <v>700</v>
       </c>
-      <c r="DU6" s="5">
+      <c r="EI6" s="5">
         <v>750</v>
       </c>
-      <c r="DV6" s="5">
+      <c r="EJ6" s="5">
         <v>800</v>
       </c>
-      <c r="DW6" s="5">
+      <c r="EK6" s="5">
         <v>850</v>
       </c>
-      <c r="DX6" s="5">
+      <c r="EL6" s="5">
         <v>900</v>
       </c>
-      <c r="DY6" s="5">
+      <c r="EM6" s="5">
         <v>950</v>
       </c>
-      <c r="DZ6" s="5">
+      <c r="EN6" s="5">
         <v>1000</v>
       </c>
-      <c r="EA6" s="5">
+      <c r="EO6" s="5">
         <v>1050</v>
       </c>
-      <c r="EB6" s="5">
+      <c r="EP6" s="5">
         <v>1100</v>
       </c>
-      <c r="EC6" s="5">
+      <c r="EQ6" s="5">
         <v>1150</v>
       </c>
-      <c r="ED6" s="5">
+      <c r="ER6" s="5">
         <v>1200</v>
       </c>
-      <c r="EE6" s="5">
+      <c r="ES6" s="5">
         <v>1250</v>
       </c>
-      <c r="EF6" s="5">
+      <c r="ET6" s="5">
         <v>1300</v>
       </c>
-      <c r="EG6" s="5">
+      <c r="EU6" s="5">
         <v>1350</v>
       </c>
-      <c r="EH6" s="5">
+      <c r="EV6" s="5">
         <v>1400</v>
       </c>
-      <c r="EI6" s="5">
+      <c r="EW6" s="5">
         <v>1450</v>
       </c>
-      <c r="EJ6" s="5">
+      <c r="EX6" s="5">
         <v>1500</v>
       </c>
-      <c r="EK6" s="5"/>
-      <c r="EL6" s="5"/>
-      <c r="EM6" s="5"/>
-      <c r="EN6" s="5"/>
-      <c r="EO6" s="5"/>
-      <c r="EP6" s="5"/>
-      <c r="EQ6" s="5"/>
-      <c r="ER6" s="5"/>
-      <c r="ES6" s="5"/>
-      <c r="ET6" s="5"/>
-      <c r="EU6" s="5"/>
-      <c r="EV6" s="5"/>
-      <c r="EW6" s="5"/>
-      <c r="EX6" s="5"/>
       <c r="EY6" s="5"/>
       <c r="EZ6" s="5"/>
       <c r="FA6" s="5"/>
@@ -12359,8 +12615,22 @@
       <c r="FO6" s="5"/>
       <c r="FP6" s="5"/>
       <c r="FQ6" s="5"/>
+      <c r="FR6" s="5"/>
+      <c r="FS6" s="5"/>
+      <c r="FT6" s="5"/>
+      <c r="FU6" s="5"/>
+      <c r="FV6" s="5"/>
+      <c r="FW6" s="5"/>
+      <c r="FX6" s="5"/>
+      <c r="FY6" s="5"/>
+      <c r="FZ6" s="5"/>
+      <c r="GA6" s="5"/>
+      <c r="GB6" s="5"/>
+      <c r="GC6" s="5"/>
+      <c r="GD6" s="5"/>
+      <c r="GE6" s="5"/>
     </row>
-    <row r="7" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>48</v>
       </c>
@@ -12530,106 +12800,106 @@
         <v>9</v>
       </c>
       <c r="BE7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BF7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BG7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BH7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BI7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BJ7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BK7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BL7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BM7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BN7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BO7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BP7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BQ7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BR7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="BS7" s="5" t="s">
         <v>507</v>
       </c>
-      <c r="BF7" s="5" t="s">
+      <c r="BT7" s="5" t="s">
         <v>507</v>
       </c>
-      <c r="BG7" s="5" t="s">
+      <c r="BU7" s="5" t="s">
         <v>507</v>
       </c>
-      <c r="BH7" s="5" t="s">
+      <c r="BV7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="BI7" s="5" t="s">
+      <c r="BW7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="BJ7" s="5" t="s">
+      <c r="BX7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="BK7" s="5" t="s">
+      <c r="BY7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BL7" s="5" t="s">
+      <c r="BZ7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BM7" s="5" t="s">
+      <c r="CA7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BN7" s="5" t="s">
+      <c r="CB7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BO7" s="5" t="s">
+      <c r="CC7" s="5" t="s">
         <v>507</v>
       </c>
-      <c r="BP7" s="5" t="s">
+      <c r="CD7" s="5" t="s">
         <v>507</v>
       </c>
-      <c r="BQ7" s="5" t="s">
+      <c r="CE7" s="5" t="s">
         <v>507</v>
       </c>
-      <c r="BR7" s="5" t="s">
+      <c r="CF7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="BS7" s="5" t="s">
+      <c r="CG7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="BT7" s="5" t="s">
+      <c r="CH7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="BU7" s="5" t="s">
+      <c r="CI7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BV7" s="5" t="s">
+      <c r="CJ7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BW7" s="5" t="s">
+      <c r="CK7" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="BX7" s="5" t="s">
+      <c r="CL7" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="BY7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="BZ7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="CA7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="CB7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="CC7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="CD7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="CE7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="CF7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="CG7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="CH7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="CI7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="CJ7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="CK7" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="CL7" s="5" t="s">
-        <v>506</v>
       </c>
       <c r="CM7" s="5" t="s">
         <v>506</v>
@@ -12638,13 +12908,13 @@
         <v>506</v>
       </c>
       <c r="CO7" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="CP7" s="5" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="CQ7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CR7" s="5" t="s">
         <v>506</v>
@@ -12653,13 +12923,13 @@
         <v>506</v>
       </c>
       <c r="CT7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CU7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CV7" s="5" t="s">
-        <v>506</v>
+        <v>137</v>
       </c>
       <c r="CW7" s="5" t="s">
         <v>506</v>
@@ -12781,20 +13051,48 @@
       <c r="EJ7" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="EK7" s="5"/>
-      <c r="EL7" s="5"/>
-      <c r="EM7" s="5"/>
-      <c r="EN7" s="5"/>
-      <c r="EO7" s="5"/>
-      <c r="EP7" s="5"/>
-      <c r="EQ7" s="5"/>
-      <c r="ER7" s="5"/>
-      <c r="ES7" s="5"/>
-      <c r="ET7" s="5"/>
-      <c r="EU7" s="5"/>
-      <c r="EV7" s="5"/>
-      <c r="EW7" s="5"/>
-      <c r="EX7" s="5"/>
+      <c r="EK7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EL7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EM7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EN7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EO7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EP7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EQ7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="ER7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="ES7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="ET7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EU7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EV7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EW7" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="EX7" s="5" t="s">
+        <v>506</v>
+      </c>
       <c r="EY7" s="5"/>
       <c r="EZ7" s="5"/>
       <c r="FA7" s="5"/>
@@ -12814,8 +13112,22 @@
       <c r="FO7" s="5"/>
       <c r="FP7" s="5"/>
       <c r="FQ7" s="5"/>
+      <c r="FR7" s="5"/>
+      <c r="FS7" s="5"/>
+      <c r="FT7" s="5"/>
+      <c r="FU7" s="5"/>
+      <c r="FV7" s="5"/>
+      <c r="FW7" s="5"/>
+      <c r="FX7" s="5"/>
+      <c r="FY7" s="5"/>
+      <c r="FZ7" s="5"/>
+      <c r="GA7" s="5"/>
+      <c r="GB7" s="5"/>
+      <c r="GC7" s="5"/>
+      <c r="GD7" s="5"/>
+      <c r="GE7" s="5"/>
     </row>
-    <row r="8" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>47</v>
       </c>
@@ -12925,331 +13237,359 @@
         <v>2.15</v>
       </c>
       <c r="AK8" s="5">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="AL8" s="5">
+        <v>0.62</v>
+      </c>
+      <c r="AM8" s="5">
+        <v>0.78500000000000003</v>
+      </c>
+      <c r="AN8" s="5">
+        <v>0.94</v>
+      </c>
+      <c r="AO8" s="5">
+        <v>1.34</v>
+      </c>
+      <c r="AP8" s="5">
+        <v>1.67</v>
+      </c>
+      <c r="AQ8" s="5">
+        <v>2.1800000000000002</v>
+      </c>
+      <c r="AR8" s="5">
         <v>0.46500000000000002</v>
       </c>
-      <c r="AL8" s="5">
+      <c r="AS8" s="5">
         <v>0.55000000000000004</v>
       </c>
-      <c r="AM8" s="5">
+      <c r="AT8" s="5">
         <v>0.68400000000000005</v>
       </c>
-      <c r="AN8" s="5">
+      <c r="AU8" s="5">
         <v>1</v>
       </c>
-      <c r="AO8" s="5">
+      <c r="AV8" s="5">
         <v>1.3149999999999999</v>
       </c>
-      <c r="AP8" s="5">
+      <c r="AW8" s="5">
         <v>1.72</v>
       </c>
-      <c r="AQ8" s="5">
+      <c r="AX8" s="5">
         <v>2.15</v>
       </c>
-      <c r="AR8" s="5">
+      <c r="AY8" s="5">
+        <v>0.46500000000000002</v>
+      </c>
+      <c r="AZ8" s="5">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="BA8" s="5">
+        <v>0.7</v>
+      </c>
+      <c r="BB8" s="5">
+        <v>0.95199999999999996</v>
+      </c>
+      <c r="BC8" s="5">
+        <v>1.3149999999999999</v>
+      </c>
+      <c r="BD8" s="5">
+        <v>1.78</v>
+      </c>
+      <c r="BE8" s="5">
+        <v>2.23</v>
+      </c>
+      <c r="BF8" s="5">
         <v>1.375</v>
       </c>
-      <c r="AS8" s="5">
+      <c r="BG8" s="5">
         <v>1.82</v>
       </c>
-      <c r="AT8" s="5">
+      <c r="BH8" s="5">
         <v>2.27</v>
       </c>
-      <c r="AU8" s="5">
+      <c r="BI8" s="5">
         <v>2.71</v>
       </c>
-      <c r="AV8" s="5">
+      <c r="BJ8" s="5">
         <v>1.52</v>
       </c>
-      <c r="AW8" s="5">
+      <c r="BK8" s="5">
         <v>2.67</v>
       </c>
-      <c r="AX8" s="5">
+      <c r="BL8" s="5">
         <v>2.23</v>
       </c>
-      <c r="AY8" s="5">
+      <c r="BM8" s="5">
         <v>2.8</v>
       </c>
-      <c r="AZ8" s="5">
+      <c r="BN8" s="5">
         <v>1.9</v>
       </c>
-      <c r="BA8" s="5">
+      <c r="BO8" s="5">
         <v>1.9</v>
       </c>
-      <c r="BB8" s="5">
+      <c r="BP8" s="5">
         <v>2.88</v>
       </c>
-      <c r="BC8" s="5">
+      <c r="BQ8" s="5">
         <v>4</v>
       </c>
-      <c r="BD8" s="5">
+      <c r="BR8" s="5">
         <v>4.8</v>
       </c>
-      <c r="BE8" s="5">
+      <c r="BS8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BF8" s="5">
+      <c r="BT8" s="5">
         <v>4</v>
       </c>
-      <c r="BG8" s="5">
+      <c r="BU8" s="5">
         <v>4.8</v>
       </c>
-      <c r="BH8" s="5">
+      <c r="BV8" s="5">
         <v>2.88</v>
       </c>
-      <c r="BI8" s="5">
+      <c r="BW8" s="5">
         <v>4</v>
       </c>
-      <c r="BJ8" s="5">
+      <c r="BX8" s="5">
         <v>4.8</v>
       </c>
-      <c r="BK8" s="5">
+      <c r="BY8" s="5">
         <v>1.88</v>
       </c>
-      <c r="BL8" s="5">
+      <c r="BZ8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BM8" s="5">
+      <c r="CA8" s="5">
         <v>3.75</v>
       </c>
-      <c r="BN8" s="5">
+      <c r="CB8" s="5">
         <v>4.7</v>
       </c>
-      <c r="BO8" s="5">
+      <c r="CC8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BP8" s="5">
+      <c r="CD8" s="5">
         <v>3.75</v>
       </c>
-      <c r="BQ8" s="5">
+      <c r="CE8" s="5">
         <v>4.7</v>
       </c>
-      <c r="BR8" s="5">
+      <c r="CF8" s="5">
         <v>2.86</v>
       </c>
-      <c r="BS8" s="5">
+      <c r="CG8" s="5">
         <v>3.75</v>
       </c>
-      <c r="BT8" s="5">
+      <c r="CH8" s="5">
         <v>4.7</v>
       </c>
-      <c r="BU8" s="5">
+      <c r="CI8" s="5">
         <v>2.25</v>
       </c>
-      <c r="BV8" s="5">
+      <c r="CJ8" s="5">
         <v>2.66</v>
       </c>
-      <c r="BW8" s="5">
+      <c r="CK8" s="5">
         <v>3.08</v>
       </c>
-      <c r="BX8" s="5">
+      <c r="CL8" s="5">
         <v>3.97</v>
       </c>
-      <c r="BY8" s="5">
+      <c r="CM8" s="5">
         <v>6.72</v>
       </c>
-      <c r="BZ8" s="5">
+      <c r="CN8" s="5">
         <v>8.93</v>
       </c>
-      <c r="CA8" s="5">
+      <c r="CO8" s="5">
         <v>6.3</v>
       </c>
-      <c r="CB8" s="5">
+      <c r="CP8" s="5">
         <v>7.8</v>
       </c>
-      <c r="CC8" s="5">
+      <c r="CQ8" s="5">
         <v>4.3899999999999997</v>
       </c>
-      <c r="CD8" s="5">
+      <c r="CR8" s="5">
         <v>5.91</v>
       </c>
-      <c r="CE8" s="5">
+      <c r="CS8" s="5">
         <v>7.51</v>
       </c>
-      <c r="CF8" s="5">
+      <c r="CT8" s="5">
         <v>2.81</v>
       </c>
-      <c r="CG8" s="5">
+      <c r="CU8" s="5">
         <v>3.28</v>
       </c>
-      <c r="CH8" s="5">
+      <c r="CV8" s="5">
         <v>4.01</v>
       </c>
-      <c r="CI8" s="5">
+      <c r="CW8" s="5">
         <v>5.32</v>
       </c>
-      <c r="CJ8" s="5">
+      <c r="CX8" s="5">
         <v>7.26</v>
       </c>
-      <c r="CK8" s="5">
+      <c r="CY8" s="5">
         <v>9.26</v>
       </c>
-      <c r="CL8" s="5">
+      <c r="CZ8" s="5">
         <v>11.35</v>
       </c>
-      <c r="CM8" s="5">
+      <c r="DA8" s="5">
         <v>12.15</v>
       </c>
-      <c r="CN8" s="5">
+      <c r="DB8" s="5">
         <v>14.82</v>
       </c>
-      <c r="CO8" s="5">
+      <c r="DC8" s="5">
         <v>16.239999999999998</v>
       </c>
-      <c r="CP8" s="5">
+      <c r="DD8" s="5">
         <v>16.52</v>
       </c>
-      <c r="CQ8" s="5">
+      <c r="DE8" s="5">
         <v>18.52</v>
       </c>
-      <c r="CR8" s="5">
+      <c r="DF8" s="5">
         <v>20.61</v>
       </c>
-      <c r="CS8" s="5">
+      <c r="DG8" s="5">
         <v>21.41</v>
       </c>
-      <c r="CT8" s="5">
+      <c r="DH8" s="5">
         <v>23.5</v>
       </c>
-      <c r="CU8" s="5">
+      <c r="DI8" s="5">
         <v>26.17</v>
       </c>
-      <c r="CV8" s="5">
+      <c r="DJ8" s="5">
         <v>26.97</v>
       </c>
-      <c r="CW8" s="5">
+      <c r="DK8" s="5">
         <v>29.64</v>
       </c>
-      <c r="CX8" s="5">
+      <c r="DL8" s="5">
         <v>31.06</v>
       </c>
-      <c r="CY8" s="5">
+      <c r="DM8" s="5">
         <v>32.479999999999997</v>
       </c>
-      <c r="CZ8" s="5">
+      <c r="DN8" s="5">
         <v>33.340000000000003</v>
       </c>
-      <c r="DA8" s="5">
+      <c r="DO8" s="5">
         <v>34.76</v>
       </c>
-      <c r="DB8" s="5">
+      <c r="DP8" s="5">
         <v>37.520000000000003</v>
       </c>
-      <c r="DC8" s="5">
+      <c r="DQ8" s="5">
         <v>38.32</v>
       </c>
-      <c r="DD8" s="5">
+      <c r="DR8" s="5">
         <v>40.99</v>
       </c>
-      <c r="DE8" s="5">
+      <c r="DS8" s="5">
         <v>41.79</v>
       </c>
-      <c r="DF8" s="5">
+      <c r="DT8" s="5">
         <v>44.46</v>
       </c>
-      <c r="DG8" s="5">
+      <c r="DU8" s="5">
         <v>45.88</v>
       </c>
-      <c r="DH8" s="5">
+      <c r="DV8" s="5">
         <v>47.3</v>
       </c>
-      <c r="DI8" s="5">
+      <c r="DW8" s="5">
         <v>48.72</v>
       </c>
-      <c r="DJ8" s="5">
+      <c r="DX8" s="5">
         <v>5.65</v>
       </c>
-      <c r="DK8" s="5">
+      <c r="DY8" s="5">
         <v>7.09</v>
       </c>
-      <c r="DL8" s="5">
+      <c r="DZ8" s="5">
         <v>9.9700000000000006</v>
       </c>
-      <c r="DM8" s="5">
+      <c r="EA8" s="5">
         <v>12.08</v>
       </c>
-      <c r="DN8" s="5">
+      <c r="EB8" s="5">
         <v>13.92</v>
       </c>
-      <c r="DO8" s="5">
+      <c r="EC8" s="5">
         <v>15.07</v>
       </c>
-      <c r="DP8" s="5">
+      <c r="ED8" s="5">
         <v>16.5</v>
       </c>
-      <c r="DQ8" s="5">
+      <c r="EE8" s="5">
         <v>17.059999999999999</v>
       </c>
-      <c r="DR8" s="5">
+      <c r="EF8" s="5">
         <v>19.940000000000001</v>
       </c>
-      <c r="DS8" s="5">
+      <c r="EG8" s="5">
         <v>22.05</v>
       </c>
-      <c r="DT8" s="5">
+      <c r="EH8" s="5">
         <v>23.89</v>
       </c>
-      <c r="DU8" s="5">
+      <c r="EI8" s="5">
         <v>26</v>
       </c>
-      <c r="DV8" s="5">
+      <c r="EJ8" s="5">
         <v>27.15</v>
       </c>
-      <c r="DW8" s="5">
+      <c r="EK8" s="5">
         <v>28.99</v>
       </c>
-      <c r="DX8" s="5">
+      <c r="EL8" s="5">
         <v>30.14</v>
       </c>
-      <c r="DY8" s="5">
+      <c r="EM8" s="5">
         <v>31.57</v>
       </c>
-      <c r="DZ8" s="5">
+      <c r="EN8" s="5">
         <v>33</v>
       </c>
-      <c r="EA8" s="5">
+      <c r="EO8" s="5">
         <v>35.01</v>
       </c>
-      <c r="EB8" s="5">
+      <c r="EP8" s="5">
         <v>36.44</v>
       </c>
-      <c r="EC8" s="5">
+      <c r="EQ8" s="5">
         <v>39.229999999999997</v>
       </c>
-      <c r="ED8" s="5">
+      <c r="ER8" s="5">
         <v>41.07</v>
       </c>
-      <c r="EE8" s="5">
+      <c r="ES8" s="5">
         <v>42.22</v>
       </c>
-      <c r="EF8" s="5">
+      <c r="ET8" s="5">
         <v>44.06</v>
       </c>
-      <c r="EG8" s="5">
+      <c r="EU8" s="5">
         <v>45.21</v>
       </c>
-      <c r="EH8" s="5">
+      <c r="EV8" s="5">
         <v>46.64</v>
       </c>
-      <c r="EI8" s="5">
+      <c r="EW8" s="5">
         <v>48.07</v>
       </c>
-      <c r="EJ8" s="5">
+      <c r="EX8" s="5">
         <v>49.5</v>
       </c>
-      <c r="EK8" s="5"/>
-      <c r="EL8" s="5"/>
-      <c r="EM8" s="5"/>
-      <c r="EN8" s="5"/>
-      <c r="EO8" s="5"/>
-      <c r="EP8" s="5"/>
-      <c r="EQ8" s="5"/>
-      <c r="ER8" s="5"/>
-      <c r="ES8" s="5"/>
-      <c r="ET8" s="5"/>
-      <c r="EU8" s="5"/>
-      <c r="EV8" s="5"/>
-      <c r="EW8" s="5"/>
-      <c r="EX8" s="5"/>
       <c r="EY8" s="5"/>
       <c r="EZ8" s="5"/>
       <c r="FA8" s="5"/>
@@ -13269,8 +13609,22 @@
       <c r="FO8" s="5"/>
       <c r="FP8" s="5"/>
       <c r="FQ8" s="5"/>
+      <c r="FR8" s="5"/>
+      <c r="FS8" s="5"/>
+      <c r="FT8" s="5"/>
+      <c r="FU8" s="5"/>
+      <c r="FV8" s="5"/>
+      <c r="FW8" s="5"/>
+      <c r="FX8" s="5"/>
+      <c r="FY8" s="5"/>
+      <c r="FZ8" s="5"/>
+      <c r="GA8" s="5"/>
+      <c r="GB8" s="5"/>
+      <c r="GC8" s="5"/>
+      <c r="GD8" s="5"/>
+      <c r="GE8" s="5"/>
     </row>
-    <row r="9" spans="1:173" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:187" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>50</v>
       </c>
@@ -13380,331 +13734,359 @@
         <v>11</v>
       </c>
       <c r="AK9" s="5">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AL9" s="5">
+        <v>3.1</v>
+      </c>
+      <c r="AM9" s="5">
+        <v>3.8</v>
+      </c>
+      <c r="AN9" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="AO9" s="5">
+        <v>6.3</v>
+      </c>
+      <c r="AP9" s="5">
+        <v>7.8</v>
+      </c>
+      <c r="AQ9" s="5">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="AR9" s="5">
         <v>7.3</v>
       </c>
-      <c r="AL9" s="5" t="s">
+      <c r="AS9" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="AM9" s="5" t="s">
+      <c r="AT9" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="AN9" s="5">
+      <c r="AU9" s="5">
         <v>10</v>
       </c>
-      <c r="AO9" s="5">
+      <c r="AV9" s="5">
         <v>10</v>
       </c>
-      <c r="AP9" s="5">
+      <c r="AW9" s="5">
         <v>10</v>
-      </c>
-      <c r="AQ9" s="5">
-        <v>11</v>
-      </c>
-      <c r="AR9" s="5">
-        <v>16</v>
-      </c>
-      <c r="AS9" s="5">
-        <v>16</v>
-      </c>
-      <c r="AT9" s="5">
-        <v>16</v>
-      </c>
-      <c r="AU9" s="5">
-        <v>23</v>
-      </c>
-      <c r="AV9" s="5">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="AW9" s="5">
-        <v>16</v>
       </c>
       <c r="AX9" s="5">
         <v>11</v>
       </c>
       <c r="AY9" s="5">
+        <v>3.1</v>
+      </c>
+      <c r="AZ9" s="5">
+        <v>2.8</v>
+      </c>
+      <c r="BA9" s="5">
+        <v>3.4</v>
+      </c>
+      <c r="BB9" s="5">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="BC9" s="5">
+        <v>6.1</v>
+      </c>
+      <c r="BD9" s="5">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="BE9" s="5">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="BF9" s="5">
+        <v>16</v>
+      </c>
+      <c r="BG9" s="5">
+        <v>16</v>
+      </c>
+      <c r="BH9" s="5">
+        <v>16</v>
+      </c>
+      <c r="BI9" s="5">
+        <v>23</v>
+      </c>
+      <c r="BJ9" s="5">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="BK9" s="5">
+        <v>16</v>
+      </c>
+      <c r="BL9" s="5">
+        <v>11</v>
+      </c>
+      <c r="BM9" s="5">
         <v>15</v>
       </c>
-      <c r="AZ9" s="5">
+      <c r="BN9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BA9" s="5">
+      <c r="BO9" s="5">
         <v>15.3</v>
       </c>
-      <c r="BB9" s="5">
+      <c r="BP9" s="5">
         <v>30.3</v>
       </c>
-      <c r="BC9" s="5">
+      <c r="BQ9" s="5">
         <v>30.3</v>
       </c>
-      <c r="BD9" s="5">
+      <c r="BR9" s="5">
         <v>30.3</v>
       </c>
-      <c r="BE9" s="5">
+      <c r="BS9" s="5">
         <v>26.4</v>
       </c>
-      <c r="BF9" s="5">
+      <c r="BT9" s="5">
         <v>26.4</v>
       </c>
-      <c r="BG9" s="5">
+      <c r="BU9" s="5">
         <v>26.4</v>
       </c>
-      <c r="BH9" s="5">
+      <c r="BV9" s="5">
         <v>16.899999999999999</v>
       </c>
-      <c r="BI9" s="5">
+      <c r="BW9" s="5">
         <v>16.899999999999999</v>
       </c>
-      <c r="BJ9" s="5">
+      <c r="BX9" s="5">
         <v>16.899999999999999</v>
       </c>
-      <c r="BK9" s="5">
+      <c r="BY9" s="5">
         <v>18.8</v>
       </c>
-      <c r="BL9" s="5">
+      <c r="BZ9" s="5">
         <v>24.1</v>
       </c>
-      <c r="BM9" s="5">
+      <c r="CA9" s="5">
         <v>29.6</v>
       </c>
-      <c r="BN9" s="5">
+      <c r="CB9" s="5">
         <v>29.6</v>
       </c>
-      <c r="BO9" s="5">
+      <c r="CC9" s="5">
         <v>26.3</v>
       </c>
-      <c r="BP9" s="5">
+      <c r="CD9" s="5">
         <v>26.3</v>
       </c>
-      <c r="BQ9" s="5">
+      <c r="CE9" s="5">
         <v>26.3</v>
       </c>
-      <c r="BR9" s="5">
+      <c r="CF9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BS9" s="5">
+      <c r="CG9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BT9" s="5">
+      <c r="CH9" s="5">
         <v>16.399999999999999</v>
       </c>
-      <c r="BU9" s="5">
+      <c r="CI9" s="5">
         <v>20</v>
       </c>
-      <c r="BV9" s="5">
+      <c r="CJ9" s="5">
         <v>27</v>
       </c>
-      <c r="BW9" s="5">
+      <c r="CK9" s="5">
         <v>27</v>
       </c>
-      <c r="BX9" s="5">
+      <c r="CL9" s="5">
         <v>27</v>
       </c>
-      <c r="BY9" s="5">
+      <c r="CM9" s="5">
         <v>22</v>
       </c>
-      <c r="BZ9" s="5">
+      <c r="CN9" s="5">
         <v>24</v>
       </c>
-      <c r="CA9" s="5">
+      <c r="CO9" s="5">
         <v>26.5</v>
       </c>
-      <c r="CB9" s="5">
+      <c r="CP9" s="5">
         <v>26.5</v>
       </c>
-      <c r="CC9" s="5">
+      <c r="CQ9" s="5">
         <v>21.1</v>
       </c>
-      <c r="CD9" s="5">
+      <c r="CR9" s="5">
         <v>18.5</v>
       </c>
-      <c r="CE9" s="5">
+      <c r="CS9" s="5">
         <v>18.5</v>
       </c>
-      <c r="CF9" s="5">
+      <c r="CT9" s="5">
         <v>17.5</v>
       </c>
-      <c r="CG9" s="5">
+      <c r="CU9" s="5">
         <v>27</v>
       </c>
-      <c r="CH9" s="5">
+      <c r="CV9" s="5">
         <v>27</v>
       </c>
-      <c r="CI9" s="5">
+      <c r="CW9" s="5">
         <v>16.100000000000001</v>
       </c>
-      <c r="CJ9" s="5">
+      <c r="CX9" s="5">
         <v>21.2</v>
       </c>
-      <c r="CK9" s="5">
+      <c r="CY9" s="5">
         <v>22.5</v>
       </c>
-      <c r="CL9" s="5">
+      <c r="CZ9" s="5">
         <v>30.2</v>
       </c>
-      <c r="CM9" s="5">
+      <c r="DA9" s="5">
         <v>33.700000000000003</v>
       </c>
-      <c r="CN9" s="5">
+      <c r="DB9" s="5">
         <v>34.5</v>
       </c>
-      <c r="CO9" s="5">
+      <c r="DC9" s="5">
         <v>38.5</v>
       </c>
-      <c r="CP9" s="5">
+      <c r="DD9" s="5">
         <v>43.7</v>
       </c>
-      <c r="CQ9" s="5">
+      <c r="DE9" s="5">
         <v>45</v>
       </c>
-      <c r="CR9" s="5">
+      <c r="DF9" s="5">
         <v>52.7</v>
       </c>
-      <c r="CS9" s="5">
+      <c r="DG9" s="5">
         <v>56.2</v>
       </c>
-      <c r="CT9" s="5">
+      <c r="DH9" s="5">
         <v>63.9</v>
       </c>
-      <c r="CU9" s="5">
+      <c r="DI9" s="5">
         <v>64.7</v>
       </c>
-      <c r="CV9" s="5">
+      <c r="DJ9" s="5">
         <v>68.2</v>
       </c>
-      <c r="CW9" s="5">
+      <c r="DK9" s="5">
         <v>69</v>
       </c>
-      <c r="CX9" s="5">
+      <c r="DL9" s="5">
         <v>73</v>
       </c>
-      <c r="CY9" s="5">
+      <c r="DM9" s="5">
         <v>77</v>
       </c>
-      <c r="CZ9" s="5">
+      <c r="DN9" s="5">
         <v>79.5</v>
       </c>
-      <c r="DA9" s="5">
+      <c r="DO9" s="5">
         <v>83.5</v>
       </c>
-      <c r="DB9" s="5">
+      <c r="DP9" s="5">
         <v>94.9</v>
       </c>
-      <c r="DC9" s="5">
+      <c r="DQ9" s="5">
         <v>98.4</v>
       </c>
-      <c r="DD9" s="5">
+      <c r="DR9" s="5">
         <v>99.2</v>
       </c>
-      <c r="DE9" s="5">
+      <c r="DS9" s="5">
         <v>102.7</v>
       </c>
-      <c r="DF9" s="5">
+      <c r="DT9" s="5">
         <v>103.5</v>
       </c>
-      <c r="DG9" s="5">
+      <c r="DU9" s="5">
         <v>107.5</v>
       </c>
-      <c r="DH9" s="5">
+      <c r="DV9" s="5">
         <v>111.5</v>
       </c>
-      <c r="DI9" s="5">
+      <c r="DW9" s="5">
         <v>115.5</v>
       </c>
-      <c r="DJ9" s="5">
+      <c r="DX9" s="5">
         <v>16.100000000000001</v>
       </c>
-      <c r="DK9" s="5">
+      <c r="DY9" s="5">
         <v>21.5</v>
       </c>
-      <c r="DL9" s="5">
+      <c r="DZ9" s="5">
         <v>22.9</v>
       </c>
-      <c r="DM9" s="5">
+      <c r="EA9" s="5">
         <v>30.2</v>
       </c>
-      <c r="DN9" s="5">
+      <c r="EB9" s="5">
         <v>34</v>
       </c>
-      <c r="DO9" s="5">
+      <c r="EC9" s="5">
         <v>34.700000000000003</v>
       </c>
-      <c r="DP9" s="5">
+      <c r="ED9" s="5">
         <v>39.700000000000003</v>
       </c>
-      <c r="DQ9" s="5">
+      <c r="EE9" s="5">
         <v>44.4</v>
       </c>
-      <c r="DR9" s="5">
+      <c r="EF9" s="5">
         <v>45.8</v>
       </c>
-      <c r="DS9" s="5">
+      <c r="EG9" s="5">
         <v>53.1</v>
       </c>
-      <c r="DT9" s="5">
+      <c r="EH9" s="5">
         <v>56.9</v>
       </c>
-      <c r="DU9" s="5">
+      <c r="EI9" s="5">
         <v>64.2</v>
       </c>
-      <c r="DV9" s="5">
+      <c r="EJ9" s="5">
         <v>64.900000000000006</v>
       </c>
-      <c r="DW9" s="5">
+      <c r="EK9" s="5">
         <v>68.7</v>
       </c>
-      <c r="DX9" s="5">
+      <c r="EL9" s="5">
         <v>69.400000000000006</v>
       </c>
-      <c r="DY9" s="5">
+      <c r="EM9" s="5">
         <v>74.400000000000006</v>
       </c>
-      <c r="DZ9" s="5">
+      <c r="EN9" s="5">
         <v>79.400000000000006</v>
       </c>
-      <c r="EA9" s="5">
+      <c r="EO9" s="5">
         <v>80.5</v>
       </c>
-      <c r="EB9" s="5">
+      <c r="EP9" s="5">
         <v>85.5</v>
       </c>
-      <c r="EC9" s="5">
+      <c r="EQ9" s="5">
         <v>95.1</v>
       </c>
-      <c r="ED9" s="5">
+      <c r="ER9" s="5">
         <v>98.9</v>
       </c>
-      <c r="EE9" s="5">
+      <c r="ES9" s="5">
         <v>99.6</v>
       </c>
-      <c r="EF9" s="5">
+      <c r="ET9" s="5">
         <v>103.4</v>
       </c>
-      <c r="EG9" s="5">
+      <c r="EU9" s="5">
         <v>104.1</v>
       </c>
-      <c r="EH9" s="5">
+      <c r="EV9" s="5">
         <v>109.1</v>
       </c>
-      <c r="EI9" s="5">
+      <c r="EW9" s="5">
         <v>114.1</v>
       </c>
-      <c r="EJ9" s="5">
+      <c r="EX9" s="5">
         <v>119.1</v>
       </c>
-      <c r="EK9" s="5"/>
-      <c r="EL9" s="5"/>
-      <c r="EM9" s="5"/>
-      <c r="EN9" s="5"/>
-      <c r="EO9" s="5"/>
-      <c r="EP9" s="5"/>
-      <c r="EQ9" s="5"/>
-      <c r="ER9" s="5"/>
-      <c r="ES9" s="5"/>
-      <c r="ET9" s="5"/>
-      <c r="EU9" s="5"/>
-      <c r="EV9" s="5"/>
-      <c r="EW9" s="5"/>
-      <c r="EX9" s="5"/>
       <c r="EY9" s="5"/>
       <c r="EZ9" s="5"/>
       <c r="FA9" s="5"/>
@@ -13724,8 +14106,22 @@
       <c r="FO9" s="5"/>
       <c r="FP9" s="5"/>
       <c r="FQ9" s="5"/>
+      <c r="FR9" s="5"/>
+      <c r="FS9" s="5"/>
+      <c r="FT9" s="5"/>
+      <c r="FU9" s="5"/>
+      <c r="FV9" s="5"/>
+      <c r="FW9" s="5"/>
+      <c r="FX9" s="5"/>
+      <c r="FY9" s="5"/>
+      <c r="FZ9" s="5"/>
+      <c r="GA9" s="5"/>
+      <c r="GB9" s="5"/>
+      <c r="GC9" s="5"/>
+      <c r="GD9" s="5"/>
+      <c r="GE9" s="5"/>
     </row>
-    <row r="10" spans="1:173" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:187" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>49</v>
       </c>
@@ -13851,77 +14247,77 @@
       <c r="AQ10" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AR10" s="5">
+      <c r="AR10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AS10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AU10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AV10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AW10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AX10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AY10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AZ10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="BA10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="BB10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="BC10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="BD10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="BE10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="BF10" s="5">
         <v>20</v>
       </c>
-      <c r="AS10" s="5">
+      <c r="BG10" s="5">
         <v>20</v>
-      </c>
-      <c r="AT10" s="5">
-        <v>20</v>
-      </c>
-      <c r="AU10" s="5">
-        <v>30</v>
-      </c>
-      <c r="AV10" s="5">
-        <v>10</v>
-      </c>
-      <c r="AW10" s="5">
-        <v>20</v>
-      </c>
-      <c r="AX10" s="5">
-        <v>19.600000000000001</v>
-      </c>
-      <c r="AY10" s="5">
-        <v>20</v>
-      </c>
-      <c r="AZ10" s="5">
-        <v>20</v>
-      </c>
-      <c r="BA10" s="5">
-        <v>16</v>
-      </c>
-      <c r="BB10" s="5">
-        <v>32</v>
-      </c>
-      <c r="BC10" s="5">
-        <v>32</v>
-      </c>
-      <c r="BD10" s="5">
-        <v>32</v>
-      </c>
-      <c r="BE10" s="5">
-        <v>32</v>
-      </c>
-      <c r="BF10" s="5">
-        <v>32</v>
-      </c>
-      <c r="BG10" s="5">
-        <v>32</v>
       </c>
       <c r="BH10" s="5">
         <v>20</v>
       </c>
       <c r="BI10" s="5">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="BJ10" s="5">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="BK10" s="5">
         <v>20</v>
       </c>
       <c r="BL10" s="5">
-        <v>25</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="BM10" s="5">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="BN10" s="5">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="BO10" s="5">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="BP10" s="5">
         <v>32</v>
@@ -13930,232 +14326,260 @@
         <v>32</v>
       </c>
       <c r="BR10" s="5">
+        <v>32</v>
+      </c>
+      <c r="BS10" s="5">
+        <v>32</v>
+      </c>
+      <c r="BT10" s="5">
+        <v>32</v>
+      </c>
+      <c r="BU10" s="5">
+        <v>32</v>
+      </c>
+      <c r="BV10" s="5">
         <v>20</v>
       </c>
-      <c r="BS10" s="5">
+      <c r="BW10" s="5">
         <v>20</v>
       </c>
-      <c r="BT10" s="5">
+      <c r="BX10" s="5">
         <v>20</v>
       </c>
-      <c r="BU10" s="5">
+      <c r="BY10" s="5">
+        <v>20</v>
+      </c>
+      <c r="BZ10" s="5">
         <v>25</v>
       </c>
-      <c r="BV10" s="5">
+      <c r="CA10" s="5">
+        <v>32</v>
+      </c>
+      <c r="CB10" s="5">
+        <v>32</v>
+      </c>
+      <c r="CC10" s="5">
+        <v>32</v>
+      </c>
+      <c r="CD10" s="5">
+        <v>32</v>
+      </c>
+      <c r="CE10" s="5">
+        <v>32</v>
+      </c>
+      <c r="CF10" s="5">
+        <v>20</v>
+      </c>
+      <c r="CG10" s="5">
+        <v>20</v>
+      </c>
+      <c r="CH10" s="5">
+        <v>20</v>
+      </c>
+      <c r="CI10" s="5">
+        <v>25</v>
+      </c>
+      <c r="CJ10" s="5">
         <v>30</v>
       </c>
-      <c r="BW10" s="5">
+      <c r="CK10" s="5">
         <v>30</v>
       </c>
-      <c r="BX10" s="5">
+      <c r="CL10" s="5">
         <v>30</v>
       </c>
-      <c r="BY10" s="5">
+      <c r="CM10" s="5">
         <v>25</v>
       </c>
-      <c r="BZ10" s="5">
+      <c r="CN10" s="5">
         <v>30</v>
       </c>
-      <c r="CA10" s="5">
+      <c r="CO10" s="5">
         <v>30</v>
       </c>
-      <c r="CB10" s="5">
+      <c r="CP10" s="5">
         <v>30</v>
       </c>
-      <c r="CC10" s="5">
+      <c r="CQ10" s="5">
         <v>30</v>
       </c>
-      <c r="CD10" s="5">
+      <c r="CR10" s="5">
         <v>25</v>
       </c>
-      <c r="CE10" s="5">
+      <c r="CS10" s="5">
         <v>25</v>
       </c>
-      <c r="CF10" s="5">
+      <c r="CT10" s="5">
         <v>25</v>
       </c>
-      <c r="CG10" s="5">
+      <c r="CU10" s="5">
         <v>30</v>
       </c>
-      <c r="CH10" s="5">
+      <c r="CV10" s="5">
         <v>30</v>
       </c>
-      <c r="CI10" s="5">
+      <c r="CW10" s="5">
         <v>20</v>
       </c>
-      <c r="CJ10" s="5">
+      <c r="CX10" s="5">
         <v>25</v>
       </c>
-      <c r="CK10" s="5">
+      <c r="CY10" s="5">
         <v>25</v>
       </c>
-      <c r="CL10" s="5">
+      <c r="CZ10" s="5">
         <v>35</v>
       </c>
-      <c r="CM10" s="5">
+      <c r="DA10" s="5">
         <v>40</v>
       </c>
-      <c r="CN10" s="5">
+      <c r="DB10" s="5">
         <v>40</v>
       </c>
-      <c r="CO10" s="5">
+      <c r="DC10" s="5">
         <v>45</v>
       </c>
-      <c r="CP10" s="5">
+      <c r="DD10" s="5">
         <v>50</v>
       </c>
-      <c r="CQ10" s="5">
+      <c r="DE10" s="5">
         <v>50</v>
       </c>
-      <c r="CR10" s="5">
+      <c r="DF10" s="5">
         <v>60</v>
       </c>
-      <c r="CS10" s="5">
+      <c r="DG10" s="5">
         <v>70</v>
       </c>
-      <c r="CT10" s="5">
+      <c r="DH10" s="5">
         <v>80</v>
       </c>
-      <c r="CU10" s="5">
+      <c r="DI10" s="5">
         <v>80</v>
       </c>
-      <c r="CV10" s="5">
+      <c r="DJ10" s="5">
         <v>80</v>
       </c>
-      <c r="CW10" s="5">
+      <c r="DK10" s="5">
         <v>80</v>
       </c>
-      <c r="CX10" s="5">
+      <c r="DL10" s="5">
         <v>90</v>
       </c>
-      <c r="CY10" s="5">
+      <c r="DM10" s="5">
         <v>90</v>
       </c>
-      <c r="CZ10" s="5">
+      <c r="DN10" s="5">
         <v>90</v>
       </c>
-      <c r="DA10" s="5">
+      <c r="DO10" s="5">
         <v>100</v>
       </c>
-      <c r="DB10" s="5">
+      <c r="DP10" s="5">
         <v>110</v>
       </c>
-      <c r="DC10" s="5">
+      <c r="DQ10" s="5">
         <v>110</v>
       </c>
-      <c r="DD10" s="5">
+      <c r="DR10" s="5">
         <v>110</v>
       </c>
-      <c r="DE10" s="5">
+      <c r="DS10" s="5">
         <v>125</v>
       </c>
-      <c r="DF10" s="5">
+      <c r="DT10" s="5">
         <v>125</v>
       </c>
-      <c r="DG10" s="5">
+      <c r="DU10" s="5">
         <v>125</v>
       </c>
-      <c r="DH10" s="5">
+      <c r="DV10" s="5">
         <v>125</v>
       </c>
-      <c r="DI10" s="5">
+      <c r="DW10" s="5">
         <v>150</v>
       </c>
-      <c r="DJ10" s="5">
+      <c r="DX10" s="5">
         <v>20</v>
       </c>
-      <c r="DK10" s="5">
+      <c r="DY10" s="5">
         <v>25</v>
       </c>
-      <c r="DL10" s="5">
+      <c r="DZ10" s="5">
         <v>30</v>
       </c>
-      <c r="DM10" s="5">
+      <c r="EA10" s="5">
         <v>35</v>
       </c>
-      <c r="DN10" s="5">
+      <c r="EB10" s="5">
         <v>40</v>
       </c>
-      <c r="DO10" s="5">
+      <c r="EC10" s="5">
         <v>40</v>
       </c>
-      <c r="DP10" s="5">
+      <c r="ED10" s="5">
         <v>45</v>
       </c>
-      <c r="DQ10" s="5">
+      <c r="EE10" s="5">
         <v>50</v>
       </c>
-      <c r="DR10" s="5">
+      <c r="EF10" s="5">
         <v>60</v>
       </c>
-      <c r="DS10" s="5">
+      <c r="EG10" s="5">
         <v>60</v>
       </c>
-      <c r="DT10" s="5">
+      <c r="EH10" s="5">
         <v>70</v>
       </c>
-      <c r="DU10" s="5">
+      <c r="EI10" s="5">
         <v>80</v>
       </c>
-      <c r="DV10" s="5">
+      <c r="EJ10" s="5">
         <v>80</v>
       </c>
-      <c r="DW10" s="5">
+      <c r="EK10" s="5">
         <v>80</v>
       </c>
-      <c r="DX10" s="5">
+      <c r="EL10" s="5">
         <v>80</v>
       </c>
-      <c r="DY10" s="5">
+      <c r="EM10" s="5">
         <v>90</v>
       </c>
-      <c r="DZ10" s="5">
+      <c r="EN10" s="5">
         <v>90</v>
       </c>
-      <c r="EA10" s="5">
+      <c r="EO10" s="5">
         <v>90</v>
       </c>
-      <c r="EB10" s="5">
+      <c r="EP10" s="5">
         <v>100</v>
       </c>
-      <c r="EC10" s="5">
+      <c r="EQ10" s="5">
         <v>110</v>
       </c>
-      <c r="ED10" s="5">
+      <c r="ER10" s="5">
         <v>110</v>
       </c>
-      <c r="EE10" s="5">
+      <c r="ES10" s="5">
         <v>110</v>
       </c>
-      <c r="EF10" s="5">
+      <c r="ET10" s="5">
         <v>125</v>
       </c>
-      <c r="EG10" s="5">
+      <c r="EU10" s="5">
         <v>125</v>
       </c>
-      <c r="EH10" s="5">
+      <c r="EV10" s="5">
         <v>125</v>
       </c>
-      <c r="EI10" s="5">
+      <c r="EW10" s="5">
         <v>150</v>
       </c>
-      <c r="EJ10" s="5">
+      <c r="EX10" s="5">
         <v>150</v>
       </c>
-      <c r="EK10" s="5"/>
-      <c r="EL10" s="5"/>
-      <c r="EM10" s="5"/>
-      <c r="EN10" s="5"/>
-      <c r="EO10" s="5"/>
-      <c r="EP10" s="5"/>
-      <c r="EQ10" s="5"/>
-      <c r="ER10" s="5"/>
-      <c r="ES10" s="5"/>
-      <c r="ET10" s="5"/>
-      <c r="EU10" s="5"/>
-      <c r="EV10" s="5"/>
-      <c r="EW10" s="5"/>
-      <c r="EX10" s="5"/>
       <c r="EY10" s="5"/>
       <c r="EZ10" s="5"/>
       <c r="FA10" s="5"/>
@@ -14175,8 +14599,22 @@
       <c r="FO10" s="5"/>
       <c r="FP10" s="5"/>
       <c r="FQ10" s="5"/>
+      <c r="FR10" s="5"/>
+      <c r="FS10" s="5"/>
+      <c r="FT10" s="5"/>
+      <c r="FU10" s="5"/>
+      <c r="FV10" s="5"/>
+      <c r="FW10" s="5"/>
+      <c r="FX10" s="5"/>
+      <c r="FY10" s="5"/>
+      <c r="FZ10" s="5"/>
+      <c r="GA10" s="5"/>
+      <c r="GB10" s="5"/>
+      <c r="GC10" s="5"/>
+      <c r="GD10" s="5"/>
+      <c r="GE10" s="5"/>
     </row>
-    <row r="11" spans="1:173" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:187" ht="25.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>58</v>
       </c>
@@ -14391,89 +14829,89 @@
       <c r="BT11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="BU11" s="15">
+      <c r="BU11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BV11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BW11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BX11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BY11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="BZ11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CA11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CB11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CC11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CD11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CE11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CF11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CG11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CH11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CI11" s="15">
         <v>40</v>
       </c>
-      <c r="BV11" s="15">
+      <c r="CJ11" s="15">
         <v>40</v>
       </c>
-      <c r="BW11" s="15">
+      <c r="CK11" s="15">
         <v>40</v>
       </c>
-      <c r="BX11" s="15">
+      <c r="CL11" s="15">
         <v>40</v>
       </c>
-      <c r="BY11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="BZ11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CA11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CB11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CC11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CD11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CE11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CF11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CG11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CH11" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="CI11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CJ11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CK11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CL11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CM11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CN11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CO11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CP11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CQ11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CR11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CS11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CT11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CU11" s="15">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="CV11" s="15">
-        <v>78.400000000000006</v>
+      <c r="CM11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CN11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CO11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CP11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CQ11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CR11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CS11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CT11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CU11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="CV11" s="15" t="s">
+        <v>37</v>
       </c>
       <c r="CW11" s="15">
         <v>78.400000000000006</v>
@@ -14595,20 +15033,48 @@
       <c r="EJ11" s="15">
         <v>78.400000000000006</v>
       </c>
-      <c r="EK11" s="15"/>
-      <c r="EL11" s="15"/>
-      <c r="EM11" s="15"/>
-      <c r="EN11" s="15"/>
-      <c r="EO11" s="15"/>
-      <c r="EP11" s="15"/>
-      <c r="EQ11" s="15"/>
-      <c r="ER11" s="15"/>
-      <c r="ES11" s="15"/>
-      <c r="ET11" s="15"/>
-      <c r="EU11" s="15"/>
-      <c r="EV11" s="15"/>
-      <c r="EW11" s="15"/>
-      <c r="EX11" s="15"/>
+      <c r="EK11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EL11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EM11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EN11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EO11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EP11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EQ11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="ER11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="ES11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="ET11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EU11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EV11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EW11" s="15">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="EX11" s="15">
+        <v>78.400000000000006</v>
+      </c>
       <c r="EY11" s="15"/>
       <c r="EZ11" s="15"/>
       <c r="FA11" s="15"/>
@@ -14628,8 +15094,22 @@
       <c r="FO11" s="15"/>
       <c r="FP11" s="15"/>
       <c r="FQ11" s="15"/>
+      <c r="FR11" s="15"/>
+      <c r="FS11" s="15"/>
+      <c r="FT11" s="15"/>
+      <c r="FU11" s="15"/>
+      <c r="FV11" s="15"/>
+      <c r="FW11" s="15"/>
+      <c r="FX11" s="15"/>
+      <c r="FY11" s="15"/>
+      <c r="FZ11" s="15"/>
+      <c r="GA11" s="15"/>
+      <c r="GB11" s="15"/>
+      <c r="GC11" s="15"/>
+      <c r="GD11" s="15"/>
+      <c r="GE11" s="15"/>
     </row>
-    <row r="12" spans="1:173" ht="60" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:187" ht="60" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>51</v>
       </c>
@@ -14739,103 +15219,103 @@
         <v>71</v>
       </c>
       <c r="AK12" s="15" t="s">
+        <v>523</v>
+      </c>
+      <c r="AL12" s="15" t="s">
+        <v>523</v>
+      </c>
+      <c r="AM12" s="15" t="s">
+        <v>535</v>
+      </c>
+      <c r="AN12" s="15" t="s">
+        <v>535</v>
+      </c>
+      <c r="AO12" s="15" t="s">
+        <v>535</v>
+      </c>
+      <c r="AP12" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="AQ12" s="15" t="s">
+        <v>525</v>
+      </c>
+      <c r="AR12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="AL12" s="15" t="s">
+      <c r="AS12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="AM12" s="15" t="s">
+      <c r="AT12" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="AN12" s="15" t="s">
+      <c r="AU12" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="AO12" s="15" t="s">
+      <c r="AV12" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="AP12" s="15" t="s">
+      <c r="AW12" s="15" t="s">
         <v>71</v>
-      </c>
-      <c r="AQ12" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="AR12" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="AS12" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="AT12" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="AU12" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="AV12" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="AW12" s="15" t="s">
-        <v>72</v>
       </c>
       <c r="AX12" s="15" t="s">
         <v>71</v>
       </c>
       <c r="AY12" s="15" t="s">
-        <v>74</v>
+        <v>523</v>
       </c>
       <c r="AZ12" s="15" t="s">
-        <v>71</v>
+        <v>523</v>
       </c>
       <c r="BA12" s="15" t="s">
-        <v>71</v>
+        <v>523</v>
       </c>
       <c r="BB12" s="15" t="s">
-        <v>74</v>
+        <v>524</v>
       </c>
       <c r="BC12" s="15" t="s">
-        <v>74</v>
+        <v>524</v>
       </c>
       <c r="BD12" s="15" t="s">
-        <v>74</v>
+        <v>524</v>
       </c>
       <c r="BE12" s="15" t="s">
-        <v>74</v>
+        <v>524</v>
       </c>
       <c r="BF12" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="BG12" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="BH12" s="15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="BI12" s="15" t="s">
         <v>74</v>
       </c>
       <c r="BJ12" s="15" t="s">
-        <v>74</v>
+        <v>40</v>
       </c>
       <c r="BK12" s="15" t="s">
-        <v>128</v>
+        <v>72</v>
       </c>
       <c r="BL12" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="BM12" s="15" t="s">
         <v>74</v>
       </c>
       <c r="BN12" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="BO12" s="15" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="BP12" s="15" t="s">
         <v>74</v>
       </c>
       <c r="BQ12" s="15" t="s">
-        <v>133</v>
+        <v>74</v>
       </c>
       <c r="BR12" s="15" t="s">
         <v>74</v>
@@ -14847,37 +15327,37 @@
         <v>74</v>
       </c>
       <c r="BU12" s="15" t="s">
-        <v>132</v>
+        <v>74</v>
       </c>
       <c r="BV12" s="15" t="s">
-        <v>132</v>
+        <v>74</v>
       </c>
       <c r="BW12" s="15" t="s">
-        <v>132</v>
+        <v>74</v>
       </c>
       <c r="BX12" s="15" t="s">
-        <v>132</v>
+        <v>74</v>
       </c>
       <c r="BY12" s="15" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="BZ12" s="15" t="s">
-        <v>153</v>
+        <v>74</v>
       </c>
       <c r="CA12" s="15" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="CB12" s="15" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="CC12" s="15" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="CD12" s="15" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="CE12" s="15" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="CF12" s="15" t="s">
         <v>74</v>
@@ -14889,181 +15369,209 @@
         <v>74</v>
       </c>
       <c r="CI12" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="CJ12" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="CK12" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="CL12" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="CM12" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="CN12" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="CO12" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="CP12" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="CQ12" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="CR12" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="CS12" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="CT12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="CU12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="CV12" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="CW12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CJ12" s="15" t="s">
+      <c r="CX12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CK12" s="15" t="s">
+      <c r="CY12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="CL12" s="15" t="s">
+      <c r="CZ12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CM12" s="15" t="s">
+      <c r="DA12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CN12" s="15" t="s">
+      <c r="DB12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CO12" s="15" t="s">
+      <c r="DC12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="CP12" s="15" t="s">
+      <c r="DD12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="CQ12" s="15" t="s">
+      <c r="DE12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="CR12" s="15" t="s">
+      <c r="DF12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="CS12" s="15" t="s">
+      <c r="DG12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="CT12" s="15" t="s">
+      <c r="DH12" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="CU12" s="15" t="s">
+      <c r="DI12" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="CV12" s="15" t="s">
+      <c r="DJ12" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="CW12" s="15" t="s">
+      <c r="DK12" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="CX12" s="15" t="s">
+      <c r="DL12" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="CY12" s="15" t="s">
+      <c r="DM12" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="CZ12" s="15" t="s">
+      <c r="DN12" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="DA12" s="15" t="s">
+      <c r="DO12" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="DB12" s="15" t="s">
+      <c r="DP12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DC12" s="15" t="s">
+      <c r="DQ12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DD12" s="15" t="s">
+      <c r="DR12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DE12" s="15" t="s">
+      <c r="DS12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DF12" s="15" t="s">
+      <c r="DT12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DG12" s="15" t="s">
+      <c r="DU12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DH12" s="15" t="s">
+      <c r="DV12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DI12" s="15" t="s">
+      <c r="DW12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="DJ12" s="15" t="s">
+      <c r="DX12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DK12" s="15" t="s">
+      <c r="DY12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DL12" s="15" t="s">
+      <c r="DZ12" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="DM12" s="15" t="s">
+      <c r="EA12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DN12" s="15" t="s">
+      <c r="EB12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DO12" s="15" t="s">
+      <c r="EC12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DP12" s="15" t="s">
+      <c r="ED12" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="DQ12" s="15" t="s">
+      <c r="EE12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="DR12" s="15" t="s">
+      <c r="EF12" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="DS12" s="15" t="s">
+      <c r="EG12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="DT12" s="15" t="s">
+      <c r="EH12" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="DU12" s="15" t="s">
+      <c r="EI12" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="DV12" s="15" t="s">
+      <c r="EJ12" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="DW12" s="15" t="s">
+      <c r="EK12" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="DX12" s="15" t="s">
+      <c r="EL12" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="DY12" s="15" t="s">
+      <c r="EM12" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="DZ12" s="15" t="s">
+      <c r="EN12" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="EA12" s="15" t="s">
+      <c r="EO12" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="EB12" s="15" t="s">
+      <c r="EP12" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="EC12" s="15" t="s">
+      <c r="EQ12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="ED12" s="15" t="s">
+      <c r="ER12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EE12" s="15" t="s">
+      <c r="ES12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EF12" s="15" t="s">
+      <c r="ET12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EG12" s="15" t="s">
+      <c r="EU12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EH12" s="15" t="s">
+      <c r="EV12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EI12" s="15" t="s">
+      <c r="EW12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EJ12" s="15" t="s">
+      <c r="EX12" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="EK12" s="15"/>
-      <c r="EL12" s="15"/>
-      <c r="EM12" s="15"/>
-      <c r="EN12" s="15"/>
-      <c r="EO12" s="15"/>
-      <c r="EP12" s="15"/>
-      <c r="EQ12" s="15"/>
-      <c r="ER12" s="15"/>
-      <c r="ES12" s="15"/>
-      <c r="ET12" s="15"/>
-      <c r="EU12" s="15"/>
-      <c r="EV12" s="15"/>
-      <c r="EW12" s="15"/>
-      <c r="EX12" s="15"/>
       <c r="EY12" s="15"/>
       <c r="EZ12" s="15"/>
       <c r="FA12" s="15"/>
@@ -15081,8 +15589,22 @@
       <c r="FM12" s="15"/>
       <c r="FN12" s="15"/>
       <c r="FO12" s="15"/>
+      <c r="FP12" s="15"/>
+      <c r="FQ12" s="15"/>
+      <c r="FR12" s="15"/>
+      <c r="FS12" s="15"/>
+      <c r="FT12" s="15"/>
+      <c r="FU12" s="15"/>
+      <c r="FV12" s="15"/>
+      <c r="FW12" s="15"/>
+      <c r="FX12" s="15"/>
+      <c r="FY12" s="15"/>
+      <c r="FZ12" s="15"/>
+      <c r="GA12" s="15"/>
+      <c r="GB12" s="15"/>
+      <c r="GC12" s="15"/>
     </row>
-    <row r="13" spans="1:173" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:187" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
         <v>54</v>
       </c>
@@ -15310,25 +15832,25 @@
         <v>56</v>
       </c>
       <c r="BY13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="BZ13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="CA13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="CB13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="CC13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="CD13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="CE13" s="12" t="s">
-        <v>155</v>
+        <v>56</v>
       </c>
       <c r="CF13" s="12" t="s">
         <v>56</v>
@@ -15340,46 +15862,46 @@
         <v>56</v>
       </c>
       <c r="CI13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CJ13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CK13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CL13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CM13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CN13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CO13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CP13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CQ13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CR13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CS13" s="12" t="s">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="CT13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CU13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CV13" s="12" t="s">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="CW13" s="12" t="s">
         <v>200</v>
@@ -15501,20 +16023,48 @@
       <c r="EJ13" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="EK13" s="12"/>
-      <c r="EL13" s="12"/>
-      <c r="EM13" s="12"/>
-      <c r="EN13" s="12"/>
-      <c r="EO13" s="12"/>
-      <c r="EP13" s="12"/>
-      <c r="EQ13" s="12"/>
-      <c r="ER13" s="12"/>
-      <c r="ES13" s="12"/>
-      <c r="ET13" s="12"/>
-      <c r="EU13" s="12"/>
-      <c r="EV13" s="12"/>
-      <c r="EW13" s="12"/>
-      <c r="EX13" s="12"/>
+      <c r="EK13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EL13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EM13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EN13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EO13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EP13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EQ13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="ER13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="ES13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="ET13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EU13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EV13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EW13" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="EX13" s="12" t="s">
+        <v>200</v>
+      </c>
       <c r="EY13" s="12"/>
       <c r="EZ13" s="12"/>
       <c r="FA13" s="12"/>
@@ -15534,6 +16084,20 @@
       <c r="FO13" s="12"/>
       <c r="FP13" s="12"/>
       <c r="FQ13" s="12"/>
+      <c r="FR13" s="12"/>
+      <c r="FS13" s="12"/>
+      <c r="FT13" s="12"/>
+      <c r="FU13" s="12"/>
+      <c r="FV13" s="12"/>
+      <c r="FW13" s="12"/>
+      <c r="FX13" s="12"/>
+      <c r="FY13" s="12"/>
+      <c r="FZ13" s="12"/>
+      <c r="GA13" s="12"/>
+      <c r="GB13" s="12"/>
+      <c r="GC13" s="12"/>
+      <c r="GD13" s="12"/>
+      <c r="GE13" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
release: v2.10.0 (2026.09.09) - optimize comparison toolbar scaling and preserve custom space geometry
</commit_message>
<xml_diff>
--- a/backend/product_database/EQUIPMENT_Data.xlsx
+++ b/backend/product_database/EQUIPMENT_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4319295-DF61-4E19-A223-D9095CBD8CF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650D0DD4-A300-44B5-9104-F2F595BE1E16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
+    <workbookView xWindow="60" yWindow="48" windowWidth="11832" windowHeight="12240" xr2:uid="{B9AE4098-F0A1-4C76-B9D5-37F1BE2208A4}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_units" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3120" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3528" uniqueCount="562">
   <si>
     <t>資料型態</t>
   </si>
@@ -2029,6 +2029,123 @@
     <t>冷暖上吹型</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>轉接小P版</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>集控轉接基板</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>室外機分歧頭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>遙控器型號</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>無線接收器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRC084C45</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>內建</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRP067A42</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRP072C42</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRP980B42</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KRP928BB2S</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRP084C45</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VRV / SA / RA</t>
+  </si>
+  <si>
+    <r>
+      <t>（必填）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve"> 區分系統，對應現有程式的判定。</t>
+    </r>
+  </si>
+  <si>
+    <t>橫綱V系列 / FXSQ</t>
+  </si>
+  <si>
+    <r>
+      <t>（必填）主鍵</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>，不可重複。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>（必填）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="微軟正黑體"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve"> 程式計算的核心冷房能力（kW）。</t>
+    </r>
+  </si>
+  <si>
+    <t>80 或 2.5馬力</t>
+  </si>
+  <si>
+    <t>最高靜壓（Pa），隱埋機型專屬，沒靜壓的填 0 或空著。</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>kRP928BB2S</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BRP072C42-1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -2037,7 +2154,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0_ "/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2089,6 +2206,29 @@
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="微軟正黑體"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="2"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -2104,7 +2244,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -2179,13 +2319,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2256,6 +2422,72 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -2572,7 +2804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E6F3F9-85F0-48DB-9A66-1B3BA6E48A6F}">
-  <dimension ref="A1:GL12"/>
+  <dimension ref="A1:GL16"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.109375" style="2" customWidth="1"/>
@@ -2584,222 +2816,222 @@
     <col min="194" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:194" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4"/>
-      <c r="AD1" s="4"/>
-      <c r="AE1" s="4"/>
-      <c r="AF1" s="4"/>
-      <c r="AG1" s="4"/>
-      <c r="AH1" s="4"/>
-      <c r="AI1" s="4"/>
-      <c r="AJ1" s="4"/>
-      <c r="AK1" s="4"/>
-      <c r="AL1" s="4"/>
-      <c r="AM1" s="4"/>
-      <c r="AN1" s="4"/>
-      <c r="AO1" s="4"/>
-      <c r="AP1" s="4"/>
-      <c r="AQ1" s="4"/>
-      <c r="AR1" s="4"/>
-      <c r="AS1" s="4"/>
-      <c r="AT1" s="4"/>
-      <c r="AU1" s="4"/>
-      <c r="AV1" s="4"/>
-      <c r="AW1" s="4"/>
-      <c r="AX1" s="4"/>
-      <c r="AY1" s="4"/>
-      <c r="AZ1" s="4"/>
-      <c r="BA1" s="4"/>
-      <c r="BB1" s="4"/>
-      <c r="BC1" s="4"/>
-      <c r="BD1" s="4"/>
-      <c r="BE1" s="4"/>
-      <c r="BF1" s="4"/>
-      <c r="BG1" s="4"/>
-      <c r="BH1" s="4"/>
-      <c r="BI1" s="4"/>
-      <c r="BJ1" s="4"/>
-      <c r="BK1" s="4"/>
-      <c r="BL1" s="4"/>
-      <c r="BM1" s="4"/>
-      <c r="BN1" s="4"/>
-      <c r="BO1" s="4"/>
-      <c r="BP1" s="4"/>
-      <c r="BQ1" s="4"/>
-      <c r="BR1" s="4"/>
-      <c r="BS1" s="4"/>
-      <c r="BT1" s="4"/>
-      <c r="BU1" s="4"/>
-      <c r="BV1" s="4"/>
-      <c r="BW1" s="4"/>
-      <c r="BX1" s="4"/>
-      <c r="BY1" s="4"/>
-      <c r="BZ1" s="4"/>
-      <c r="CA1" s="4"/>
-      <c r="CB1" s="4"/>
-      <c r="CC1" s="4"/>
-      <c r="CD1" s="4"/>
-      <c r="CE1" s="4"/>
-      <c r="CF1" s="4"/>
-      <c r="CG1" s="4"/>
-      <c r="CH1" s="4"/>
-      <c r="CI1" s="4"/>
-      <c r="CJ1" s="4"/>
-      <c r="CK1" s="4"/>
-      <c r="CL1" s="4"/>
-      <c r="CM1" s="4"/>
-      <c r="CN1" s="4"/>
-      <c r="CO1" s="4"/>
-      <c r="CP1" s="4"/>
-      <c r="CQ1" s="4"/>
-      <c r="CR1" s="4"/>
-      <c r="CS1" s="4"/>
-      <c r="CT1" s="4"/>
-      <c r="CU1" s="4"/>
-      <c r="CV1" s="4"/>
-      <c r="CW1" s="4"/>
-      <c r="CX1" s="4"/>
-      <c r="CY1" s="4"/>
-      <c r="CZ1" s="4"/>
-      <c r="DA1" s="4"/>
-      <c r="DB1" s="4"/>
-      <c r="DC1" s="4"/>
-      <c r="DD1" s="4"/>
-      <c r="DE1" s="4"/>
-      <c r="DF1" s="4"/>
-      <c r="DG1" s="4"/>
-      <c r="DH1" s="4"/>
-      <c r="DI1" s="4"/>
-      <c r="DJ1" s="4"/>
-      <c r="DK1" s="4"/>
-      <c r="DL1" s="4"/>
-      <c r="DM1" s="4"/>
-      <c r="DN1" s="4"/>
-      <c r="DO1" s="4"/>
-      <c r="DP1" s="4"/>
-      <c r="DQ1" s="4"/>
-      <c r="DR1" s="4"/>
-      <c r="DS1" s="4"/>
-      <c r="DT1" s="4"/>
-      <c r="DU1" s="4"/>
-      <c r="DV1" s="4"/>
-      <c r="DW1" s="4"/>
-      <c r="DX1" s="4"/>
-      <c r="DY1" s="4"/>
-      <c r="DZ1" s="4"/>
-      <c r="EA1" s="4"/>
-      <c r="EB1" s="4"/>
-      <c r="EC1" s="4"/>
-      <c r="ED1" s="4"/>
-      <c r="EE1" s="4"/>
-      <c r="EF1" s="4"/>
-      <c r="EG1" s="4"/>
-      <c r="EH1" s="4"/>
-      <c r="EI1" s="4"/>
-      <c r="EJ1" s="4"/>
-      <c r="EK1" s="4"/>
-      <c r="EL1" s="4"/>
-      <c r="EM1" s="4"/>
-      <c r="EN1" s="4"/>
-      <c r="EO1" s="4"/>
-      <c r="EP1" s="4"/>
-      <c r="EQ1" s="4"/>
-      <c r="ER1" s="4"/>
-      <c r="ES1" s="4"/>
-      <c r="ET1" s="4"/>
-      <c r="EU1" s="4"/>
-      <c r="EV1" s="4"/>
-      <c r="EW1" s="4"/>
-      <c r="EX1" s="4"/>
-      <c r="EY1" s="4"/>
-      <c r="EZ1" s="4"/>
-      <c r="FA1" s="4"/>
-      <c r="FB1" s="4"/>
-      <c r="FC1" s="4"/>
-      <c r="FD1" s="4"/>
-      <c r="FE1" s="4"/>
-      <c r="FF1" s="4"/>
-      <c r="FG1" s="4"/>
-      <c r="FH1" s="4"/>
-      <c r="FI1" s="4"/>
-      <c r="FJ1" s="4"/>
-      <c r="FK1" s="4"/>
-      <c r="FL1" s="4"/>
-      <c r="FM1" s="4"/>
-      <c r="FN1" s="4"/>
-      <c r="FO1" s="4"/>
-      <c r="FP1" s="4"/>
-      <c r="FQ1" s="4"/>
-      <c r="FR1" s="4"/>
-      <c r="FS1" s="4"/>
-      <c r="FT1" s="4"/>
-      <c r="FU1" s="4"/>
-      <c r="FV1" s="4"/>
-      <c r="FW1" s="4"/>
-      <c r="FX1" s="4"/>
-      <c r="FY1" s="4"/>
-      <c r="FZ1" s="4"/>
-      <c r="GA1" s="4"/>
-      <c r="GB1" s="4"/>
-      <c r="GC1" s="4"/>
-      <c r="GD1" s="4"/>
-      <c r="GE1" s="4"/>
-      <c r="GF1" s="4"/>
-      <c r="GG1" s="4"/>
-      <c r="GH1" s="4"/>
-      <c r="GI1" s="4"/>
-      <c r="GJ1" s="4"/>
-      <c r="GK1" s="4"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
+      <c r="O1" s="33"/>
+      <c r="P1" s="33"/>
+      <c r="Q1" s="33"/>
+      <c r="R1" s="33"/>
+      <c r="S1" s="33"/>
+      <c r="T1" s="33"/>
+      <c r="U1" s="33"/>
+      <c r="V1" s="33"/>
+      <c r="W1" s="33"/>
+      <c r="X1" s="33"/>
+      <c r="Y1" s="33"/>
+      <c r="Z1" s="33"/>
+      <c r="AA1" s="33"/>
+      <c r="AB1" s="33"/>
+      <c r="AC1" s="33"/>
+      <c r="AD1" s="33"/>
+      <c r="AE1" s="33"/>
+      <c r="AF1" s="33"/>
+      <c r="AG1" s="33"/>
+      <c r="AH1" s="33"/>
+      <c r="AI1" s="33"/>
+      <c r="AJ1" s="33"/>
+      <c r="AK1" s="33"/>
+      <c r="AL1" s="33"/>
+      <c r="AM1" s="33"/>
+      <c r="AN1" s="33"/>
+      <c r="AO1" s="33"/>
+      <c r="AP1" s="33"/>
+      <c r="AQ1" s="33"/>
+      <c r="AR1" s="33"/>
+      <c r="AS1" s="33"/>
+      <c r="AT1" s="33"/>
+      <c r="AU1" s="33"/>
+      <c r="AV1" s="33"/>
+      <c r="AW1" s="33"/>
+      <c r="AX1" s="33"/>
+      <c r="AY1" s="33"/>
+      <c r="AZ1" s="33"/>
+      <c r="BA1" s="33"/>
+      <c r="BB1" s="33"/>
+      <c r="BC1" s="33"/>
+      <c r="BD1" s="33"/>
+      <c r="BE1" s="33"/>
+      <c r="BF1" s="33"/>
+      <c r="BG1" s="33"/>
+      <c r="BH1" s="33"/>
+      <c r="BI1" s="33"/>
+      <c r="BJ1" s="33"/>
+      <c r="BK1" s="33"/>
+      <c r="BL1" s="33"/>
+      <c r="BM1" s="33"/>
+      <c r="BN1" s="33"/>
+      <c r="BO1" s="33"/>
+      <c r="BP1" s="33"/>
+      <c r="BQ1" s="33"/>
+      <c r="BR1" s="33"/>
+      <c r="BS1" s="33"/>
+      <c r="BT1" s="33"/>
+      <c r="BU1" s="33"/>
+      <c r="BV1" s="33"/>
+      <c r="BW1" s="33"/>
+      <c r="BX1" s="33"/>
+      <c r="BY1" s="33"/>
+      <c r="BZ1" s="33"/>
+      <c r="CA1" s="33"/>
+      <c r="CB1" s="33"/>
+      <c r="CC1" s="33"/>
+      <c r="CD1" s="33"/>
+      <c r="CE1" s="33"/>
+      <c r="CF1" s="33"/>
+      <c r="CG1" s="33"/>
+      <c r="CH1" s="33"/>
+      <c r="CI1" s="33"/>
+      <c r="CJ1" s="33"/>
+      <c r="CK1" s="33"/>
+      <c r="CL1" s="33"/>
+      <c r="CM1" s="33"/>
+      <c r="CN1" s="33"/>
+      <c r="CO1" s="33"/>
+      <c r="CP1" s="33"/>
+      <c r="CQ1" s="33"/>
+      <c r="CR1" s="33"/>
+      <c r="CS1" s="33"/>
+      <c r="CT1" s="33"/>
+      <c r="CU1" s="33"/>
+      <c r="CV1" s="33"/>
+      <c r="CW1" s="33"/>
+      <c r="CX1" s="33"/>
+      <c r="CY1" s="33"/>
+      <c r="CZ1" s="33"/>
+      <c r="DA1" s="33"/>
+      <c r="DB1" s="33"/>
+      <c r="DC1" s="33"/>
+      <c r="DD1" s="33"/>
+      <c r="DE1" s="33"/>
+      <c r="DF1" s="33"/>
+      <c r="DG1" s="33"/>
+      <c r="DH1" s="33"/>
+      <c r="DI1" s="33"/>
+      <c r="DJ1" s="33"/>
+      <c r="DK1" s="33"/>
+      <c r="DL1" s="33"/>
+      <c r="DM1" s="33"/>
+      <c r="DN1" s="33"/>
+      <c r="DO1" s="33"/>
+      <c r="DP1" s="33"/>
+      <c r="DQ1" s="33"/>
+      <c r="DR1" s="33"/>
+      <c r="DS1" s="33"/>
+      <c r="DT1" s="33"/>
+      <c r="DU1" s="33"/>
+      <c r="DV1" s="33"/>
+      <c r="DW1" s="33"/>
+      <c r="DX1" s="33"/>
+      <c r="DY1" s="33"/>
+      <c r="DZ1" s="33"/>
+      <c r="EA1" s="33"/>
+      <c r="EB1" s="33"/>
+      <c r="EC1" s="33"/>
+      <c r="ED1" s="33"/>
+      <c r="EE1" s="33"/>
+      <c r="EF1" s="33"/>
+      <c r="EG1" s="33"/>
+      <c r="EH1" s="33"/>
+      <c r="EI1" s="33"/>
+      <c r="EJ1" s="33"/>
+      <c r="EK1" s="33"/>
+      <c r="EL1" s="33"/>
+      <c r="EM1" s="33"/>
+      <c r="EN1" s="33"/>
+      <c r="EO1" s="33"/>
+      <c r="EP1" s="33"/>
+      <c r="EQ1" s="33"/>
+      <c r="ER1" s="33"/>
+      <c r="ES1" s="33"/>
+      <c r="ET1" s="33"/>
+      <c r="EU1" s="33"/>
+      <c r="EV1" s="33"/>
+      <c r="EW1" s="33"/>
+      <c r="EX1" s="33"/>
+      <c r="EY1" s="33"/>
+      <c r="EZ1" s="33"/>
+      <c r="FA1" s="33"/>
+      <c r="FB1" s="33"/>
+      <c r="FC1" s="33"/>
+      <c r="FD1" s="33"/>
+      <c r="FE1" s="33"/>
+      <c r="FF1" s="33"/>
+      <c r="FG1" s="33"/>
+      <c r="FH1" s="33"/>
+      <c r="FI1" s="33"/>
+      <c r="FJ1" s="33"/>
+      <c r="FK1" s="33"/>
+      <c r="FL1" s="33"/>
+      <c r="FM1" s="33"/>
+      <c r="FN1" s="33"/>
+      <c r="FO1" s="33"/>
+      <c r="FP1" s="33"/>
+      <c r="FQ1" s="33"/>
+      <c r="FR1" s="33"/>
+      <c r="FS1" s="33"/>
+      <c r="FT1" s="33"/>
+      <c r="FU1" s="33"/>
+      <c r="FV1" s="33"/>
+      <c r="FW1" s="33"/>
+      <c r="FX1" s="33"/>
+      <c r="FY1" s="33"/>
+      <c r="FZ1" s="33"/>
+      <c r="GA1" s="33"/>
+      <c r="GB1" s="33"/>
+      <c r="GC1" s="33"/>
+      <c r="GD1" s="33"/>
+      <c r="GE1" s="33"/>
+      <c r="GF1" s="33"/>
+      <c r="GG1" s="33"/>
+      <c r="GH1" s="33"/>
+      <c r="GI1" s="33"/>
+      <c r="GJ1" s="33"/>
+      <c r="GK1" s="33"/>
       <c r="GL1" s="4"/>
     </row>
-    <row r="2" spans="1:194" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="34" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>17</v>
+        <v>552</v>
+      </c>
+      <c r="D2" s="35" t="s">
+        <v>553</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>218</v>
@@ -3370,17 +3602,17 @@
       </c>
       <c r="GL2" s="5"/>
     </row>
-    <row r="3" spans="1:194" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="34" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="11" t="s">
+        <v>554</v>
+      </c>
+      <c r="D3" s="36" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="5" t="s">
@@ -3953,17 +4185,17 @@
       <c r="GL3" s="5"/>
     </row>
     <row r="4" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="34" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>19</v>
+      <c r="D4" s="35" t="s">
+        <v>555</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>236</v>
@@ -4534,18 +4766,18 @@
       </c>
       <c r="GL4" s="5"/>
     </row>
-    <row r="5" spans="1:194" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="34" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5">
         <v>9</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>20</v>
+      <c r="D5" s="35" t="s">
+        <v>556</v>
       </c>
       <c r="E5" s="20">
         <v>2.2000000000000002</v>
@@ -5117,16 +5349,16 @@
       <c r="GL5" s="5"/>
     </row>
     <row r="6" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="31" t="s">
         <v>474</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="34" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="D6" s="36" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="5" t="s">
@@ -5699,16 +5931,16 @@
       <c r="GL6" s="5"/>
     </row>
     <row r="7" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="31" t="s">
         <v>475</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="34" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="36" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="5" t="s">
@@ -6281,16 +6513,16 @@
       <c r="GL7" s="5"/>
     </row>
     <row r="8" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="34" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5">
         <v>0.12</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="36" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="5" t="s">
@@ -6863,16 +7095,16 @@
       <c r="GL8" s="5"/>
     </row>
     <row r="9" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="34" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="36" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="5" t="s">
@@ -7444,18 +7676,18 @@
       </c>
       <c r="GL9" s="5"/>
     </row>
-    <row r="10" spans="1:194" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="34" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5">
         <v>50</v>
       </c>
-      <c r="D10" s="11" t="s">
-        <v>22</v>
+      <c r="D10" s="36" t="s">
+        <v>558</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>414</v>
@@ -8027,16 +8259,16 @@
       <c r="GL10" s="5"/>
     </row>
     <row r="11" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="34" t="s">
         <v>3</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="36" t="s">
         <v>14</v>
       </c>
       <c r="E11" s="5" t="s">
@@ -8608,587 +8840,1885 @@
       </c>
       <c r="GL11" s="5"/>
     </row>
-    <row r="12" spans="1:194" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:194" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="36" t="s">
         <v>466</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="I12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="J12" s="9" t="s">
+      <c r="J12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="K12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="L12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="M12" s="9" t="s">
+      <c r="M12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="N12" s="9" t="s">
+      <c r="N12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="O12" s="9" t="s">
+      <c r="O12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="P12" s="9" t="s">
+      <c r="P12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="Q12" s="9" t="s">
+      <c r="Q12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="R12" s="9" t="s">
+      <c r="R12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="S12" s="9" t="s">
+      <c r="S12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="T12" s="9" t="s">
+      <c r="T12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="U12" s="9" t="s">
+      <c r="U12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="V12" s="9" t="s">
+      <c r="V12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="W12" s="9" t="s">
+      <c r="W12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="X12" s="9" t="s">
+      <c r="X12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="Y12" s="9" t="s">
+      <c r="Y12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="Z12" s="9" t="s">
+      <c r="Z12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AA12" s="9" t="s">
+      <c r="AA12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AB12" s="9" t="s">
+      <c r="AB12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AC12" s="9" t="s">
+      <c r="AC12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AD12" s="9" t="s">
+      <c r="AD12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AE12" s="9" t="s">
+      <c r="AE12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AF12" s="9" t="s">
+      <c r="AF12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AG12" s="9" t="s">
+      <c r="AG12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AH12" s="9" t="s">
+      <c r="AH12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AI12" s="9" t="s">
+      <c r="AI12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AJ12" s="9" t="s">
+      <c r="AJ12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AK12" s="9" t="s">
+      <c r="AK12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AL12" s="9" t="s">
+      <c r="AL12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AM12" s="9" t="s">
+      <c r="AM12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AN12" s="9" t="s">
+      <c r="AN12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AO12" s="9" t="s">
+      <c r="AO12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AP12" s="9" t="s">
+      <c r="AP12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AQ12" s="9" t="s">
+      <c r="AQ12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AR12" s="9" t="s">
+      <c r="AR12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AS12" s="9" t="s">
+      <c r="AS12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AT12" s="9" t="s">
+      <c r="AT12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AU12" s="9" t="s">
+      <c r="AU12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AV12" s="9" t="s">
+      <c r="AV12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AW12" s="9" t="s">
+      <c r="AW12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AX12" s="9" t="s">
+      <c r="AX12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AY12" s="9" t="s">
+      <c r="AY12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="AZ12" s="9" t="s">
+      <c r="AZ12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BA12" s="9" t="s">
+      <c r="BA12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BB12" s="9" t="s">
+      <c r="BB12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BC12" s="9" t="s">
+      <c r="BC12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BD12" s="9" t="s">
+      <c r="BD12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BE12" s="9" t="s">
+      <c r="BE12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BF12" s="9" t="s">
+      <c r="BF12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BG12" s="9" t="s">
+      <c r="BG12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BH12" s="9" t="s">
+      <c r="BH12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BI12" s="9" t="s">
+      <c r="BI12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BJ12" s="9" t="s">
+      <c r="BJ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BK12" s="9" t="s">
+      <c r="BK12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BL12" s="9" t="s">
+      <c r="BL12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BM12" s="9" t="s">
+      <c r="BM12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BN12" s="9" t="s">
+      <c r="BN12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BO12" s="9" t="s">
+      <c r="BO12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BP12" s="9" t="s">
+      <c r="BP12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BQ12" s="9" t="s">
+      <c r="BQ12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BR12" s="9" t="s">
+      <c r="BR12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BS12" s="9" t="s">
+      <c r="BS12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BT12" s="9" t="s">
+      <c r="BT12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BU12" s="9" t="s">
+      <c r="BU12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="BV12" s="9" t="s">
+      <c r="BV12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BW12" s="9" t="s">
+      <c r="BW12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BX12" s="9" t="s">
+      <c r="BX12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BY12" s="9" t="s">
+      <c r="BY12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="BZ12" s="9" t="s">
+      <c r="BZ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CA12" s="9" t="s">
+      <c r="CA12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CB12" s="9" t="s">
+      <c r="CB12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CC12" s="9" t="s">
+      <c r="CC12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CD12" s="9" t="s">
+      <c r="CD12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CE12" s="9" t="s">
+      <c r="CE12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CF12" s="9" t="s">
+      <c r="CF12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CG12" s="9" t="s">
+      <c r="CG12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CH12" s="9" t="s">
+      <c r="CH12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CI12" s="9" t="s">
+      <c r="CI12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="CJ12" s="9" t="s">
+      <c r="CJ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CK12" s="9" t="s">
+      <c r="CK12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CL12" s="9" t="s">
+      <c r="CL12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CM12" s="9" t="s">
+      <c r="CM12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CN12" s="9" t="s">
+      <c r="CN12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CO12" s="9" t="s">
+      <c r="CO12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CP12" s="9" t="s">
+      <c r="CP12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CQ12" s="9" t="s">
+      <c r="CQ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CR12" s="9" t="s">
+      <c r="CR12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CS12" s="9" t="s">
+      <c r="CS12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CT12" s="9" t="s">
+      <c r="CT12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CU12" s="9" t="s">
+      <c r="CU12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CV12" s="9" t="s">
+      <c r="CV12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CW12" s="9" t="s">
+      <c r="CW12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CX12" s="9" t="s">
+      <c r="CX12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CY12" s="9" t="s">
+      <c r="CY12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="CZ12" s="9" t="s">
+      <c r="CZ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DA12" s="9" t="s">
+      <c r="DA12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DB12" s="9" t="s">
+      <c r="DB12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DC12" s="9" t="s">
+      <c r="DC12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DD12" s="9" t="s">
+      <c r="DD12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DE12" s="9" t="s">
+      <c r="DE12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DF12" s="9" t="s">
+      <c r="DF12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DG12" s="9" t="s">
+      <c r="DG12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DH12" s="9" t="s">
+      <c r="DH12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DI12" s="9" t="s">
+      <c r="DI12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DJ12" s="9" t="s">
+      <c r="DJ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DK12" s="9" t="s">
+      <c r="DK12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DL12" s="9" t="s">
+      <c r="DL12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DM12" s="9" t="s">
+      <c r="DM12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DN12" s="9" t="s">
+      <c r="DN12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DO12" s="9" t="s">
+      <c r="DO12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DP12" s="9" t="s">
+      <c r="DP12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DQ12" s="9" t="s">
+      <c r="DQ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DR12" s="9" t="s">
+      <c r="DR12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DS12" s="9" t="s">
+      <c r="DS12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DT12" s="9" t="s">
+      <c r="DT12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DU12" s="9" t="s">
+      <c r="DU12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DV12" s="9" t="s">
+      <c r="DV12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DW12" s="9" t="s">
+      <c r="DW12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DX12" s="9" t="s">
+      <c r="DX12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DY12" s="9" t="s">
+      <c r="DY12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="DZ12" s="9" t="s">
+      <c r="DZ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="EA12" s="9" t="s">
+      <c r="EA12" s="5" t="s">
         <v>470</v>
       </c>
-      <c r="EB12" s="9" t="s">
+      <c r="EB12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EC12" s="9" t="s">
+      <c r="EC12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="ED12" s="9" t="s">
+      <c r="ED12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EE12" s="9" t="s">
+      <c r="EE12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EF12" s="9" t="s">
+      <c r="EF12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EG12" s="9" t="s">
+      <c r="EG12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EH12" s="9" t="s">
+      <c r="EH12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EI12" s="9" t="s">
+      <c r="EI12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EJ12" s="9" t="s">
+      <c r="EJ12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EK12" s="9" t="s">
+      <c r="EK12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EL12" s="9" t="s">
+      <c r="EL12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EM12" s="9" t="s">
+      <c r="EM12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EN12" s="9" t="s">
+      <c r="EN12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EO12" s="9" t="s">
+      <c r="EO12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EP12" s="9" t="s">
+      <c r="EP12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="EQ12" s="9" t="s">
+      <c r="EQ12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="ER12" s="9" t="s">
+      <c r="ER12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="ES12" s="9" t="s">
+      <c r="ES12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="ET12" s="9" t="s">
+      <c r="ET12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="EU12" s="9" t="s">
+      <c r="EU12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="EV12" s="9" t="s">
+      <c r="EV12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="EW12" s="9" t="s">
+      <c r="EW12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="EX12" s="9" t="s">
+      <c r="EX12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="EY12" s="9" t="s">
+      <c r="EY12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="EZ12" s="9" t="s">
+      <c r="EZ12" s="5" t="s">
         <v>471</v>
       </c>
-      <c r="FA12" s="9" t="s">
+      <c r="FA12" s="5" t="s">
         <v>471</v>
       </c>
-      <c r="FB12" s="9" t="s">
+      <c r="FB12" s="5" t="s">
         <v>471</v>
       </c>
-      <c r="FC12" s="9" t="s">
+      <c r="FC12" s="5" t="s">
         <v>472</v>
       </c>
-      <c r="FD12" s="9" t="s">
+      <c r="FD12" s="5" t="s">
         <v>472</v>
       </c>
-      <c r="FE12" s="9" t="s">
+      <c r="FE12" s="5" t="s">
         <v>472</v>
       </c>
-      <c r="FF12" s="9" t="s">
+      <c r="FF12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FG12" s="9" t="s">
+      <c r="FG12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FH12" s="9" t="s">
+      <c r="FH12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FI12" s="9" t="s">
+      <c r="FI12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FJ12" s="9" t="s">
+      <c r="FJ12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FK12" s="9" t="s">
+      <c r="FK12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FL12" s="9" t="s">
+      <c r="FL12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FM12" s="9" t="s">
+      <c r="FM12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FN12" s="9" t="s">
+      <c r="FN12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FO12" s="9" t="s">
+      <c r="FO12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FP12" s="9" t="s">
+      <c r="FP12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FQ12" s="9" t="s">
+      <c r="FQ12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FR12" s="9" t="s">
+      <c r="FR12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FS12" s="9" t="s">
+      <c r="FS12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FT12" s="9" t="s">
+      <c r="FT12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FU12" s="9" t="s">
+      <c r="FU12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FV12" s="9" t="s">
+      <c r="FV12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FW12" s="9" t="s">
+      <c r="FW12" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="FX12" s="9" t="s">
+      <c r="FX12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="FY12" s="9" t="s">
+      <c r="FY12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="FZ12" s="9" t="s">
+      <c r="FZ12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="GA12" s="9" t="s">
+      <c r="GA12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="GB12" s="9" t="s">
+      <c r="GB12" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="GC12" s="9" t="s">
+      <c r="GC12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GD12" s="9" t="s">
+      <c r="GD12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GE12" s="9" t="s">
+      <c r="GE12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GF12" s="9" t="s">
+      <c r="GF12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GG12" s="9" t="s">
+      <c r="GG12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GH12" s="9" t="s">
+      <c r="GH12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GI12" s="9" t="s">
+      <c r="GI12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GJ12" s="9" t="s">
+      <c r="GJ12" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="GK12" s="9" t="s">
+      <c r="GK12" s="5" t="s">
         <v>467</v>
       </c>
       <c r="GL12" s="9"/>
+    </row>
+    <row r="13" spans="1:194" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="39" t="s">
+        <v>543</v>
+      </c>
+      <c r="B13" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="40"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="40"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="39"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
+      <c r="Q13" s="39"/>
+      <c r="R13" s="39"/>
+      <c r="S13" s="39"/>
+      <c r="T13" s="39"/>
+      <c r="U13" s="39"/>
+      <c r="V13" s="39"/>
+      <c r="W13" s="39"/>
+      <c r="X13" s="39"/>
+      <c r="Y13" s="39"/>
+      <c r="Z13" s="39"/>
+      <c r="AA13" s="39"/>
+      <c r="AB13" s="39"/>
+      <c r="AC13" s="39"/>
+      <c r="AD13" s="39"/>
+      <c r="AE13" s="39"/>
+      <c r="AF13" s="39"/>
+      <c r="AG13" s="39"/>
+      <c r="AH13" s="39"/>
+      <c r="AI13" s="39"/>
+      <c r="AJ13" s="39"/>
+      <c r="AK13" s="39"/>
+      <c r="AL13" s="39"/>
+      <c r="AM13" s="39"/>
+      <c r="AN13" s="39"/>
+      <c r="AO13" s="39"/>
+      <c r="AP13" s="39"/>
+      <c r="AQ13" s="39"/>
+      <c r="AR13" s="39"/>
+      <c r="AS13" s="39"/>
+      <c r="AT13" s="39"/>
+      <c r="AU13" s="39"/>
+      <c r="AV13" s="39"/>
+      <c r="AW13" s="39"/>
+      <c r="AX13" s="39"/>
+      <c r="AY13" s="39"/>
+      <c r="AZ13" s="39"/>
+      <c r="BA13" s="39"/>
+      <c r="BB13" s="39"/>
+      <c r="BC13" s="39"/>
+      <c r="BD13" s="39"/>
+      <c r="BE13" s="39"/>
+      <c r="BF13" s="39"/>
+      <c r="BG13" s="39"/>
+      <c r="BH13" s="39"/>
+      <c r="BI13" s="39"/>
+      <c r="BJ13" s="39"/>
+      <c r="BK13" s="39"/>
+      <c r="BL13" s="39"/>
+      <c r="BM13" s="39"/>
+      <c r="BN13" s="39"/>
+      <c r="BO13" s="39"/>
+      <c r="BP13" s="39"/>
+      <c r="BQ13" s="39"/>
+      <c r="BR13" s="39"/>
+      <c r="BS13" s="39"/>
+      <c r="BT13" s="39"/>
+      <c r="BU13" s="39"/>
+      <c r="BV13" s="39"/>
+      <c r="BW13" s="39" t="s">
+        <v>559</v>
+      </c>
+      <c r="BX13" s="39"/>
+      <c r="BY13" s="39"/>
+      <c r="BZ13" s="39"/>
+      <c r="CA13" s="39"/>
+      <c r="CB13" s="39"/>
+      <c r="CC13" s="39"/>
+      <c r="CD13" s="39"/>
+      <c r="CE13" s="39"/>
+      <c r="CF13" s="39"/>
+      <c r="CG13" s="39"/>
+      <c r="CH13" s="39"/>
+      <c r="CI13" s="39"/>
+      <c r="CJ13" s="39"/>
+      <c r="CK13" s="39"/>
+      <c r="CL13" s="39"/>
+      <c r="CM13" s="39"/>
+      <c r="CN13" s="39"/>
+      <c r="CO13" s="39"/>
+      <c r="CP13" s="39"/>
+      <c r="CQ13" s="39"/>
+      <c r="CR13" s="39"/>
+      <c r="CS13" s="39"/>
+      <c r="CT13" s="39"/>
+      <c r="CU13" s="39"/>
+      <c r="CV13" s="39"/>
+      <c r="CW13" s="39"/>
+      <c r="CX13" s="39"/>
+      <c r="CY13" s="39"/>
+      <c r="CZ13" s="39"/>
+      <c r="DA13" s="39"/>
+      <c r="DB13" s="39"/>
+      <c r="DC13" s="39"/>
+      <c r="DD13" s="39"/>
+      <c r="DE13" s="39"/>
+      <c r="DF13" s="39"/>
+      <c r="DG13" s="39"/>
+      <c r="DH13" s="39"/>
+      <c r="DI13" s="39"/>
+      <c r="DJ13" s="39"/>
+      <c r="DK13" s="39"/>
+      <c r="DL13" s="39"/>
+      <c r="DM13" s="39"/>
+      <c r="DN13" s="39"/>
+      <c r="DO13" s="39"/>
+      <c r="DP13" s="39"/>
+      <c r="DQ13" s="39"/>
+      <c r="DR13" s="39"/>
+      <c r="DS13" s="39"/>
+      <c r="DT13" s="39"/>
+      <c r="DU13" s="39"/>
+      <c r="DV13" s="39"/>
+      <c r="DW13" s="39"/>
+      <c r="DX13" s="39"/>
+      <c r="DY13" s="39"/>
+      <c r="DZ13" s="39"/>
+      <c r="EA13" s="39"/>
+      <c r="EB13" s="39"/>
+      <c r="EC13" s="39"/>
+      <c r="ED13" s="39"/>
+      <c r="EE13" s="39"/>
+      <c r="EF13" s="39"/>
+      <c r="EG13" s="39"/>
+      <c r="EH13" s="39"/>
+      <c r="EI13" s="39"/>
+      <c r="EJ13" s="39"/>
+      <c r="EK13" s="39"/>
+      <c r="EL13" s="39"/>
+      <c r="EM13" s="39"/>
+      <c r="EN13" s="39"/>
+      <c r="EO13" s="39"/>
+      <c r="EP13" s="39"/>
+      <c r="EQ13" s="39"/>
+      <c r="ER13" s="39"/>
+      <c r="ES13" s="39"/>
+      <c r="ET13" s="39"/>
+      <c r="EU13" s="39"/>
+      <c r="EV13" s="39"/>
+      <c r="EW13" s="39"/>
+      <c r="EX13" s="39"/>
+      <c r="EY13" s="39"/>
+      <c r="EZ13" s="39"/>
+      <c r="FA13" s="39"/>
+      <c r="FB13" s="39"/>
+      <c r="FC13" s="39"/>
+      <c r="FD13" s="39"/>
+      <c r="FE13" s="39"/>
+      <c r="FF13" s="39"/>
+      <c r="FG13" s="39"/>
+      <c r="FH13" s="39"/>
+      <c r="FI13" s="39"/>
+      <c r="FJ13" s="39"/>
+      <c r="FK13" s="39"/>
+      <c r="FL13" s="39"/>
+      <c r="FM13" s="39"/>
+      <c r="FN13" s="39"/>
+      <c r="FO13" s="39"/>
+      <c r="FP13" s="39"/>
+      <c r="FQ13" s="39"/>
+      <c r="FR13" s="39"/>
+      <c r="FS13" s="39"/>
+      <c r="FT13" s="39"/>
+      <c r="FU13" s="39"/>
+      <c r="FV13" s="39"/>
+      <c r="FW13" s="39"/>
+      <c r="FX13" s="39"/>
+      <c r="FY13" s="39"/>
+      <c r="FZ13" s="39"/>
+      <c r="GA13" s="39"/>
+      <c r="GB13" s="39"/>
+      <c r="GC13" s="39"/>
+      <c r="GD13" s="39"/>
+      <c r="GE13" s="39"/>
+      <c r="GF13" s="39"/>
+      <c r="GG13" s="39"/>
+      <c r="GH13" s="39"/>
+      <c r="GI13" s="39"/>
+      <c r="GJ13" s="39"/>
+      <c r="GK13" s="39"/>
+    </row>
+    <row r="14" spans="1:194" customFormat="1" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="38" t="s">
+        <v>540</v>
+      </c>
+      <c r="B14" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="42"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="L14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="N14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="O14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="P14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="R14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="T14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="U14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="V14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="W14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="X14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AE14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AF14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AG14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AH14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AI14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AJ14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AK14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AL14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AM14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AN14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AO14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AP14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AQ14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AR14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AS14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AT14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AU14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AV14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AW14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AX14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="AY14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="AZ14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="BA14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="BB14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="BC14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="BD14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="BE14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="BF14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BG14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BH14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BI14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BJ14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BK14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BL14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BM14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BN14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BO14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BP14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BQ14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BR14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BS14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BT14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BU14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BV14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BW14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BX14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BY14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="BZ14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="CA14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="CB14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="CC14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="CD14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="CE14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="CF14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="CG14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="CH14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="CI14" s="29" t="s">
+        <v>549</v>
+      </c>
+      <c r="CJ14" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="CK14" s="43"/>
+      <c r="CL14" s="43"/>
+      <c r="CM14" s="43"/>
+      <c r="CN14" s="43"/>
+      <c r="CO14" s="43"/>
+      <c r="CP14" s="43"/>
+      <c r="CQ14" s="43"/>
+      <c r="CR14" s="43"/>
+      <c r="CS14" s="43"/>
+      <c r="CT14" s="43"/>
+      <c r="CU14" s="43"/>
+      <c r="CV14" s="43"/>
+      <c r="CW14" s="43"/>
+      <c r="CX14" s="43"/>
+      <c r="CY14" s="43"/>
+      <c r="CZ14" s="43"/>
+      <c r="DA14" s="43"/>
+      <c r="DB14" s="43"/>
+      <c r="DC14" s="43"/>
+      <c r="DD14" s="43"/>
+      <c r="DE14" s="43"/>
+      <c r="DF14" s="43"/>
+      <c r="DG14" s="43"/>
+      <c r="DH14" s="43"/>
+      <c r="DI14" s="43"/>
+      <c r="DJ14" s="43"/>
+      <c r="DK14" s="43"/>
+      <c r="DL14" s="43"/>
+      <c r="DM14" s="43"/>
+      <c r="DN14" s="43"/>
+      <c r="DO14" s="43"/>
+      <c r="DP14" s="43"/>
+      <c r="DQ14" s="43"/>
+      <c r="DR14" s="43"/>
+      <c r="DS14" s="43"/>
+      <c r="DT14" s="43"/>
+      <c r="DU14" s="43"/>
+      <c r="DV14" s="43"/>
+      <c r="DW14" s="43"/>
+      <c r="DX14" s="43"/>
+      <c r="DY14" s="43"/>
+      <c r="DZ14" s="43"/>
+      <c r="EA14" s="43"/>
+      <c r="EB14" s="43"/>
+      <c r="EC14" s="43"/>
+      <c r="ED14" s="43"/>
+      <c r="EE14" s="43"/>
+      <c r="EF14" s="43"/>
+      <c r="EG14" s="43"/>
+      <c r="EH14" s="43"/>
+      <c r="EI14" s="43"/>
+      <c r="EJ14" s="43"/>
+      <c r="EK14" s="43"/>
+      <c r="EL14" s="43"/>
+      <c r="EM14" s="43"/>
+      <c r="EN14" s="43"/>
+      <c r="EO14" s="43"/>
+      <c r="EP14" s="43"/>
+      <c r="EQ14" s="43"/>
+      <c r="ER14" s="43"/>
+      <c r="ES14" s="43"/>
+      <c r="ET14" s="43"/>
+      <c r="EU14" s="43"/>
+      <c r="EV14" s="43"/>
+      <c r="EW14" s="43"/>
+      <c r="EX14" s="43"/>
+      <c r="EY14" s="43"/>
+      <c r="EZ14" s="43"/>
+      <c r="FA14" s="43"/>
+      <c r="FB14" s="43"/>
+      <c r="FC14" s="43"/>
+      <c r="FD14" s="43"/>
+      <c r="FE14" s="43"/>
+      <c r="FF14" s="43"/>
+      <c r="FG14" s="43"/>
+      <c r="FH14" s="43"/>
+      <c r="FI14" s="43"/>
+      <c r="FJ14" s="43"/>
+      <c r="FK14" s="43"/>
+      <c r="FL14" s="43"/>
+      <c r="FM14" s="43"/>
+      <c r="FN14" s="43"/>
+      <c r="FO14" s="43"/>
+      <c r="FP14" s="43"/>
+      <c r="FQ14" s="43"/>
+      <c r="FR14" s="43"/>
+      <c r="FS14" s="43"/>
+      <c r="FT14" s="43"/>
+      <c r="FU14" s="43"/>
+      <c r="FV14" s="43"/>
+      <c r="FW14" s="43"/>
+      <c r="FX14" s="43"/>
+      <c r="FY14" s="43"/>
+      <c r="FZ14" s="43"/>
+      <c r="GA14" s="43"/>
+      <c r="GB14" s="43"/>
+      <c r="GC14" s="43"/>
+      <c r="GD14" s="43"/>
+      <c r="GE14" s="43"/>
+      <c r="GF14" s="43"/>
+      <c r="GG14" s="43"/>
+      <c r="GH14" s="43"/>
+      <c r="GI14" s="43"/>
+      <c r="GJ14" s="43"/>
+      <c r="GK14" s="43"/>
+    </row>
+    <row r="15" spans="1:194" customFormat="1" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="38" t="s">
+        <v>544</v>
+      </c>
+      <c r="B15" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="42"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="G15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="H15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="I15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="J15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="K15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="L15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="M15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="N15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="O15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="P15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="Q15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="R15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="S15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="T15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="U15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="V15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="W15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="X15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="Y15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="Z15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="AA15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="AB15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="AC15" s="43" t="s">
+        <v>545</v>
+      </c>
+      <c r="AD15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AE15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AF15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AG15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AH15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AI15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AJ15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AK15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AL15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AM15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AN15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AO15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AP15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AQ15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AR15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AS15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AT15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AU15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AV15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AW15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AX15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AY15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="AZ15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BA15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BB15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BC15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BD15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BE15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BF15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BG15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BH15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BI15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BJ15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BK15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BL15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BM15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BN15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BO15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BP15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BQ15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BR15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BS15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BT15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BU15" s="43" t="s">
+        <v>546</v>
+      </c>
+      <c r="BV15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BW15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BX15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BY15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="BZ15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CA15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CB15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CC15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CD15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CE15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CF15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CG15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CH15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CI15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="CJ15" s="43"/>
+      <c r="CK15" s="43"/>
+      <c r="CL15" s="43"/>
+      <c r="CM15" s="43"/>
+      <c r="CN15" s="43"/>
+      <c r="CO15" s="43"/>
+      <c r="CP15" s="43"/>
+      <c r="CQ15" s="43"/>
+      <c r="CR15" s="43"/>
+      <c r="CS15" s="43"/>
+      <c r="CT15" s="43"/>
+      <c r="CU15" s="43"/>
+      <c r="CV15" s="43"/>
+      <c r="CW15" s="43"/>
+      <c r="CX15" s="43"/>
+      <c r="CY15" s="43"/>
+      <c r="CZ15" s="43"/>
+      <c r="DA15" s="43"/>
+      <c r="DB15" s="43"/>
+      <c r="DC15" s="43"/>
+      <c r="DD15" s="43"/>
+      <c r="DE15" s="43"/>
+      <c r="DF15" s="43"/>
+      <c r="DG15" s="43"/>
+      <c r="DH15" s="43"/>
+      <c r="DI15" s="43"/>
+      <c r="DJ15" s="43"/>
+      <c r="DK15" s="43"/>
+      <c r="DL15" s="43"/>
+      <c r="DM15" s="43"/>
+      <c r="DN15" s="43"/>
+      <c r="DO15" s="43"/>
+      <c r="DP15" s="43"/>
+      <c r="DQ15" s="43"/>
+      <c r="DR15" s="43"/>
+      <c r="DS15" s="43"/>
+      <c r="DT15" s="43"/>
+      <c r="DU15" s="43"/>
+      <c r="DV15" s="43"/>
+      <c r="DW15" s="43"/>
+      <c r="DX15" s="43"/>
+      <c r="DY15" s="43"/>
+      <c r="DZ15" s="43"/>
+      <c r="EA15" s="43"/>
+      <c r="EB15" s="43"/>
+      <c r="EC15" s="43"/>
+      <c r="ED15" s="43"/>
+      <c r="EE15" s="43"/>
+      <c r="EF15" s="43"/>
+      <c r="EG15" s="43"/>
+      <c r="EH15" s="43"/>
+      <c r="EI15" s="43"/>
+      <c r="EJ15" s="43"/>
+      <c r="EK15" s="43"/>
+      <c r="EL15" s="43"/>
+      <c r="EM15" s="43"/>
+      <c r="EN15" s="43"/>
+      <c r="EO15" s="43"/>
+      <c r="EP15" s="43"/>
+      <c r="EQ15" s="43"/>
+      <c r="ER15" s="43"/>
+      <c r="ES15" s="43"/>
+      <c r="ET15" s="43"/>
+      <c r="EU15" s="43"/>
+      <c r="EV15" s="43"/>
+      <c r="EW15" s="43"/>
+      <c r="EX15" s="43"/>
+      <c r="EY15" s="43"/>
+      <c r="EZ15" s="43"/>
+      <c r="FA15" s="43"/>
+      <c r="FB15" s="43"/>
+      <c r="FC15" s="43"/>
+      <c r="FD15" s="43"/>
+      <c r="FE15" s="43"/>
+      <c r="FF15" s="43"/>
+      <c r="FG15" s="43"/>
+      <c r="FH15" s="43"/>
+      <c r="FI15" s="43"/>
+      <c r="FJ15" s="43"/>
+      <c r="FK15" s="43"/>
+      <c r="FL15" s="43"/>
+      <c r="FM15" s="43"/>
+      <c r="FN15" s="43"/>
+      <c r="FO15" s="43"/>
+      <c r="FP15" s="43"/>
+      <c r="FQ15" s="43"/>
+      <c r="FR15" s="43"/>
+      <c r="FS15" s="43"/>
+      <c r="FT15" s="43"/>
+      <c r="FU15" s="43"/>
+      <c r="FV15" s="43"/>
+      <c r="FW15" s="43"/>
+      <c r="FX15" s="43"/>
+      <c r="FY15" s="43"/>
+      <c r="FZ15" s="43"/>
+      <c r="GA15" s="43"/>
+      <c r="GB15" s="43"/>
+      <c r="GC15" s="43"/>
+      <c r="GD15" s="43"/>
+      <c r="GE15" s="43"/>
+      <c r="GF15" s="43"/>
+      <c r="GG15" s="43"/>
+      <c r="GH15" s="43"/>
+      <c r="GI15" s="43"/>
+      <c r="GJ15" s="43"/>
+      <c r="GK15" s="43"/>
+    </row>
+    <row r="16" spans="1:194" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="38" t="s">
+        <v>541</v>
+      </c>
+      <c r="B16" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="42"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="F16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="G16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="H16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="I16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="J16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="K16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="L16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="M16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="N16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="O16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="P16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="Q16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="R16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="S16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="T16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="U16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="V16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="W16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="X16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="Y16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="Z16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AA16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AB16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AC16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AD16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AE16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AF16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AG16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AH16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AI16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AJ16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AK16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AL16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AM16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AN16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AO16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AP16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AQ16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AR16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AS16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AT16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AU16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AV16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AW16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AX16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AY16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="AZ16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BA16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BB16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BC16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BD16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BE16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BF16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BG16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BH16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BI16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BJ16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BK16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BL16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BM16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BN16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BO16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BP16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BQ16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BR16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BS16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BT16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BU16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BV16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BW16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BX16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BY16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="BZ16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CA16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CB16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CC16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CD16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CE16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CF16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CG16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CH16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CI16" s="43" t="s">
+        <v>550</v>
+      </c>
+      <c r="CJ16" s="43"/>
+      <c r="CK16" s="43"/>
+      <c r="CL16" s="43"/>
+      <c r="CM16" s="43"/>
+      <c r="CN16" s="43"/>
+      <c r="CO16" s="43"/>
+      <c r="CP16" s="43"/>
+      <c r="CQ16" s="43"/>
+      <c r="CR16" s="43"/>
+      <c r="CS16" s="43"/>
+      <c r="CT16" s="43"/>
+      <c r="CU16" s="43"/>
+      <c r="CV16" s="43"/>
+      <c r="CW16" s="43"/>
+      <c r="CX16" s="43"/>
+      <c r="CY16" s="43"/>
+      <c r="CZ16" s="43"/>
+      <c r="DA16" s="43"/>
+      <c r="DB16" s="43"/>
+      <c r="DC16" s="43"/>
+      <c r="DD16" s="43"/>
+      <c r="DE16" s="43"/>
+      <c r="DF16" s="43"/>
+      <c r="DG16" s="43"/>
+      <c r="DH16" s="43"/>
+      <c r="DI16" s="43"/>
+      <c r="DJ16" s="43"/>
+      <c r="DK16" s="43"/>
+      <c r="DL16" s="43"/>
+      <c r="DM16" s="43"/>
+      <c r="DN16" s="43"/>
+      <c r="DO16" s="43"/>
+      <c r="DP16" s="43"/>
+      <c r="DQ16" s="43"/>
+      <c r="DR16" s="43"/>
+      <c r="DS16" s="43"/>
+      <c r="DT16" s="43"/>
+      <c r="DU16" s="43"/>
+      <c r="DV16" s="43"/>
+      <c r="DW16" s="43"/>
+      <c r="DX16" s="43"/>
+      <c r="DY16" s="43"/>
+      <c r="DZ16" s="43"/>
+      <c r="EA16" s="43"/>
+      <c r="EB16" s="43"/>
+      <c r="EC16" s="43"/>
+      <c r="ED16" s="43"/>
+      <c r="EE16" s="43"/>
+      <c r="EF16" s="43"/>
+      <c r="EG16" s="43"/>
+      <c r="EH16" s="43"/>
+      <c r="EI16" s="43"/>
+      <c r="EJ16" s="43"/>
+      <c r="EK16" s="43"/>
+      <c r="EL16" s="43"/>
+      <c r="EM16" s="43"/>
+      <c r="EN16" s="43"/>
+      <c r="EO16" s="43"/>
+      <c r="EP16" s="43"/>
+      <c r="EQ16" s="43"/>
+      <c r="ER16" s="43"/>
+      <c r="ES16" s="43"/>
+      <c r="ET16" s="43"/>
+      <c r="EU16" s="43"/>
+      <c r="EV16" s="43"/>
+      <c r="EW16" s="43"/>
+      <c r="EX16" s="43"/>
+      <c r="EY16" s="43"/>
+      <c r="EZ16" s="43"/>
+      <c r="FA16" s="43"/>
+      <c r="FB16" s="43"/>
+      <c r="FC16" s="43"/>
+      <c r="FD16" s="43"/>
+      <c r="FE16" s="43"/>
+      <c r="FF16" s="43"/>
+      <c r="FG16" s="43"/>
+      <c r="FH16" s="43"/>
+      <c r="FI16" s="43"/>
+      <c r="FJ16" s="43"/>
+      <c r="FK16" s="43"/>
+      <c r="FL16" s="43"/>
+      <c r="FM16" s="43"/>
+      <c r="FN16" s="43"/>
+      <c r="FO16" s="43"/>
+      <c r="FP16" s="43"/>
+      <c r="FQ16" s="43"/>
+      <c r="FR16" s="43"/>
+      <c r="FS16" s="43"/>
+      <c r="FT16" s="43"/>
+      <c r="FU16" s="43"/>
+      <c r="FV16" s="43"/>
+      <c r="FW16" s="43"/>
+      <c r="FX16" s="43"/>
+      <c r="FY16" s="43"/>
+      <c r="FZ16" s="43"/>
+      <c r="GA16" s="43"/>
+      <c r="GB16" s="43"/>
+      <c r="GC16" s="43"/>
+      <c r="GD16" s="43"/>
+      <c r="GE16" s="43"/>
+      <c r="GF16" s="43"/>
+      <c r="GG16" s="43"/>
+      <c r="GH16" s="43"/>
+      <c r="GI16" s="43"/>
+      <c r="GJ16" s="43"/>
+      <c r="GK16" s="43"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -9199,7 +10729,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14518F8B-544C-42CB-BD27-24B9976359F4}">
-  <dimension ref="A1:FG13"/>
+  <dimension ref="A1:FG14"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
@@ -13894,7 +15424,7 @@
       <c r="A13" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="24" t="s">
         <v>55</v>
       </c>
       <c r="C13" s="12" t="s">
@@ -14313,6 +15843,291 @@
       <c r="FF13" s="12"/>
       <c r="FG13" s="12"/>
     </row>
+    <row r="14" spans="1:163" ht="25.35" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="21"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="L14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="N14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="O14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="P14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="R14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="T14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="U14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="V14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="W14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="X14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AF14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AG14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AH14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AI14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AK14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AL14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AN14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AO14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AP14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AQ14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AR14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AT14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AU14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AV14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AW14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AX14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AY14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="AZ14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BA14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BB14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BC14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BD14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BE14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BF14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BG14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BH14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BI14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BJ14" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="BK14" s="21"/>
+      <c r="BL14" s="21"/>
+      <c r="BM14" s="21"/>
+      <c r="BN14" s="21"/>
+      <c r="BO14" s="21"/>
+      <c r="BP14" s="21"/>
+      <c r="BQ14" s="21"/>
+      <c r="BR14" s="21"/>
+      <c r="BS14" s="21"/>
+      <c r="BT14" s="21"/>
+      <c r="BU14" s="21"/>
+      <c r="BV14" s="21"/>
+      <c r="BW14" s="21"/>
+      <c r="BX14" s="21"/>
+      <c r="BY14" s="21"/>
+      <c r="BZ14" s="21"/>
+      <c r="CA14" s="21"/>
+      <c r="CB14" s="21"/>
+      <c r="CC14" s="21"/>
+      <c r="CD14" s="21"/>
+      <c r="CE14" s="21"/>
+      <c r="CF14" s="21"/>
+      <c r="CG14" s="21"/>
+      <c r="CH14" s="21"/>
+      <c r="CI14" s="21"/>
+      <c r="CJ14" s="21"/>
+      <c r="CK14" s="21"/>
+      <c r="CL14" s="21"/>
+      <c r="CM14" s="21"/>
+      <c r="CN14" s="21"/>
+      <c r="CO14" s="21"/>
+      <c r="CP14" s="21"/>
+      <c r="CQ14" s="21"/>
+      <c r="CR14" s="21"/>
+      <c r="CS14" s="21"/>
+      <c r="CT14" s="21"/>
+      <c r="CU14" s="21"/>
+      <c r="CV14" s="21"/>
+      <c r="CW14" s="21"/>
+      <c r="CX14" s="21"/>
+      <c r="CY14" s="21"/>
+      <c r="CZ14" s="21"/>
+      <c r="DA14" s="21"/>
+      <c r="DB14" s="21"/>
+      <c r="DC14" s="21"/>
+      <c r="DD14" s="21"/>
+      <c r="DE14" s="21"/>
+      <c r="DF14" s="21"/>
+      <c r="DG14" s="21"/>
+      <c r="DH14" s="21"/>
+      <c r="DI14" s="21"/>
+      <c r="DJ14" s="21"/>
+      <c r="DK14" s="21"/>
+      <c r="DL14" s="21"/>
+      <c r="DM14" s="21"/>
+      <c r="DN14" s="21"/>
+      <c r="DO14" s="21"/>
+      <c r="DP14" s="21"/>
+      <c r="DQ14" s="21"/>
+      <c r="DR14" s="21"/>
+      <c r="DS14" s="21"/>
+      <c r="DT14" s="21"/>
+      <c r="DU14" s="21"/>
+      <c r="DV14" s="21"/>
+      <c r="DW14" s="21"/>
+      <c r="DX14" s="21"/>
+      <c r="DY14" s="21"/>
+      <c r="DZ14" s="21"/>
+      <c r="EA14" s="21"/>
+      <c r="EB14" s="21"/>
+      <c r="EC14" s="21"/>
+      <c r="ED14" s="21"/>
+      <c r="EE14" s="21"/>
+      <c r="EF14" s="21"/>
+      <c r="EG14" s="21"/>
+      <c r="EH14" s="21"/>
+      <c r="EI14" s="21"/>
+      <c r="EJ14" s="21"/>
+      <c r="EK14" s="21"/>
+      <c r="EL14" s="21"/>
+      <c r="EM14" s="21"/>
+      <c r="EN14" s="21"/>
+      <c r="EO14" s="21"/>
+      <c r="EP14" s="21"/>
+      <c r="EQ14" s="21"/>
+      <c r="ER14" s="21"/>
+      <c r="ES14" s="21"/>
+      <c r="ET14" s="21"/>
+      <c r="EU14" s="21"/>
+      <c r="EV14" s="21"/>
+      <c r="EW14" s="21"/>
+      <c r="EX14" s="21"/>
+      <c r="EY14" s="21"/>
+      <c r="EZ14" s="21"/>
+      <c r="FA14" s="21"/>
+      <c r="FB14" s="21"/>
+      <c r="FC14" s="21"/>
+      <c r="FD14" s="21"/>
+      <c r="FE14" s="21"/>
+      <c r="FF14" s="21"/>
+      <c r="FG14" s="21"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14322,7 +16137,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB764343-28B8-406D-977B-66BB2AAB408D}">
-  <dimension ref="A1:AF12"/>
+  <dimension ref="A1:AF16"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.109375" style="2" customWidth="1"/>
@@ -15430,6 +17245,314 @@
         <v>468</v>
       </c>
       <c r="AF12" s="9"/>
+    </row>
+    <row r="13" spans="1:32" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="22"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="22"/>
+      <c r="J13" s="22"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="22"/>
+      <c r="Q13" s="22"/>
+      <c r="R13" s="22"/>
+      <c r="S13" s="22"/>
+      <c r="T13" s="22"/>
+      <c r="U13" s="22"/>
+      <c r="V13" s="22"/>
+      <c r="W13" s="22"/>
+      <c r="X13" s="22"/>
+      <c r="Y13" s="22"/>
+      <c r="Z13" s="22"/>
+      <c r="AA13" s="22"/>
+      <c r="AB13" s="22"/>
+      <c r="AC13" s="22"/>
+      <c r="AD13" s="22"/>
+      <c r="AE13" s="22"/>
+      <c r="AF13" s="22"/>
+    </row>
+    <row r="14" spans="1:32" customFormat="1" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="17" t="s">
+        <v>540</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="E14" s="29" t="s">
+        <v>547</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="K14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="L14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="N14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="O14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="P14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="R14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="S14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="T14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="U14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="V14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="W14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="X14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD14" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE14" s="28" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="E15" s="29" t="s">
+        <v>548</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>551</v>
+      </c>
+      <c r="G15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="H15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="I15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="J15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="K15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="L15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="M15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="N15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="O15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="P15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="Q15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="R15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="S15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="T15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="U15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="V15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="W15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="X15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="Y15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="Z15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="AA15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="AB15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="AC15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="AD15" s="28" t="s">
+        <v>561</v>
+      </c>
+      <c r="AE15" s="28" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" customFormat="1" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="17" t="s">
+        <v>541</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="E16" s="29" t="s">
+        <v>560</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>560</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="I16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="J16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="K16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="L16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="M16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="N16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="O16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="P16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="R16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="S16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="T16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="U16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="V16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="W16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="X16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="Z16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE16" s="28" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>